<commit_message>
feat: Sincronizacao 100% de Mounjaro na tabela de SKUs + Botao Copiar Resumo WhatsApp + Barra Flutuante de Atalhos Rapidos
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -274,15 +274,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -291,7 +291,7 @@
     <xf numFmtId="167" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -702,7 +702,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: 08/09/2026 09:54:12 (09:54) • Tríade Estoque x Preço x Demanda</t>
+          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: 08/09/2026 10:52:58 (10:52) • Tríade Estoque x Preço x Demanda</t>
         </is>
       </c>
     </row>
@@ -795,25 +795,25 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>10053130</t>
+          <t>10046653</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>OZIVY 1MG 1CAN 3ML EMS</t>
+          <t>MOUNJARO 5MG 4CAN APLIC LILLY</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>999</v>
+        <v>11801.58</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>4571.32</v>
+        <v>26228.82</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>-3572.32</v>
+        <v>-14427.24</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>-0.7809999999999999</v>
+        <v>-0.55</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>155</v>
@@ -837,7 +837,7 @@
       </c>
       <c r="P5" s="13" t="inlineStr">
         <is>
-          <t>Detrator Moderado</t>
+          <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
@@ -847,59 +847,49 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>10050648</t>
+          <t>10046652</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
+          <t>MOUNJARO 2,5MG 4CAN APLIC LILLY</t>
         </is>
       </c>
       <c r="D6" s="18" t="n">
-        <v>899</v>
+        <v>8237.6</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>2055.01</v>
+        <v>17698.96</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>-1156.01</v>
+        <v>-9461.360000000001</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.535</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>56</v>
+        <v>115</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J6" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K6" s="18" t="n">
-        <v>988.22</v>
-      </c>
-      <c r="L6" s="23" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M6" s="18" t="n">
-        <v>988.22</v>
-      </c>
-      <c r="N6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="23" t="inlineStr">
-        <is>
-          <t>Preço Alinhado</t>
-        </is>
-      </c>
-      <c r="P6" s="23" t="inlineStr">
-        <is>
-          <t>Detrator Moderado</t>
+      <c r="K6" s="23" t="inlineStr"/>
+      <c r="L6" s="24" t="inlineStr"/>
+      <c r="M6" s="23" t="inlineStr"/>
+      <c r="N6" s="25" t="inlineStr"/>
+      <c r="O6" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P6" s="24" t="inlineStr">
+        <is>
+          <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
@@ -909,28 +899,28 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>10041262</t>
+          <t>10046655</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
+          <t>MOUNJARO 10MG 4CAN APLIC LILLY</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>416.84</v>
+        <v>3998</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>1225.93</v>
+        <v>10670.71</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-809.09</v>
+        <v>-6672.71</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-0.66</v>
+        <v>-0.625</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>0.01</v>
@@ -951,7 +941,7 @@
       </c>
       <c r="P7" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
@@ -961,49 +951,49 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>10052534</t>
+          <t>10042969</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO XXG 112UN</t>
         </is>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0</v>
+        <v>2596.72</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>793.25</v>
+        <v>7482.46</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>-793.25</v>
+        <v>-4885.74</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>-1</v>
+        <v>-0.653</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>289</v>
+        <v>339</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="J8" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K8" s="25" t="inlineStr"/>
-      <c r="L8" s="23" t="inlineStr"/>
-      <c r="M8" s="25" t="inlineStr"/>
-      <c r="N8" s="26" t="inlineStr"/>
-      <c r="O8" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P8" s="23" t="inlineStr">
-        <is>
-          <t>Neutro</t>
+      <c r="K8" s="23" t="inlineStr"/>
+      <c r="L8" s="24" t="inlineStr"/>
+      <c r="M8" s="23" t="inlineStr"/>
+      <c r="N8" s="25" t="inlineStr"/>
+      <c r="O8" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P8" s="24" t="inlineStr">
+        <is>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1013,31 +1003,31 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>10050440</t>
+          <t>10053130</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>AMMY 4MG 72CP REV MANTECORP</t>
+          <t>OZIVY 1MG 1CAN 3ML EMS</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0</v>
+        <v>1998</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>415.4</v>
+        <v>6782.27</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-415.4</v>
+        <v>-4784.27</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>-1</v>
+        <v>-0.705</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>9</v>
+        <v>286</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01</v>
+        <v>0.25</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
@@ -1055,7 +1045,7 @@
       </c>
       <c r="P9" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1065,49 +1055,49 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>10052535</t>
+          <t>10042968</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX G 92UN</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO XG 116UN</t>
         </is>
       </c>
       <c r="D10" s="18" t="n">
-        <v>0</v>
+        <v>1520.92</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>414.85</v>
+        <v>4615.84</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>-414.85</v>
+        <v>-3094.92</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>-1</v>
+        <v>-0.67</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>141</v>
+        <v>55</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="J10" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K10" s="25" t="inlineStr"/>
-      <c r="L10" s="23" t="inlineStr"/>
-      <c r="M10" s="25" t="inlineStr"/>
-      <c r="N10" s="26" t="inlineStr"/>
-      <c r="O10" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P10" s="23" t="inlineStr">
-        <is>
-          <t>Neutro</t>
+      <c r="K10" s="23" t="inlineStr"/>
+      <c r="L10" s="24" t="inlineStr"/>
+      <c r="M10" s="23" t="inlineStr"/>
+      <c r="N10" s="25" t="inlineStr"/>
+      <c r="O10" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P10" s="24" t="inlineStr">
+        <is>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1117,31 +1107,31 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>10028708</t>
+          <t>10042967</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO G 128UN</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>73.98999999999999</v>
+        <v>1227.61</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>480.27</v>
+        <v>3682.98</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-406.28</v>
+        <v>-2455.37</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>-0.846</v>
+        <v>-0.667</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>726</v>
+        <v>97</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.63</v>
+        <v>0.08</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -1159,7 +1149,7 @@
       </c>
       <c r="P11" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1169,59 +1159,49 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>10102163</t>
+          <t>10040750</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>QLAIRA 26CP+2CP REV BIOLAB</t>
+          <t>WEGOVY 1MG 3ML NOVO NORDISK</t>
         </is>
       </c>
       <c r="D12" s="18" t="n">
-        <v>74.22</v>
+        <v>0</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>452.46</v>
+        <v>2154.6</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>-378.24</v>
+        <v>-2154.6</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-0.836</v>
+        <v>-1</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>582</v>
+        <v>3</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="J12" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K12" s="18" t="n">
-        <v>74.22</v>
-      </c>
-      <c r="L12" s="23" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M12" s="18" t="n">
-        <v>55.67</v>
-      </c>
-      <c r="N12" s="27" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O12" s="23" t="inlineStr">
-        <is>
-          <t>São João Mais Cara</t>
-        </is>
-      </c>
-      <c r="P12" s="23" t="inlineStr">
-        <is>
-          <t>Neutro</t>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K12" s="23" t="inlineStr"/>
+      <c r="L12" s="24" t="inlineStr"/>
+      <c r="M12" s="23" t="inlineStr"/>
+      <c r="N12" s="25" t="inlineStr"/>
+      <c r="O12" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P12" s="24" t="inlineStr">
+        <is>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1231,59 +1211,59 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>10097312</t>
+          <t>10050648</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>NESTOGENO 2 800G NESTLE</t>
+          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
+        <v>899</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>3048.93</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>-2149.93</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>-0.705</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>136</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>988.22</v>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>988.22</v>
+      </c>
+      <c r="N13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="7" t="n">
-        <v>339.25</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>-339.25</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>210</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>67.98999999999999</v>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>61.06</v>
-      </c>
-      <c r="N13" s="28" t="n">
-        <v>0.113</v>
-      </c>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P13" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1293,49 +1273,49 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>10052532</t>
+          <t>10050654</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXXG 70UN</t>
+          <t>POVIZTRA 2,4MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D14" s="18" t="n">
-        <v>1103.21</v>
+        <v>2338</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>1429.94</v>
+        <v>3930.14</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>-326.73</v>
+        <v>-1592.14</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>-0.228</v>
+        <v>-0.405</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>825</v>
+        <v>27</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>0.72</v>
+        <v>0.02</v>
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K14" s="25" t="inlineStr"/>
-      <c r="L14" s="23" t="inlineStr"/>
-      <c r="M14" s="25" t="inlineStr"/>
-      <c r="N14" s="26" t="inlineStr"/>
-      <c r="O14" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P14" s="23" t="inlineStr">
-        <is>
-          <t>Neutro</t>
+      <c r="K14" s="23" t="inlineStr"/>
+      <c r="L14" s="24" t="inlineStr"/>
+      <c r="M14" s="23" t="inlineStr"/>
+      <c r="N14" s="25" t="inlineStr"/>
+      <c r="O14" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P14" s="24" t="inlineStr">
+        <is>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1345,31 +1325,31 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>10006600</t>
+          <t>10040801</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>LEITE NINHO 800G 1+PREBIO 20% DESC 2ªUN</t>
+          <t>WEGOVY 1,7MG 3ML NOVO NORDISK</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>268.48</v>
+        <v>1508.65</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-268.48</v>
+        <v>-1508.65</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1387,7 +1367,7 @@
       </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1397,59 +1377,49 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>10049738</t>
+          <t>10041262</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>OLIRE 6MG/ML 3ML 3APLIC INJ EMS</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
         </is>
       </c>
       <c r="D16" s="18" t="n">
-        <v>0</v>
+        <v>628.64</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>236.11</v>
+        <v>1818.86</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>-236.11</v>
+        <v>-1190.22</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>-1</v>
+        <v>-0.654</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="J16" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K16" s="18" t="n">
-        <v>866.24</v>
-      </c>
-      <c r="L16" s="23" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M16" s="18" t="n">
-        <v>866.24</v>
-      </c>
-      <c r="N16" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="23" t="inlineStr">
-        <is>
-          <t>Preço Alinhado</t>
-        </is>
-      </c>
-      <c r="P16" s="23" t="inlineStr">
-        <is>
-          <t>Neutro</t>
+      <c r="K16" s="23" t="inlineStr"/>
+      <c r="L16" s="24" t="inlineStr"/>
+      <c r="M16" s="23" t="inlineStr"/>
+      <c r="N16" s="25" t="inlineStr"/>
+      <c r="O16" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P16" s="24" t="inlineStr">
+        <is>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1459,59 +1429,49 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>10033757</t>
+          <t>10052534</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT HIPER XXG 54UN</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>169.8</v>
+        <v>0</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>359.35</v>
+        <v>1176.91</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-189.55</v>
+        <v>-1176.91</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>-0.527</v>
+        <v>-1</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>309</v>
+        <v>605</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.27</v>
+        <v>0.53</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K17" s="7" t="n">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="L17" s="13" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M17" s="7" t="n">
-        <v>72.90000000000001</v>
-      </c>
-      <c r="N17" s="28" t="n">
-        <v>0.165</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="inlineStr"/>
+      <c r="L17" s="13" t="inlineStr"/>
+      <c r="M17" s="12" t="inlineStr"/>
+      <c r="N17" s="14" t="inlineStr"/>
       <c r="O17" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P17" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1521,57 +1481,47 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>100013179</t>
+          <t>10041261</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>UTROGESTAN 200MG 42CAP BESINS</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XXG 7</t>
         </is>
       </c>
       <c r="D18" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>188.89</v>
+        <v>816.53</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>-188.89</v>
+        <v>-816.53</v>
       </c>
       <c r="G18" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="J18" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K18" s="18" t="n">
-        <v>246.91</v>
-      </c>
-      <c r="L18" s="23" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M18" s="18" t="n">
-        <v>209.07</v>
-      </c>
-      <c r="N18" s="27" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="O18" s="23" t="inlineStr">
-        <is>
-          <t>São João Mais Cara</t>
-        </is>
-      </c>
-      <c r="P18" s="23" t="inlineStr">
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K18" s="23" t="inlineStr"/>
+      <c r="L18" s="24" t="inlineStr"/>
+      <c r="M18" s="23" t="inlineStr"/>
+      <c r="N18" s="25" t="inlineStr"/>
+      <c r="O18" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P18" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -1583,54 +1533,44 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>10105170</t>
+          <t>10041263</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>TOALHAS UMED NATURAL BABY LV100 PG80</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>212.99</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>394.78</v>
+        <v>842.66</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-181.79</v>
+        <v>-746.76</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.46</v>
+        <v>-0.8859999999999999</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>4975</v>
-      </c>
-      <c r="I19" s="29" t="n">
-        <v>4.34</v>
+        <v>6</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>0.01</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K19" s="7" t="n">
-        <v>14.99</v>
-      </c>
-      <c r="L19" s="13" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M19" s="7" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="N19" s="28" t="n">
-        <v>0.375</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K19" s="12" t="inlineStr"/>
+      <c r="L19" s="13" t="inlineStr"/>
+      <c r="M19" s="12" t="inlineStr"/>
+      <c r="N19" s="14" t="inlineStr"/>
       <c r="O19" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
@@ -1645,31 +1585,31 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>8277</t>
+          <t>100016230</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>SYSTEN CONTI 8 ADESIVOS THERAMEX</t>
+          <t>NEUTROGENA GEL HID FACIAL 50G HYDRO BOOST WATER</t>
         </is>
       </c>
       <c r="D20" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>179.92</v>
+        <v>720.55</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>-179.92</v>
+        <v>-720.55</v>
       </c>
       <c r="G20" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="J20" s="15" t="inlineStr">
         <is>
@@ -1677,25 +1617,25 @@
         </is>
       </c>
       <c r="K20" s="18" t="n">
-        <v>170.87</v>
-      </c>
-      <c r="L20" s="23" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
+        <v>94.98999999999999</v>
+      </c>
+      <c r="L20" s="24" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M20" s="18" t="n">
-        <v>125.98</v>
+        <v>58.99</v>
       </c>
       <c r="N20" s="27" t="n">
-        <v>0.356</v>
-      </c>
-      <c r="O20" s="23" t="inlineStr">
+        <v>0.61</v>
+      </c>
+      <c r="O20" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P20" s="23" t="inlineStr">
+      <c r="P20" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -1707,40 +1647,38 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>10041842</t>
+          <t>10042966</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>TOALHAS UMED PURO AMOR PAC 500TOALHAS PREMIUM</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO M 148UN</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>174.97</v>
+        <v>467.13</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>348.15</v>
+        <v>1115.96</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-173.18</v>
+        <v>-648.83</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>-0.4970000000000001</v>
+        <v>-0.581</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>328</v>
+        <v>21</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>0.29</v>
+        <v>0.02</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K21" s="7" t="n">
-        <v>59.99</v>
-      </c>
+      <c r="K21" s="12" t="inlineStr"/>
       <c r="L21" s="13" t="inlineStr"/>
       <c r="M21" s="12" t="inlineStr"/>
       <c r="N21" s="14" t="inlineStr"/>
@@ -1761,57 +1699,47 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>10047543</t>
+          <t>10028708</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>DULOXETINA 60MG 60CAP GEN EMS (C1)</t>
+          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>0</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>171.54</v>
+        <v>712.5599999999999</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>-171.54</v>
+        <v>-638.5700000000001</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>-1</v>
+        <v>-0.8959999999999999</v>
       </c>
       <c r="H22" s="21" t="n">
-        <v>120</v>
+        <v>964</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>0.1</v>
+        <v>0.84</v>
       </c>
       <c r="J22" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K22" s="18" t="n">
-        <v>162.69</v>
-      </c>
-      <c r="L22" s="23" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M22" s="18" t="n">
-        <v>154.99</v>
-      </c>
-      <c r="N22" s="27" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="O22" s="23" t="inlineStr">
-        <is>
-          <t>São João Mais Cara</t>
-        </is>
-      </c>
-      <c r="P22" s="23" t="inlineStr">
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K22" s="23" t="inlineStr"/>
+      <c r="L22" s="24" t="inlineStr"/>
+      <c r="M22" s="23" t="inlineStr"/>
+      <c r="N22" s="25" t="inlineStr"/>
+      <c r="O22" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P22" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -1823,31 +1751,31 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>10052533</t>
+          <t>10050440</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
+          <t>AMMY 4MG 72CP REV MANTECORP</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>463.6</v>
+        <v>0</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>631.95</v>
+        <v>616.3</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-168.35</v>
+        <v>-616.3</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>-0.266</v>
+        <v>-1</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>540</v>
+        <v>6</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>0.47</v>
+        <v>0.01</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -1875,53 +1803,47 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>10039205</t>
+          <t>10052535</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>SERUM CORP DOVE 380ML NIACINAMIDA</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX G 92UN</t>
         </is>
       </c>
       <c r="D24" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>167.9</v>
+        <v>615.49</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>-167.9</v>
+        <v>-615.49</v>
       </c>
       <c r="G24" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>120</v>
+        <v>252</v>
       </c>
       <c r="I24" s="22" t="n">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="J24" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K24" s="25" t="inlineStr"/>
-      <c r="L24" s="23" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="M24" s="18" t="n">
-        <v>29.89</v>
-      </c>
-      <c r="N24" s="26" t="inlineStr"/>
-      <c r="O24" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P24" s="23" t="inlineStr">
+      <c r="K24" s="23" t="inlineStr"/>
+      <c r="L24" s="24" t="inlineStr"/>
+      <c r="M24" s="23" t="inlineStr"/>
+      <c r="N24" s="25" t="inlineStr"/>
+      <c r="O24" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P24" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -1933,44 +1855,54 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>10028706</t>
+          <t>10102163</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XG 58UN</t>
+          <t>QLAIRA 26CP+2CP REV BIOLAB</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>73.98999999999999</v>
+        <v>74.22</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>241.35</v>
+        <v>671.29</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-167.36</v>
+        <v>-597.0700000000001</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>-0.6929999999999999</v>
+        <v>-0.889</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>457</v>
+        <v>700</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>0.4</v>
+        <v>0.61</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K25" s="12" t="inlineStr"/>
-      <c r="L25" s="13" t="inlineStr"/>
-      <c r="M25" s="12" t="inlineStr"/>
-      <c r="N25" s="14" t="inlineStr"/>
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>74.22</v>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="N25" s="28" t="n">
+        <v>0.333</v>
+      </c>
       <c r="O25" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P25" s="13" t="inlineStr">
@@ -1985,47 +1917,57 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>10051318</t>
+          <t>999697</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>DAPAGLIFLOZINA 10MG 30CP GEN EMS</t>
+          <t>EVRA 0,6+6MG 3ADES GEDEON RICHTER</t>
         </is>
       </c>
       <c r="D26" s="18" t="n">
-        <v>87.98999999999999</v>
+        <v>149.4</v>
       </c>
       <c r="E26" s="18" t="n">
-        <v>240.86</v>
+        <v>717.02</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>-152.87</v>
+        <v>-567.62</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>-0.635</v>
+        <v>-0.792</v>
       </c>
       <c r="H26" s="21" t="n">
-        <v>5067</v>
-      </c>
-      <c r="I26" s="30" t="n">
-        <v>4.42</v>
+        <v>60</v>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>0.05</v>
       </c>
       <c r="J26" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K26" s="25" t="inlineStr"/>
-      <c r="L26" s="23" t="inlineStr"/>
-      <c r="M26" s="25" t="inlineStr"/>
-      <c r="N26" s="26" t="inlineStr"/>
-      <c r="O26" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P26" s="23" t="inlineStr">
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K26" s="18" t="n">
+        <v>149.4</v>
+      </c>
+      <c r="L26" s="24" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M26" s="18" t="n">
+        <v>107</v>
+      </c>
+      <c r="N26" s="27" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="O26" s="24" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P26" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2037,31 +1979,31 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>10099263</t>
+          <t>10034724</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>VENLAFAXINA 150MG 30CAP GEN EMS (C1)</t>
+          <t>CONTRAVE 8+90MG 120CP REV LIB PROL MERCK (C1)</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>146.86</v>
+        <v>564.64</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>-146.86</v>
+        <v>-564.64</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
@@ -2089,47 +2031,47 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>10021286</t>
+          <t>10052532</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>TRELEGY 100+62,5+25MG 30DOSES GSK</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXXG 70UN</t>
         </is>
       </c>
       <c r="D28" s="18" t="n">
-        <v>0</v>
+        <v>1557.83</v>
       </c>
       <c r="E28" s="18" t="n">
-        <v>146.68</v>
+        <v>2121.53</v>
       </c>
       <c r="F28" s="19" t="n">
-        <v>-146.68</v>
+        <v>-563.7</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>-1</v>
+        <v>-0.266</v>
       </c>
       <c r="H28" s="21" t="n">
-        <v>12</v>
+        <v>1220</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>0.01</v>
+        <v>1.06</v>
       </c>
       <c r="J28" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K28" s="25" t="inlineStr"/>
-      <c r="L28" s="23" t="inlineStr"/>
-      <c r="M28" s="25" t="inlineStr"/>
-      <c r="N28" s="26" t="inlineStr"/>
-      <c r="O28" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P28" s="23" t="inlineStr">
+      <c r="K28" s="23" t="inlineStr"/>
+      <c r="L28" s="24" t="inlineStr"/>
+      <c r="M28" s="23" t="inlineStr"/>
+      <c r="N28" s="25" t="inlineStr"/>
+      <c r="O28" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P28" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2141,54 +2083,44 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>10098096</t>
+          <t>10028895</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>FR BIGFRAL DERMA PLUS ADULTO NOTURNA G 7UN</t>
+          <t>IZIZ 2,5MG+1,5MG 84CP LIBBS</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>140.83</v>
+        <v>514.0599999999999</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-140.83</v>
+        <v>-514.0599999999999</v>
       </c>
       <c r="G29" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="n">
-        <v>30.99</v>
-      </c>
-      <c r="L29" s="13" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="N29" s="28" t="n">
-        <v>0.245</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr"/>
+      <c r="L29" s="13" t="inlineStr"/>
+      <c r="M29" s="12" t="inlineStr"/>
+      <c r="N29" s="14" t="inlineStr"/>
       <c r="O29" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P29" s="13" t="inlineStr">
@@ -2203,47 +2135,47 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>10028705</t>
+          <t>10004419</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG G 60UN</t>
+          <t>OZEMPIC 1MG 4AGULHAS NOVOFINE 4MM NOVO NORDISK</t>
         </is>
       </c>
       <c r="D30" s="18" t="n">
+        <v>999</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <v>1508.11</v>
+      </c>
+      <c r="F30" s="19" t="n">
+        <v>-509.11</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <v>-0.338</v>
+      </c>
+      <c r="H30" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="I30" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="18" t="n">
-        <v>140.42</v>
-      </c>
-      <c r="F30" s="19" t="n">
-        <v>-140.42</v>
-      </c>
-      <c r="G30" s="20" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H30" s="21" t="n">
-        <v>359</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>0.31</v>
-      </c>
       <c r="J30" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K30" s="25" t="inlineStr"/>
-      <c r="L30" s="23" t="inlineStr"/>
-      <c r="M30" s="25" t="inlineStr"/>
-      <c r="N30" s="26" t="inlineStr"/>
-      <c r="O30" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P30" s="23" t="inlineStr">
+      <c r="K30" s="23" t="inlineStr"/>
+      <c r="L30" s="24" t="inlineStr"/>
+      <c r="M30" s="23" t="inlineStr"/>
+      <c r="N30" s="25" t="inlineStr"/>
+      <c r="O30" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P30" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2255,31 +2187,31 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>10040659</t>
+          <t>10050634</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>KIT DOVE SH 350+COND 150ML BOND INTENSE REPAIR</t>
+          <t>EXTENSIOR 1MG 3ML NOVO EUROFARMA</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>119.6</v>
+        <v>0</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>259.07</v>
+        <v>504.32</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-139.47</v>
+        <v>-504.32</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>-0.5379999999999999</v>
+        <v>-1</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>252</v>
+        <v>49</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>0.22</v>
+        <v>0.04</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
@@ -2307,57 +2239,47 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>10043691</t>
+          <t>10050642</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>BUP XL 150MG 60CP REV PROL 24H EUROFARMA (C1)</t>
+          <t>POVIZTRA 0,5MG 1,5ML EUROFARMA</t>
         </is>
       </c>
       <c r="D32" s="18" t="n">
-        <v>0</v>
+        <v>590</v>
       </c>
       <c r="E32" s="18" t="n">
-        <v>135.21</v>
+        <v>1087.36</v>
       </c>
       <c r="F32" s="19" t="n">
-        <v>-135.21</v>
+        <v>-497.36</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>-1</v>
+        <v>-0.457</v>
       </c>
       <c r="H32" s="21" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="J32" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K32" s="18" t="n">
-        <v>182.2</v>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
-        </is>
-      </c>
-      <c r="M32" s="18" t="n">
-        <v>152</v>
-      </c>
-      <c r="N32" s="27" t="n">
-        <v>0.199</v>
-      </c>
-      <c r="O32" s="23" t="inlineStr">
-        <is>
-          <t>São João Mais Cara</t>
-        </is>
-      </c>
-      <c r="P32" s="23" t="inlineStr">
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K32" s="23" t="inlineStr"/>
+      <c r="L32" s="24" t="inlineStr"/>
+      <c r="M32" s="23" t="inlineStr"/>
+      <c r="N32" s="25" t="inlineStr"/>
+      <c r="O32" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P32" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2369,31 +2291,31 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>10033463</t>
+          <t>10052533</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>480.66</v>
+        <v>463.6</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>611.5700000000001</v>
+        <v>937.6</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-130.91</v>
+        <v>-474</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>-0.214</v>
+        <v>-0.506</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>370</v>
+        <v>742</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>0.32</v>
+        <v>0.65</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
@@ -2421,47 +2343,47 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>1006900</t>
+          <t>10025098</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>NISTATINA+OXID ZINCO 60G GEN EMS</t>
+          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
-        <v>21.99</v>
+        <v>0</v>
       </c>
       <c r="E34" s="18" t="n">
-        <v>143.2</v>
+        <v>467.78</v>
       </c>
       <c r="F34" s="19" t="n">
-        <v>-121.21</v>
+        <v>-467.78</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>-0.846</v>
+        <v>-1</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>1361</v>
+        <v>0</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>1.19</v>
+        <v>0</v>
       </c>
       <c r="J34" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K34" s="25" t="inlineStr"/>
-      <c r="L34" s="23" t="inlineStr"/>
-      <c r="M34" s="25" t="inlineStr"/>
-      <c r="N34" s="26" t="inlineStr"/>
-      <c r="O34" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P34" s="23" t="inlineStr">
+      <c r="K34" s="23" t="inlineStr"/>
+      <c r="L34" s="24" t="inlineStr"/>
+      <c r="M34" s="23" t="inlineStr"/>
+      <c r="N34" s="25" t="inlineStr"/>
+      <c r="O34" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P34" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2473,31 +2395,31 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>10033462</t>
+          <t>10053171</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER M 68UN</t>
+          <t>OZIVY 0,25MG+0,5MG 1CAN 1,5ML EMS</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>117.38</v>
+        <v>451.12</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>-117.38</v>
+        <v>-451.12</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
@@ -2525,47 +2447,47 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>1008501</t>
+          <t>10033758</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>KALOBA 20ML GOTAS HERBARIUM</t>
+          <t>FR HUGGIES MAXIMA PROT HIPER XG 56UN</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
-        <v>0</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E36" s="18" t="n">
-        <v>116.32</v>
+        <v>529.6799999999999</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>-116.32</v>
+        <v>-444.78</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>-1</v>
+        <v>-0.84</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>39</v>
+        <v>286</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>0.03</v>
+        <v>0.25</v>
       </c>
       <c r="J36" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K36" s="25" t="inlineStr"/>
-      <c r="L36" s="23" t="inlineStr"/>
-      <c r="M36" s="25" t="inlineStr"/>
-      <c r="N36" s="26" t="inlineStr"/>
-      <c r="O36" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P36" s="23" t="inlineStr">
+      <c r="K36" s="23" t="inlineStr"/>
+      <c r="L36" s="24" t="inlineStr"/>
+      <c r="M36" s="23" t="inlineStr"/>
+      <c r="N36" s="25" t="inlineStr"/>
+      <c r="O36" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P36" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2577,31 +2499,31 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>10049083</t>
+          <t>10050640</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>KIT DOVE SH 350ML+COND 175ML RECONSTRUCAO+AMINOACIDOS</t>
+          <t>POVIZTRA 0,25MG 1,5ML EUROFARMA</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>59.8</v>
+        <v>590</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>174.08</v>
+        <v>1007.38</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-114.28</v>
+        <v>-417.38</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>-0.6559999999999999</v>
+        <v>-0.414</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>161</v>
+        <v>33</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>0.14</v>
+        <v>0.03</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -2629,49 +2551,47 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>10046212</t>
+          <t>10030120</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>PAPEL HIG FLORAX PREMIUM FOLHA DUPLA 20M</t>
+          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
         </is>
       </c>
       <c r="D38" s="18" t="n">
-        <v>83.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="E38" s="18" t="n">
-        <v>196.55</v>
+        <v>413.38</v>
       </c>
       <c r="F38" s="19" t="n">
-        <v>-112.62</v>
+        <v>-413.38</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>-0.573</v>
+        <v>-1</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>25982</v>
-      </c>
-      <c r="I38" s="30" t="n">
-        <v>22.65</v>
+        <v>8</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>0.01</v>
       </c>
       <c r="J38" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K38" s="18" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="L38" s="23" t="inlineStr"/>
-      <c r="M38" s="25" t="inlineStr"/>
-      <c r="N38" s="26" t="inlineStr"/>
-      <c r="O38" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P38" s="23" t="inlineStr">
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr"/>
+      <c r="L38" s="24" t="inlineStr"/>
+      <c r="M38" s="23" t="inlineStr"/>
+      <c r="N38" s="25" t="inlineStr"/>
+      <c r="O38" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P38" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2683,31 +2603,31 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>10030229</t>
+          <t>10006600</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>DR GOOD FINI MELATONINA 60GOMAS</t>
+          <t>LEITE NINHO 800G 1+PREBIO 20% DESC 2ªUN</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>107.93</v>
+        <v>398.34</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-107.93</v>
+        <v>-398.34</v>
       </c>
       <c r="G39" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>16</v>
+        <v>95</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>0.01</v>
+        <v>0.08</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
@@ -2735,53 +2655,57 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>6051</t>
+          <t>10097312</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>HASTES J&amp;J 75UN COTONETES</t>
+          <t>NESTOGENO 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D40" s="18" t="n">
-        <v>18.18</v>
+        <v>135.98</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>125.05</v>
+        <v>503.32</v>
       </c>
       <c r="F40" s="19" t="n">
-        <v>-106.87</v>
+        <v>-367.34</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>-0.855</v>
+        <v>-0.73</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>160</v>
+        <v>279</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>0.14</v>
+        <v>0.24</v>
       </c>
       <c r="J40" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K40" s="25" t="inlineStr"/>
-      <c r="L40" s="23" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K40" s="18" t="n">
+        <v>67.98999999999999</v>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>DROGARAIA</t>
         </is>
       </c>
       <c r="M40" s="18" t="n">
-        <v>5.98</v>
-      </c>
-      <c r="N40" s="26" t="inlineStr"/>
-      <c r="O40" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P40" s="23" t="inlineStr">
+        <v>61.06</v>
+      </c>
+      <c r="N40" s="27" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="O40" s="24" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P40" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2793,44 +2717,54 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>100012568</t>
+          <t>10033757</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>DUTASTERIDA 0,5MG 30CAP GEN BIOSINTETICA</t>
+          <t>FR HUGGIES MAXIMA PROT HIPER XXG 54UN</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>0</v>
+        <v>169.8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>105.26</v>
+        <v>533.15</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-105.26</v>
+        <v>-363.35</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>-1</v>
+        <v>-0.6820000000000001</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>16</v>
+        <v>543</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>0.01</v>
+        <v>0.47</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K41" s="12" t="inlineStr"/>
-      <c r="L41" s="13" t="inlineStr"/>
-      <c r="M41" s="12" t="inlineStr"/>
-      <c r="N41" s="14" t="inlineStr"/>
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="L41" s="13" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="N41" s="28" t="n">
+        <v>0.165</v>
+      </c>
       <c r="O41" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P41" s="13" t="inlineStr">
@@ -2845,57 +2779,47 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>10007354</t>
+          <t>10033463</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>ITRACONAZOL 100MG 15CAP GEN GEOLAB</t>
+          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
-        <v>49.9</v>
+        <v>550.5599999999999</v>
       </c>
       <c r="E42" s="18" t="n">
-        <v>154.92</v>
+        <v>907.35</v>
       </c>
       <c r="F42" s="19" t="n">
-        <v>-105.02</v>
+        <v>-356.79</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>-0.6779999999999999</v>
+        <v>-0.393</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>15</v>
+        <v>461</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>0.01</v>
+        <v>0.4</v>
       </c>
       <c r="J42" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K42" s="18" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="L42" s="23" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
-        </is>
-      </c>
-      <c r="M42" s="18" t="n">
-        <v>75.98999999999999</v>
-      </c>
-      <c r="N42" s="24" t="n">
-        <v>-0.343</v>
-      </c>
-      <c r="O42" s="23" t="inlineStr">
-        <is>
-          <t>Líder de Preço</t>
-        </is>
-      </c>
-      <c r="P42" s="23" t="inlineStr">
+      <c r="K42" s="23" t="inlineStr"/>
+      <c r="L42" s="24" t="inlineStr"/>
+      <c r="M42" s="23" t="inlineStr"/>
+      <c r="N42" s="25" t="inlineStr"/>
+      <c r="O42" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P42" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2907,44 +2831,54 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>100022388</t>
+          <t>10097311</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>ENTRESTO 100MG 60CP REV NOVARTIS</t>
+          <t>NESTOGENO 1 800G NESTLE</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>0</v>
+        <v>203.97</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>101.17</v>
+        <v>557.35</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-101.17</v>
+        <v>-353.38</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>-1</v>
+        <v>-0.634</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>21</v>
+        <v>266</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>0.02</v>
+        <v>0.23</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K43" s="12" t="inlineStr"/>
-      <c r="L43" s="13" t="inlineStr"/>
-      <c r="M43" s="12" t="inlineStr"/>
-      <c r="N43" s="14" t="inlineStr"/>
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="n">
+        <v>67.98999999999999</v>
+      </c>
+      <c r="L43" s="13" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="N43" s="28" t="n">
+        <v>0.081</v>
+      </c>
       <c r="O43" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P43" s="13" t="inlineStr">
@@ -2959,47 +2893,57 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>10033760</t>
+          <t>10049738</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT HIPER G 58UN</t>
+          <t>OLIRE 6MG/ML 3ML 3APLIC INJ EMS</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>100.9</v>
+        <v>350.3</v>
       </c>
       <c r="F44" s="19" t="n">
-        <v>-100.9</v>
+        <v>-350.3</v>
       </c>
       <c r="G44" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H44" s="21" t="n">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K44" s="25" t="inlineStr"/>
-      <c r="L44" s="23" t="inlineStr"/>
-      <c r="M44" s="25" t="inlineStr"/>
-      <c r="N44" s="26" t="inlineStr"/>
-      <c r="O44" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P44" s="23" t="inlineStr">
+      <c r="K44" s="18" t="n">
+        <v>866.24</v>
+      </c>
+      <c r="L44" s="24" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M44" s="18" t="n">
+        <v>866.24</v>
+      </c>
+      <c r="N44" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="24" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P44" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3011,31 +2955,31 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>10021280</t>
+          <t>100011549</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>TRIMBOW 120DOSES SPRAY CHIESI</t>
+          <t>NAN SUPREME 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>0</v>
+        <v>132.49</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>100.7</v>
+        <v>482.35</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-100.7</v>
+        <v>-349.86</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>-1</v>
+        <v>-0.725</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>2</v>
+        <v>88</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
@@ -3063,31 +3007,31 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>10107350</t>
+          <t>100020215</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>PRIMOGYNA 2MG 28DRG GENOM</t>
+          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>95.04000000000001</v>
+        <v>327.46</v>
       </c>
       <c r="F46" s="19" t="n">
-        <v>-95.04000000000001</v>
+        <v>-327.46</v>
       </c>
       <c r="G46" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H46" s="21" t="n">
-        <v>23</v>
+        <v>420</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="J46" s="15" t="inlineStr">
         <is>
@@ -3095,25 +3039,25 @@
         </is>
       </c>
       <c r="K46" s="18" t="n">
-        <v>117.25</v>
-      </c>
-      <c r="L46" s="23" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
+        <v>25.9</v>
+      </c>
+      <c r="L46" s="24" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M46" s="18" t="n">
-        <v>92.58</v>
+        <v>15.9</v>
       </c>
       <c r="N46" s="27" t="n">
-        <v>0.266</v>
-      </c>
-      <c r="O46" s="23" t="inlineStr">
+        <v>0.629</v>
+      </c>
+      <c r="O46" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P46" s="23" t="inlineStr">
+      <c r="P46" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3125,31 +3069,31 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>10037546</t>
+          <t>10052539</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 16UN</t>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>0</v>
+        <v>377.7</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>91.31999999999999</v>
+        <v>701.91</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-91.31999999999999</v>
+        <v>-324.21</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>-1</v>
+        <v>-0.462</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>686</v>
+        <v>40</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>0.6</v>
+        <v>0.03</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
@@ -3177,47 +3121,47 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>100011177</t>
+          <t>10049094</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>SUMAXPRO 85MG+500MG 2CP REV LIBBS</t>
+          <t>NUSTENDI 180MG/10MG 30CP DAIICHI</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
-        <v>0</v>
+        <v>203.67</v>
       </c>
       <c r="E48" s="18" t="n">
-        <v>90.05</v>
+        <v>514.46</v>
       </c>
       <c r="F48" s="19" t="n">
-        <v>-90.05</v>
+        <v>-310.79</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>-1</v>
+        <v>-0.604</v>
       </c>
       <c r="H48" s="21" t="n">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
       <c r="J48" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K48" s="25" t="inlineStr"/>
-      <c r="L48" s="23" t="inlineStr"/>
-      <c r="M48" s="25" t="inlineStr"/>
-      <c r="N48" s="26" t="inlineStr"/>
-      <c r="O48" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P48" s="23" t="inlineStr">
+      <c r="K48" s="23" t="inlineStr"/>
+      <c r="L48" s="24" t="inlineStr"/>
+      <c r="M48" s="23" t="inlineStr"/>
+      <c r="N48" s="25" t="inlineStr"/>
+      <c r="O48" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P48" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3229,54 +3173,44 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>10005584</t>
+          <t>10029021</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>TANSULOSINA 0,4MG 30CP LIB PROL GEN EMS</t>
+          <t>PANT SEC 50MG/ML SOL CAPI 3FR 50ML+1VALVSPR ACHE</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>87.28</v>
+        <v>307.22</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-87.28</v>
+        <v>-307.22</v>
       </c>
       <c r="G49" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>132</v>
+        <v>3</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K49" s="7" t="n">
-        <v>75.89</v>
-      </c>
-      <c r="L49" s="13" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M49" s="7" t="n">
-        <v>65.89</v>
-      </c>
-      <c r="N49" s="28" t="n">
-        <v>0.152</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K49" s="12" t="inlineStr"/>
+      <c r="L49" s="13" t="inlineStr"/>
+      <c r="M49" s="12" t="inlineStr"/>
+      <c r="N49" s="14" t="inlineStr"/>
       <c r="O49" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P49" s="13" t="inlineStr">
@@ -3291,47 +3225,57 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>100021381</t>
+          <t>10105170</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>DEXILANT 60MG 60CAP LIB RET TAKEDA</t>
+          <t>TOALHAS UMED NATURAL BABY LV100 PG80</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
-        <v>0</v>
+        <v>282.29</v>
       </c>
       <c r="E50" s="18" t="n">
-        <v>86.45</v>
+        <v>585.71</v>
       </c>
       <c r="F50" s="19" t="n">
-        <v>-86.45</v>
+        <v>-303.42</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>-1</v>
+        <v>-0.518</v>
       </c>
       <c r="H50" s="21" t="n">
-        <v>90</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>0.08</v>
+        <v>8221</v>
+      </c>
+      <c r="I50" s="30" t="n">
+        <v>7.17</v>
       </c>
       <c r="J50" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K50" s="25" t="inlineStr"/>
-      <c r="L50" s="23" t="inlineStr"/>
-      <c r="M50" s="25" t="inlineStr"/>
-      <c r="N50" s="26" t="inlineStr"/>
-      <c r="O50" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P50" s="23" t="inlineStr">
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K50" s="18" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="L50" s="24" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M50" s="18" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="N50" s="27" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="O50" s="24" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P50" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3343,31 +3287,31 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>100001424</t>
+          <t>10034467</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>ESCITALOPRAM 10MG 60CP REV GEN EMS (C1)</t>
+          <t>SLINDA 4MG 72CP+12PLACEBOS EXELTIS</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>40.49</v>
+        <v>0</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>126.73</v>
+        <v>294.82</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-86.23999999999999</v>
+        <v>-294.82</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>-0.6809999999999999</v>
+        <v>-1</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>219</v>
+        <v>9</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>0.19</v>
+        <v>0.01</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
@@ -3395,47 +3339,47 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>10035173</t>
+          <t>10028706</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>ESC DENT COLGATE 4UN SLIMSOFT BLACK</t>
+          <t>FR SAO JOAO BABY BAG XG 58UN</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
-        <v>26.49</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>111.46</v>
+        <v>358.09</v>
       </c>
       <c r="F52" s="19" t="n">
-        <v>-84.97</v>
+        <v>-284.1</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>-0.762</v>
+        <v>-0.7929999999999999</v>
       </c>
       <c r="H52" s="21" t="n">
-        <v>125</v>
+        <v>501</v>
       </c>
       <c r="I52" s="22" t="n">
-        <v>0.11</v>
+        <v>0.44</v>
       </c>
       <c r="J52" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K52" s="25" t="inlineStr"/>
-      <c r="L52" s="23" t="inlineStr"/>
-      <c r="M52" s="25" t="inlineStr"/>
-      <c r="N52" s="26" t="inlineStr"/>
-      <c r="O52" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P52" s="23" t="inlineStr">
+      <c r="K52" s="23" t="inlineStr"/>
+      <c r="L52" s="24" t="inlineStr"/>
+      <c r="M52" s="23" t="inlineStr"/>
+      <c r="N52" s="25" t="inlineStr"/>
+      <c r="O52" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P52" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3447,54 +3391,44 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2996</t>
+          <t>10041858</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>PROCTYL POM 30G 10APLIC TAKEDA</t>
+          <t>FR PAMPERS PANTS PREMIUM CARE XXXG 80UN</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>81.29000000000001</v>
+        <v>282.01</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-81.29000000000001</v>
+        <v>-282.01</v>
       </c>
       <c r="G53" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K53" s="7" t="n">
-        <v>109.18</v>
-      </c>
-      <c r="L53" s="13" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M53" s="7" t="n">
-        <v>80.95</v>
-      </c>
-      <c r="N53" s="28" t="n">
-        <v>0.349</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr"/>
+      <c r="L53" s="13" t="inlineStr"/>
+      <c r="M53" s="12" t="inlineStr"/>
+      <c r="N53" s="14" t="inlineStr"/>
       <c r="O53" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P53" s="13" t="inlineStr">
@@ -3509,47 +3443,47 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>100015009</t>
+          <t>10046473</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>SAB DOVE 90G LV+ PG- 6UN ORIGINAL</t>
+          <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 32UN</t>
         </is>
       </c>
       <c r="D54" s="18" t="n">
-        <v>251.1</v>
+        <v>0</v>
       </c>
       <c r="E54" s="18" t="n">
-        <v>330.88</v>
+        <v>281.85</v>
       </c>
       <c r="F54" s="19" t="n">
-        <v>-79.78</v>
+        <v>-281.85</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>-0.241</v>
+        <v>-1</v>
       </c>
       <c r="H54" s="21" t="n">
-        <v>12334</v>
-      </c>
-      <c r="I54" s="30" t="n">
-        <v>10.75</v>
+        <v>290</v>
+      </c>
+      <c r="I54" s="22" t="n">
+        <v>0.25</v>
       </c>
       <c r="J54" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K54" s="25" t="inlineStr"/>
-      <c r="L54" s="23" t="inlineStr"/>
-      <c r="M54" s="25" t="inlineStr"/>
-      <c r="N54" s="26" t="inlineStr"/>
-      <c r="O54" s="23" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P54" s="23" t="inlineStr">
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="inlineStr"/>
+      <c r="L54" s="24" t="inlineStr"/>
+      <c r="M54" s="23" t="inlineStr"/>
+      <c r="N54" s="25" t="inlineStr"/>
+      <c r="O54" s="24" t="inlineStr">
+        <is>
+          <t>Não Monitorado</t>
+        </is>
+      </c>
+      <c r="P54" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>

</xml_diff>

<commit_message>
feat: integra métrica oficial Estoque Loja do Relatório Estoque Final (35k SKUs)
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -237,7 +237,7 @@
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -270,7 +270,7 @@
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -282,7 +282,10 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -291,10 +294,7 @@
     <xf numFmtId="167" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -702,7 +702,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: 08/09/2026 10:52:58 (10:52) • Tríade Estoque x Preço x Demanda</t>
+          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: 08/09/2026 12:53:08 (12:53) • Tríade Estoque x Preço x Demanda</t>
         </is>
       </c>
     </row>
@@ -804,26 +804,26 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>11801.58</v>
+        <v>19389.87</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>26228.82</v>
+        <v>43874.73</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>-14427.24</v>
+        <v>-24484.86</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>-0.55</v>
+        <v>-0.5579999999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>155</v>
+        <v>11783</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.14</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K5" s="12" t="inlineStr"/>
@@ -847,35 +847,35 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>10046652</t>
+          <t>10042969</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>MOUNJARO 2,5MG 4CAN APLIC LILLY</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO XXG 112UN</t>
         </is>
       </c>
       <c r="D6" s="18" t="n">
-        <v>8237.6</v>
+        <v>4012.69</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>17698.96</v>
+        <v>12516.41</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>-9461.360000000001</v>
+        <v>-8503.719999999999</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>-0.535</v>
+        <v>-0.679</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>115</v>
+        <v>10635</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>0.1</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="J6" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
@@ -908,26 +908,26 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>3998</v>
+        <v>10695</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>10670.71</v>
+        <v>17849.62</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-6672.71</v>
+        <v>-7154.62</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-0.625</v>
+        <v>-0.401</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>10</v>
+        <v>3194</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.01</v>
+        <v>2.54</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr"/>
@@ -951,35 +951,35 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>10042969</t>
+          <t>10053130</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC JUMBO XXG 112UN</t>
+          <t>OZIVY 1MG 1CAN 3ML EMS</t>
         </is>
       </c>
       <c r="D8" s="18" t="n">
-        <v>2596.72</v>
+        <v>4925.62</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>7482.46</v>
+        <v>11345.16</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>-4885.74</v>
+        <v>-6419.54</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>-0.653</v>
+        <v>-0.5660000000000001</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>339</v>
+        <v>12111</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>0.3</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J8" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
@@ -993,7 +993,7 @@
       </c>
       <c r="P8" s="24" t="inlineStr">
         <is>
-          <t>Detrator Moderado</t>
+          <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
@@ -1003,35 +1003,35 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>10053130</t>
+          <t>10046652</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>OZIVY 1MG 1CAN 3ML EMS</t>
+          <t>MOUNJARO 2,5MG 4CAN APLIC LILLY</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>1998</v>
+        <v>24428.3</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>6782.27</v>
+        <v>29606.25</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-4784.27</v>
+        <v>-5177.95</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>-0.705</v>
+        <v>-0.175</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>286</v>
+        <v>9805</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.25</v>
+        <v>7.79</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr"/>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="P9" s="13" t="inlineStr">
         <is>
-          <t>Detrator Moderado</t>
+          <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
@@ -1064,26 +1064,26 @@
         </is>
       </c>
       <c r="D10" s="18" t="n">
-        <v>1520.92</v>
+        <v>2720.52</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>4615.84</v>
+        <v>7721.22</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>-3094.92</v>
+        <v>-5000.7</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>-0.67</v>
+        <v>-0.648</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>55</v>
+        <v>2116</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>0.05</v>
+        <v>1.68</v>
       </c>
       <c r="J10" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="P10" s="24" t="inlineStr">
         <is>
-          <t>Detrator Moderado</t>
+          <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
@@ -1116,26 +1116,26 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>1227.61</v>
+        <v>1977.42</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>3682.98</v>
+        <v>6160.78</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-2455.37</v>
+        <v>-4183.36</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>-0.667</v>
+        <v>-0.679</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>97</v>
+        <v>7624</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.08</v>
+        <v>6.06</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr"/>
@@ -1159,31 +1159,31 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>10040750</t>
+          <t>10040801</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>WEGOVY 1MG 3ML NOVO NORDISK</t>
+          <t>WEGOVY 1,7MG 3ML NOVO NORDISK</t>
         </is>
       </c>
       <c r="D12" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>2154.6</v>
+        <v>2523.62</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>-2154.6</v>
+        <v>-2523.62</v>
       </c>
       <c r="G12" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="I12" s="22" t="n">
-        <v>0</v>
+        <v>1770</v>
+      </c>
+      <c r="I12" s="26" t="n">
+        <v>1.41</v>
       </c>
       <c r="J12" s="15" t="inlineStr">
         <is>
@@ -1211,54 +1211,44 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>10050648</t>
+          <t>10040750</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
+          <t>WEGOVY 1MG 3ML NOVO NORDISK</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>899</v>
+        <v>1398</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>3048.93</v>
+        <v>3604.14</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-2149.93</v>
+        <v>-2206.14</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>-0.705</v>
+        <v>-0.612</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>136</v>
+        <v>3359</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.12</v>
+        <v>2.67</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>988.22</v>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>988.22</v>
-      </c>
-      <c r="N13" s="26" t="n">
-        <v>0</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr"/>
+      <c r="L13" s="13" t="inlineStr"/>
+      <c r="M13" s="12" t="inlineStr"/>
+      <c r="N13" s="14" t="inlineStr"/>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P13" s="13" t="inlineStr">
@@ -1273,35 +1263,35 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>10050654</t>
+          <t>10041262</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>POVIZTRA 2,4MG 3ML EUROFARMA</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
         </is>
       </c>
       <c r="D14" s="18" t="n">
-        <v>2338</v>
+        <v>1047.81</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>3930.14</v>
+        <v>3042.52</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>-1592.14</v>
+        <v>-1994.71</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>-0.405</v>
+        <v>-0.6559999999999999</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>27</v>
+        <v>2289</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>0.02</v>
+        <v>1.82</v>
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
@@ -1325,35 +1315,35 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>10040801</t>
+          <t>10004419</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>WEGOVY 1,7MG 3ML NOVO NORDISK</t>
+          <t>OZEMPIC 1MG 4AGULHAS NOVOFINE 4MM NOVO NORDISK</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1508.65</v>
+        <v>2522.72</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-1508.65</v>
+        <v>-1523.72</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>-1</v>
+        <v>-0.604</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>4</v>
+        <v>2511</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0</v>
+        <v>1.99</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr"/>
@@ -1377,35 +1367,35 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>10041262</t>
+          <t>10052534</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
         </is>
       </c>
       <c r="D16" s="18" t="n">
-        <v>628.64</v>
+        <v>571.85</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>1818.86</v>
+        <v>1968.69</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>-1190.22</v>
+        <v>-1396.84</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>-0.654</v>
+        <v>-0.71</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>18</v>
+        <v>8641</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>0.02</v>
+        <v>6.86</v>
       </c>
       <c r="J16" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
@@ -1429,31 +1419,31 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>10052534</t>
+          <t>10041261</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XXG 7</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1176.91</v>
+        <v>1365.87</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-1176.91</v>
+        <v>-1365.87</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>605</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>0.53</v>
+        <v>1277</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>1.01</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
@@ -1481,35 +1471,35 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>10041261</t>
+          <t>10041263</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XXG 7</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
         </is>
       </c>
       <c r="D18" s="18" t="n">
-        <v>0</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>816.53</v>
+        <v>1409.57</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>-816.53</v>
+        <v>-1313.67</v>
       </c>
       <c r="G18" s="20" t="n">
-        <v>-1</v>
+        <v>-0.9320000000000001</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>9</v>
+        <v>3254</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>0.01</v>
+        <v>2.58</v>
       </c>
       <c r="J18" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
@@ -1523,7 +1513,7 @@
       </c>
       <c r="P18" s="24" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1533,35 +1523,35 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>10041263</t>
+          <t>10052532</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXXG 70UN</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>95.90000000000001</v>
+        <v>2247.93</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>842.66</v>
+        <v>3548.83</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-746.76</v>
+        <v>-1300.9</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.8859999999999999</v>
+        <v>-0.367</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>6</v>
+        <v>16881</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>0.01</v>
+        <v>13.41</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr"/>
@@ -1575,7 +1565,7 @@
       </c>
       <c r="P19" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1597,23 +1587,23 @@
         <v>0</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>720.55</v>
+        <v>1205.31</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>-720.55</v>
+        <v>-1205.31</v>
       </c>
       <c r="G20" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>3</v>
+        <v>4849</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>0</v>
+        <v>3.85</v>
       </c>
       <c r="J20" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K20" s="18" t="n">
@@ -1627,7 +1617,7 @@
       <c r="M20" s="18" t="n">
         <v>58.99</v>
       </c>
-      <c r="N20" s="27" t="n">
+      <c r="N20" s="28" t="n">
         <v>0.61</v>
       </c>
       <c r="O20" s="24" t="inlineStr">
@@ -1637,7 +1627,7 @@
       </c>
       <c r="P20" s="24" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1647,35 +1637,35 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>10042966</t>
+          <t>10028708</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC JUMBO M 148UN</t>
+          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>467.13</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>1115.96</v>
+        <v>1191.95</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-648.83</v>
+        <v>-1117.96</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>-0.581</v>
+        <v>-0.9379999999999999</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>21</v>
+        <v>40618</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>0.02</v>
+        <v>32.26</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr"/>
@@ -1689,7 +1679,7 @@
       </c>
       <c r="P21" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1699,35 +1689,35 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>10028708</t>
+          <t>10042966</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO M 148UN</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>73.98999999999999</v>
+        <v>766.9299999999999</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>712.5599999999999</v>
+        <v>1866.75</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>-638.5700000000001</v>
+        <v>-1099.82</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>-0.8959999999999999</v>
+        <v>-0.589</v>
       </c>
       <c r="H22" s="21" t="n">
-        <v>964</v>
+        <v>3834</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>0.84</v>
+        <v>3.05</v>
       </c>
       <c r="J22" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
@@ -1741,7 +1731,7 @@
       </c>
       <c r="P22" s="24" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1751,49 +1741,59 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>10050440</t>
+          <t>999697</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>AMMY 4MG 72CP REV MANTECORP</t>
+          <t>EVRA 0,6+6MG 3ADES GEDEON RICHTER</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>0</v>
+        <v>149.4</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>616.3</v>
+        <v>1199.41</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-616.3</v>
+        <v>-1050.01</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>-1</v>
+        <v>-0.875</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>6</v>
+        <v>4074</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>0.01</v>
+        <v>3.24</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K23" s="12" t="inlineStr"/>
-      <c r="L23" s="13" t="inlineStr"/>
-      <c r="M23" s="12" t="inlineStr"/>
-      <c r="N23" s="14" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>149.4</v>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>107</v>
+      </c>
+      <c r="N23" s="29" t="n">
+        <v>0.396</v>
+      </c>
       <c r="O23" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P23" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1803,31 +1803,31 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>10052535</t>
+          <t>10050440</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX G 92UN</t>
+          <t>AMMY 4MG 72CP REV MANTECORP</t>
         </is>
       </c>
       <c r="D24" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>615.49</v>
+        <v>1030.93</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>-615.49</v>
+        <v>-1030.93</v>
       </c>
       <c r="G24" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>252</v>
-      </c>
-      <c r="I24" s="22" t="n">
-        <v>0.22</v>
+        <v>864</v>
+      </c>
+      <c r="I24" s="26" t="n">
+        <v>0.6899999999999999</v>
       </c>
       <c r="J24" s="15" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="P24" s="24" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1855,39 +1855,39 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>10102163</t>
+          <t>10050648</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>QLAIRA 26CP+2CP REV BIOLAB</t>
+          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>74.22</v>
+        <v>4095</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>671.29</v>
+        <v>5100.15</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-597.0700000000001</v>
+        <v>-1005.15</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>-0.889</v>
+        <v>-0.197</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>700</v>
+        <v>9899</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>0.61</v>
+        <v>7.86</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K25" s="7" t="n">
-        <v>74.22</v>
+        <v>988.22</v>
       </c>
       <c r="L25" s="13" t="inlineStr">
         <is>
@@ -1895,19 +1895,19 @@
         </is>
       </c>
       <c r="M25" s="7" t="n">
-        <v>55.67</v>
-      </c>
-      <c r="N25" s="28" t="n">
-        <v>0.333</v>
+        <v>988.22</v>
+      </c>
+      <c r="N25" s="30" t="n">
+        <v>0</v>
       </c>
       <c r="O25" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P25" s="13" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
@@ -1917,54 +1917,44 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>999697</t>
+          <t>10034724</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>EVRA 0,6+6MG 3ADES GEDEON RICHTER</t>
+          <t>CONTRAVE 8+90MG 120CP REV LIB PROL MERCK (C1)</t>
         </is>
       </c>
       <c r="D26" s="18" t="n">
-        <v>149.4</v>
+        <v>0</v>
       </c>
       <c r="E26" s="18" t="n">
-        <v>717.02</v>
+        <v>944.51</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>-567.62</v>
+        <v>-944.51</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>-0.792</v>
+        <v>-1</v>
       </c>
       <c r="H26" s="21" t="n">
-        <v>60</v>
+        <v>2108</v>
       </c>
       <c r="I26" s="22" t="n">
-        <v>0.05</v>
+        <v>1.67</v>
       </c>
       <c r="J26" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K26" s="18" t="n">
-        <v>149.4</v>
-      </c>
-      <c r="L26" s="24" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M26" s="18" t="n">
-        <v>107</v>
-      </c>
-      <c r="N26" s="27" t="n">
-        <v>0.396</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K26" s="23" t="inlineStr"/>
+      <c r="L26" s="24" t="inlineStr"/>
+      <c r="M26" s="23" t="inlineStr"/>
+      <c r="N26" s="25" t="inlineStr"/>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P26" s="24" t="inlineStr">
@@ -1979,35 +1969,35 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>10034724</t>
+          <t>10030119</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>CONTRAVE 8+90MG 120CP REV LIB PROL MERCK (C1)</t>
+          <t>RYBELSUS 14MG 30CP NOVO NORDISK</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>0</v>
+        <v>1150</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>564.64</v>
+        <v>2074.45</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>-564.64</v>
+        <v>-924.45</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>-1</v>
+        <v>-0.446</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>3</v>
+        <v>2918</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>0</v>
+        <v>2.32</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K27" s="12" t="inlineStr"/>
@@ -2031,35 +2021,35 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>10052532</t>
+          <t>10052533</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXXG 70UN</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
         </is>
       </c>
       <c r="D28" s="18" t="n">
-        <v>1557.83</v>
+        <v>695.4</v>
       </c>
       <c r="E28" s="18" t="n">
-        <v>2121.53</v>
+        <v>1568.39</v>
       </c>
       <c r="F28" s="19" t="n">
-        <v>-563.7</v>
+        <v>-872.99</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>-0.266</v>
+        <v>-0.5570000000000001</v>
       </c>
       <c r="H28" s="21" t="n">
-        <v>1220</v>
+        <v>16250</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>1.06</v>
+        <v>12.91</v>
       </c>
       <c r="J28" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr"/>
@@ -2083,31 +2073,31 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>10028895</t>
+          <t>10025098</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>IZIZ 2,5MG+1,5MG 84CP LIBBS</t>
+          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>514.0599999999999</v>
+        <v>782.49</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-514.0599999999999</v>
+        <v>-782.49</v>
       </c>
       <c r="G29" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="I29" s="11" t="n">
-        <v>0.04</v>
+        <v>212</v>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>0.17</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -2135,31 +2125,31 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>10004419</t>
+          <t>10053171</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>OZEMPIC 1MG 4AGULHAS NOVOFINE 4MM NOVO NORDISK</t>
+          <t>OZIVY 0,25MG+0,5MG 1CAN 1,5ML EMS</t>
         </is>
       </c>
       <c r="D30" s="18" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="E30" s="18" t="n">
-        <v>1508.11</v>
+        <v>754.62</v>
       </c>
       <c r="F30" s="19" t="n">
-        <v>-509.11</v>
+        <v>-754.62</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>-0.338</v>
+        <v>-1</v>
       </c>
       <c r="H30" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>0</v>
+        <v>1643</v>
+      </c>
+      <c r="I30" s="26" t="n">
+        <v>1.31</v>
       </c>
       <c r="J30" s="15" t="inlineStr">
         <is>
@@ -2187,44 +2177,54 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>10050634</t>
+          <t>10102163</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>EXTENSIOR 1MG 3ML NOVO EUROFARMA</t>
+          <t>QLAIRA 26CP+2CP REV BIOLAB</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>0</v>
+        <v>379</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>504.32</v>
+        <v>1122.92</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-504.32</v>
+        <v>-743.92</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>-1</v>
+        <v>-0.662</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>49</v>
+        <v>17247</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>0.04</v>
+        <v>13.7</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K31" s="12" t="inlineStr"/>
-      <c r="L31" s="13" t="inlineStr"/>
-      <c r="M31" s="12" t="inlineStr"/>
-      <c r="N31" s="14" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>74.22</v>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="N31" s="29" t="n">
+        <v>0.333</v>
+      </c>
       <c r="O31" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P31" s="13" t="inlineStr">
@@ -2239,35 +2239,35 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>10050642</t>
+          <t>10030120</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>POVIZTRA 0,5MG 1,5ML EUROFARMA</t>
+          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
         </is>
       </c>
       <c r="D32" s="18" t="n">
-        <v>590</v>
+        <v>0</v>
       </c>
       <c r="E32" s="18" t="n">
-        <v>1087.36</v>
+        <v>691.48</v>
       </c>
       <c r="F32" s="19" t="n">
-        <v>-497.36</v>
+        <v>-691.48</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>-0.457</v>
+        <v>-1</v>
       </c>
       <c r="H32" s="21" t="n">
-        <v>45</v>
+        <v>2004</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>0.04</v>
+        <v>1.59</v>
       </c>
       <c r="J32" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr"/>
@@ -2291,35 +2291,35 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>10052533</t>
+          <t>10052535</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX G 92UN</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>463.6</v>
+        <v>340.62</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>937.6</v>
+        <v>1029.57</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-474</v>
+        <v>-688.95</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>-0.506</v>
+        <v>-0.669</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>742</v>
+        <v>11671</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>0.65</v>
+        <v>9.27</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K33" s="12" t="inlineStr"/>
@@ -2343,35 +2343,35 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>10025098</t>
+          <t>10049094</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
+          <t>NUSTENDI 180MG/10MG 30CP DAIICHI</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
-        <v>0</v>
+        <v>203.67</v>
       </c>
       <c r="E34" s="18" t="n">
-        <v>467.78</v>
+        <v>860.5700000000001</v>
       </c>
       <c r="F34" s="19" t="n">
-        <v>-467.78</v>
+        <v>-656.9</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>-1</v>
+        <v>-0.763</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>0</v>
+        <v>2850</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>0</v>
+        <v>2.26</v>
       </c>
       <c r="J34" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr"/>
@@ -2395,35 +2395,35 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>10053171</t>
+          <t>10028895</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>OZIVY 0,25MG+0,5MG 1CAN 1,5ML EMS</t>
+          <t>IZIZ 2,5MG+1,5MG 84CP LIBBS</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>0</v>
+        <v>287.47</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>451.12</v>
+        <v>859.91</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>-451.12</v>
+        <v>-572.4400000000001</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>-1</v>
+        <v>-0.6659999999999999</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>8</v>
+        <v>4477</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>0.01</v>
+        <v>3.56</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K35" s="12" t="inlineStr"/>
@@ -2447,44 +2447,54 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>10033758</t>
+          <t>10097312</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT HIPER XG 56UN</t>
+          <t>NESTOGENO 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
-        <v>84.90000000000001</v>
+        <v>271.96</v>
       </c>
       <c r="E36" s="18" t="n">
-        <v>529.6799999999999</v>
+        <v>841.95</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>-444.78</v>
+        <v>-569.99</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>-0.84</v>
+        <v>-0.677</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>286</v>
+        <v>13240</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>0.25</v>
+        <v>10.52</v>
       </c>
       <c r="J36" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr"/>
-      <c r="L36" s="24" t="inlineStr"/>
-      <c r="M36" s="23" t="inlineStr"/>
-      <c r="N36" s="25" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K36" s="18" t="n">
+        <v>67.98999999999999</v>
+      </c>
+      <c r="L36" s="24" t="inlineStr">
+        <is>
+          <t>DROGARAIA</t>
+        </is>
+      </c>
+      <c r="M36" s="18" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="N36" s="28" t="n">
+        <v>0.113</v>
+      </c>
       <c r="O36" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P36" s="24" t="inlineStr">
@@ -2499,35 +2509,35 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>10050640</t>
+          <t>10006600</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>POVIZTRA 0,25MG 1,5ML EUROFARMA</t>
+          <t>LEITE NINHO 800G 1+PREBIO 20% DESC 2ªUN</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>590</v>
+        <v>98.58</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>1007.38</v>
+        <v>666.3200000000001</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-417.38</v>
+        <v>-567.74</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>-0.414</v>
+        <v>-0.852</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>33</v>
+        <v>12080</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>0.03</v>
+        <v>9.59</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K37" s="12" t="inlineStr"/>
@@ -2551,35 +2561,35 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>10030120</t>
+          <t>100011547</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
+          <t>NAN SUPREME 1 800G NESTLE</t>
         </is>
       </c>
       <c r="D38" s="18" t="n">
-        <v>0</v>
+        <v>132.49</v>
       </c>
       <c r="E38" s="18" t="n">
-        <v>413.38</v>
+        <v>685.71</v>
       </c>
       <c r="F38" s="19" t="n">
-        <v>-413.38</v>
+        <v>-553.22</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>-1</v>
+        <v>-0.8070000000000001</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>8</v>
+        <v>8308</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>0.01</v>
+        <v>6.6</v>
       </c>
       <c r="J38" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr"/>
@@ -2603,35 +2613,35 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>10006600</t>
+          <t>10033463</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>LEITE NINHO 800G 1+PREBIO 20% DESC 2ªUN</t>
+          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>0</v>
+        <v>969.96</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>398.34</v>
+        <v>1517.79</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-398.34</v>
+        <v>-547.83</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>-1</v>
+        <v>-0.361</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>95</v>
+        <v>12293</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>0.08</v>
+        <v>9.76</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K39" s="12" t="inlineStr"/>
@@ -2655,54 +2665,44 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>10097312</t>
+          <t>100011549</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>NESTOGENO 2 800G NESTLE</t>
+          <t>NAN SUPREME 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D40" s="18" t="n">
-        <v>135.98</v>
+        <v>264.98</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>503.32</v>
+        <v>806.87</v>
       </c>
       <c r="F40" s="19" t="n">
-        <v>-367.34</v>
+        <v>-541.89</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>-0.73</v>
+        <v>-0.672</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>279</v>
+        <v>7821</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>0.24</v>
+        <v>6.21</v>
       </c>
       <c r="J40" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K40" s="18" t="n">
-        <v>67.98999999999999</v>
-      </c>
-      <c r="L40" s="24" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
-        </is>
-      </c>
-      <c r="M40" s="18" t="n">
-        <v>61.06</v>
-      </c>
-      <c r="N40" s="27" t="n">
-        <v>0.113</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr"/>
+      <c r="L40" s="24" t="inlineStr"/>
+      <c r="M40" s="23" t="inlineStr"/>
+      <c r="N40" s="25" t="inlineStr"/>
       <c r="O40" s="24" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P40" s="24" t="inlineStr">
@@ -2717,54 +2717,44 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>10033757</t>
+          <t>10050634</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT HIPER XXG 54UN</t>
+          <t>EXTENSIOR 1MG 3ML NOVO EUROFARMA</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>169.8</v>
+        <v>309</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>533.15</v>
+        <v>843.61</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-363.35</v>
+        <v>-534.61</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>-0.6820000000000001</v>
+        <v>-0.634</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>543</v>
+        <v>4354</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>0.47</v>
+        <v>3.46</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="n">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="L41" s="13" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="n">
-        <v>72.90000000000001</v>
-      </c>
-      <c r="N41" s="28" t="n">
-        <v>0.165</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K41" s="12" t="inlineStr"/>
+      <c r="L41" s="13" t="inlineStr"/>
+      <c r="M41" s="12" t="inlineStr"/>
+      <c r="N41" s="14" t="inlineStr"/>
       <c r="O41" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P41" s="13" t="inlineStr">
@@ -2779,44 +2769,54 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>10033463</t>
+          <t>10097311</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
+          <t>NESTOGENO 1 800G NESTLE</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
-        <v>550.5599999999999</v>
+        <v>407.94</v>
       </c>
       <c r="E42" s="18" t="n">
-        <v>907.35</v>
+        <v>932.3200000000001</v>
       </c>
       <c r="F42" s="19" t="n">
-        <v>-356.79</v>
+        <v>-524.38</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>-0.393</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>461</v>
+        <v>10934</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>0.4</v>
+        <v>8.68</v>
       </c>
       <c r="J42" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr"/>
-      <c r="L42" s="24" t="inlineStr"/>
-      <c r="M42" s="23" t="inlineStr"/>
-      <c r="N42" s="25" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K42" s="18" t="n">
+        <v>67.98999999999999</v>
+      </c>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M42" s="18" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="N42" s="28" t="n">
+        <v>0.081</v>
+      </c>
       <c r="O42" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P42" s="24" t="inlineStr">
@@ -2831,54 +2831,44 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>10097311</t>
+          <t>10040659</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>NESTOGENO 1 800G NESTLE</t>
+          <t>KIT DOVE SH 350+COND 150ML BOND INTENSE REPAIR</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>203.97</v>
+        <v>149.5</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>557.35</v>
+        <v>642.96</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-353.38</v>
+        <v>-493.46</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>-0.634</v>
+        <v>-0.767</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>266</v>
+        <v>10271</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>0.23</v>
+        <v>8.16</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K43" s="7" t="n">
-        <v>67.98999999999999</v>
-      </c>
-      <c r="L43" s="13" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M43" s="7" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="N43" s="28" t="n">
-        <v>0.081</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K43" s="12" t="inlineStr"/>
+      <c r="L43" s="13" t="inlineStr"/>
+      <c r="M43" s="12" t="inlineStr"/>
+      <c r="N43" s="14" t="inlineStr"/>
       <c r="O43" s="13" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P43" s="13" t="inlineStr">
@@ -2893,54 +2883,44 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>10049738</t>
+          <t>10034467</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>OLIRE 6MG/ML 3ML 3APLIC INJ EMS</t>
+          <t>SLINDA 4MG 72CP+12PLACEBOS EXELTIS</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>350.3</v>
+        <v>493.16</v>
       </c>
       <c r="F44" s="19" t="n">
-        <v>-350.3</v>
+        <v>-493.16</v>
       </c>
       <c r="G44" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H44" s="21" t="n">
-        <v>8</v>
+        <v>3854</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>0.01</v>
+        <v>3.06</v>
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K44" s="18" t="n">
-        <v>866.24</v>
-      </c>
-      <c r="L44" s="24" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M44" s="18" t="n">
-        <v>866.24</v>
-      </c>
-      <c r="N44" s="29" t="n">
-        <v>0</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr"/>
+      <c r="L44" s="24" t="inlineStr"/>
+      <c r="M44" s="23" t="inlineStr"/>
+      <c r="N44" s="25" t="inlineStr"/>
       <c r="O44" s="24" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P44" s="24" t="inlineStr">
@@ -2955,31 +2935,31 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>100011549</t>
+          <t>10041858</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>NAN SUPREME 2 800G NESTLE</t>
+          <t>FR PAMPERS PANTS PREMIUM CARE XXXG 80UN</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>132.49</v>
+        <v>0</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>482.35</v>
+        <v>471.74</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-349.86</v>
+        <v>-471.74</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>-0.725</v>
+        <v>-1</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>88</v>
-      </c>
-      <c r="I45" s="11" t="n">
-        <v>0.08</v>
+        <v>666</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>0.53</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
@@ -3007,54 +2987,44 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>100020215</t>
+          <t>10046473</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
+          <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 32UN</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>327.46</v>
+        <v>471.47</v>
       </c>
       <c r="F46" s="19" t="n">
-        <v>-327.46</v>
+        <v>-471.47</v>
       </c>
       <c r="G46" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H46" s="21" t="n">
-        <v>420</v>
+        <v>19751</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>0.37</v>
+        <v>15.69</v>
       </c>
       <c r="J46" s="15" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
-        </is>
-      </c>
-      <c r="K46" s="18" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="L46" s="24" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M46" s="18" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="N46" s="27" t="n">
-        <v>0.629</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr"/>
+      <c r="L46" s="24" t="inlineStr"/>
+      <c r="M46" s="23" t="inlineStr"/>
+      <c r="N46" s="25" t="inlineStr"/>
       <c r="O46" s="24" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P46" s="24" t="inlineStr">
@@ -3069,44 +3039,54 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>10052539</t>
+          <t>100020215</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
+          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>377.7</v>
+        <v>77.7</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>701.91</v>
+        <v>547.76</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-324.21</v>
+        <v>-470.06</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>-0.462</v>
+        <v>-0.858</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>40</v>
+        <v>23012</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>0.03</v>
+        <v>18.28</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K47" s="12" t="inlineStr"/>
-      <c r="L47" s="13" t="inlineStr"/>
-      <c r="M47" s="12" t="inlineStr"/>
-      <c r="N47" s="14" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K47" s="7" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="L47" s="13" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M47" s="7" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="N47" s="29" t="n">
+        <v>0.629</v>
+      </c>
       <c r="O47" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P47" s="13" t="inlineStr">
@@ -3121,44 +3101,54 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>10049094</t>
+          <t>100013179</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>NUSTENDI 180MG/10MG 30CP DAIICHI</t>
+          <t>UTROGESTAN 200MG 42CAP BESINS</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
-        <v>203.67</v>
+        <v>0</v>
       </c>
       <c r="E48" s="18" t="n">
-        <v>514.46</v>
+        <v>468.79</v>
       </c>
       <c r="F48" s="19" t="n">
-        <v>-310.79</v>
+        <v>-468.79</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>-0.604</v>
+        <v>-1</v>
       </c>
       <c r="H48" s="21" t="n">
-        <v>123</v>
+        <v>3370</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>0.11</v>
+        <v>2.68</v>
       </c>
       <c r="J48" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr"/>
-      <c r="L48" s="24" t="inlineStr"/>
-      <c r="M48" s="23" t="inlineStr"/>
-      <c r="N48" s="25" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K48" s="18" t="n">
+        <v>246.91</v>
+      </c>
+      <c r="L48" s="24" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M48" s="18" t="n">
+        <v>209.07</v>
+      </c>
+      <c r="N48" s="28" t="n">
+        <v>0.181</v>
+      </c>
       <c r="O48" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P48" s="24" t="inlineStr">
@@ -3173,35 +3163,35 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>10029021</t>
+          <t>10050654</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>PANT SEC 50MG/ML SOL CAPI 3FR 50ML+1VALVSPR ACHE</t>
+          <t>POVIZTRA 2,4MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>0</v>
+        <v>6120</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>307.22</v>
+        <v>6574.22</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-307.22</v>
+        <v>-454.22</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>-1</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>3</v>
+        <v>4215</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>0</v>
+        <v>3.35</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K49" s="12" t="inlineStr"/>
@@ -3225,54 +3215,44 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>10105170</t>
+          <t>10052539</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>TOALHAS UMED NATURAL BABY LV100 PG80</t>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
-        <v>282.29</v>
+        <v>727.24</v>
       </c>
       <c r="E50" s="18" t="n">
-        <v>585.71</v>
+        <v>1174.13</v>
       </c>
       <c r="F50" s="19" t="n">
-        <v>-303.42</v>
+        <v>-446.89</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>-0.518</v>
+        <v>-0.381</v>
       </c>
       <c r="H50" s="21" t="n">
-        <v>8221</v>
-      </c>
-      <c r="I50" s="30" t="n">
-        <v>7.17</v>
+        <v>5078</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>4.03</v>
       </c>
       <c r="J50" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K50" s="18" t="n">
-        <v>14.99</v>
-      </c>
-      <c r="L50" s="24" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M50" s="18" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="N50" s="27" t="n">
-        <v>0.375</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="inlineStr"/>
+      <c r="L50" s="24" t="inlineStr"/>
+      <c r="M50" s="23" t="inlineStr"/>
+      <c r="N50" s="25" t="inlineStr"/>
       <c r="O50" s="24" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P50" s="24" t="inlineStr">
@@ -3287,44 +3267,54 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>10034467</t>
+          <t>8277</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>SLINDA 4MG 72CP+12PLACEBOS EXELTIS</t>
+          <t>SYSTEN CONTI 8 ADESIVOS THERAMEX</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>294.82</v>
+        <v>446.52</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-294.82</v>
+        <v>-446.52</v>
       </c>
       <c r="G51" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>9</v>
+        <v>5661</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>0.01</v>
+        <v>4.5</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K51" s="12" t="inlineStr"/>
-      <c r="L51" s="13" t="inlineStr"/>
-      <c r="M51" s="12" t="inlineStr"/>
-      <c r="N51" s="14" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="n">
+        <v>170.87</v>
+      </c>
+      <c r="L51" s="13" t="inlineStr">
+        <is>
+          <t>DROGARAIA</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="n">
+        <v>125.98</v>
+      </c>
+      <c r="N51" s="29" t="n">
+        <v>0.356</v>
+      </c>
       <c r="O51" s="13" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P51" s="13" t="inlineStr">
@@ -3339,35 +3329,35 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>10028706</t>
+          <t>10022882</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XG 58UN</t>
+          <t>ACICLOVIR 400MG 30CP GEN PRATI</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
-        <v>73.98999999999999</v>
+        <v>214.47</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>358.09</v>
+        <v>646.23</v>
       </c>
       <c r="F52" s="19" t="n">
-        <v>-284.1</v>
+        <v>-431.76</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>-0.7929999999999999</v>
+        <v>-0.6679999999999999</v>
       </c>
       <c r="H52" s="21" t="n">
-        <v>501</v>
+        <v>5328</v>
       </c>
       <c r="I52" s="22" t="n">
-        <v>0.44</v>
+        <v>4.23</v>
       </c>
       <c r="J52" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K52" s="23" t="inlineStr"/>
@@ -3391,31 +3381,31 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>10041858</t>
+          <t>10034591</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS PREMIUM CARE XXXG 80UN</t>
+          <t>PANTOGAR NEO 90CAP BIOLAB</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>282.01</v>
+        <v>429.57</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-282.01</v>
+        <v>-429.57</v>
       </c>
       <c r="G53" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="11" t="n">
-        <v>0</v>
+        <v>1755</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>1.39</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
@@ -3443,44 +3433,54 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>10046473</t>
+          <t>100011848</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 32UN</t>
+          <t>DES AXE AERO 150ML APOLLO</t>
         </is>
       </c>
       <c r="D54" s="18" t="n">
-        <v>0</v>
+        <v>74.3</v>
       </c>
       <c r="E54" s="18" t="n">
-        <v>281.85</v>
+        <v>459.59</v>
       </c>
       <c r="F54" s="19" t="n">
-        <v>-281.85</v>
+        <v>-385.29</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>-1</v>
+        <v>-0.838</v>
       </c>
       <c r="H54" s="21" t="n">
-        <v>290</v>
+        <v>58984</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>0.25</v>
+        <v>46.85</v>
       </c>
       <c r="J54" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="inlineStr"/>
-      <c r="L54" s="24" t="inlineStr"/>
-      <c r="M54" s="23" t="inlineStr"/>
-      <c r="N54" s="25" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K54" s="18" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="L54" s="24" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M54" s="18" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="N54" s="28" t="n">
+        <v>0.214</v>
+      </c>
       <c r="O54" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P54" s="24" t="inlineStr">

</xml_diff>

<commit_message>
feat: sincroniza catálogo completo de 9.005 produtos da Precifica (181 páginas)
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -209,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -241,12 +241,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -282,19 +279,25 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="167" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -826,68 +829,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr"/>
-      <c r="L5" s="13" t="inlineStr"/>
-      <c r="M5" s="12" t="inlineStr"/>
-      <c r="N5" s="14" t="inlineStr"/>
-      <c r="O5" s="13" t="inlineStr">
+      <c r="K5" s="7" t="n">
+        <v>2382.23</v>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>2382.23</v>
+      </c>
+      <c r="N5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="12" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>Detrator Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>10042969</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>FR PAMPERS CONFORTSEC JUMBO XXG 112UN</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>4012.69</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>12516.41</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>-8503.719999999999</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>-0.679</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>10635</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="inlineStr"/>
+      <c r="L6" s="23" t="inlineStr"/>
+      <c r="M6" s="22" t="inlineStr"/>
+      <c r="N6" s="24" t="inlineStr"/>
+      <c r="O6" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P5" s="13" t="inlineStr">
-        <is>
-          <t>Detrator Crítico</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>10042969</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>FR PAMPERS CONFORTSEC JUMBO XXG 112UN</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>4012.69</v>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>12516.41</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>-8503.719999999999</v>
-      </c>
-      <c r="G6" s="20" t="n">
-        <v>-0.679</v>
-      </c>
-      <c r="H6" s="21" t="n">
-        <v>10635</v>
-      </c>
-      <c r="I6" s="22" t="n">
-        <v>8.449999999999999</v>
-      </c>
-      <c r="J6" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr"/>
-      <c r="M6" s="23" t="inlineStr"/>
-      <c r="N6" s="25" t="inlineStr"/>
-      <c r="O6" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P6" s="24" t="inlineStr">
+      <c r="P6" s="23" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
         </is>
@@ -930,68 +943,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K7" s="12" t="inlineStr"/>
-      <c r="L7" s="13" t="inlineStr"/>
-      <c r="M7" s="12" t="inlineStr"/>
-      <c r="N7" s="14" t="inlineStr"/>
-      <c r="O7" s="13" t="inlineStr">
+      <c r="K7" s="7" t="n">
+        <v>3210.85</v>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>3210.85</v>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>Detrator Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>10053130</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>OZIVY 1MG 1CAN 3ML EMS</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>4925.62</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>11345.16</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>-6419.54</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>-0.5660000000000001</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>12111</v>
+      </c>
+      <c r="I8" s="21" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K8" s="22" t="inlineStr"/>
+      <c r="L8" s="23" t="inlineStr"/>
+      <c r="M8" s="22" t="inlineStr"/>
+      <c r="N8" s="24" t="inlineStr"/>
+      <c r="O8" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P7" s="13" t="inlineStr">
-        <is>
-          <t>Detrator Crítico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>10053130</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>OZIVY 1MG 1CAN 3ML EMS</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="n">
-        <v>4925.62</v>
-      </c>
-      <c r="E8" s="18" t="n">
-        <v>11345.16</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>-6419.54</v>
-      </c>
-      <c r="G8" s="20" t="n">
-        <v>-0.5660000000000001</v>
-      </c>
-      <c r="H8" s="21" t="n">
-        <v>12111</v>
-      </c>
-      <c r="I8" s="22" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr"/>
-      <c r="M8" s="23" t="inlineStr"/>
-      <c r="N8" s="25" t="inlineStr"/>
-      <c r="O8" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P8" s="24" t="inlineStr">
+      <c r="P8" s="23" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
         </is>
@@ -1034,68 +1057,88 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K9" s="12" t="inlineStr"/>
-      <c r="L9" s="13" t="inlineStr"/>
-      <c r="M9" s="12" t="inlineStr"/>
-      <c r="N9" s="14" t="inlineStr"/>
-      <c r="O9" s="13" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P9" s="13" t="inlineStr">
+      <c r="K9" s="7" t="n">
+        <v>1905.6</v>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>1905.6</v>
+      </c>
+      <c r="N9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="15" t="n">
+      <c r="A10" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>10042968</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC JUMBO XG 116UN</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="17" t="n">
         <v>2720.52</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="17" t="n">
         <v>7721.22</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>-5000.7</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="19" t="n">
         <v>-0.648</v>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="H10" s="20" t="n">
         <v>2116</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="I10" s="21" t="n">
         <v>1.68</v>
       </c>
-      <c r="J10" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr"/>
-      <c r="M10" s="23" t="inlineStr"/>
-      <c r="N10" s="25" t="inlineStr"/>
-      <c r="O10" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P10" s="24" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="N10" s="25" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P10" s="23" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
         </is>
@@ -1138,68 +1181,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr"/>
-      <c r="L11" s="13" t="inlineStr"/>
-      <c r="M11" s="12" t="inlineStr"/>
-      <c r="N11" s="14" t="inlineStr"/>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="K11" s="26" t="inlineStr"/>
+      <c r="L11" s="12" t="inlineStr"/>
+      <c r="M11" s="26" t="inlineStr"/>
+      <c r="N11" s="27" t="inlineStr"/>
+      <c r="O11" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P11" s="13" t="inlineStr">
+      <c r="P11" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="15" t="n">
+      <c r="A12" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>10040801</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>WEGOVY 1,7MG 3ML NOVO NORDISK</t>
         </is>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="17" t="n">
         <v>2523.62</v>
       </c>
-      <c r="F12" s="19" t="n">
+      <c r="F12" s="18" t="n">
         <v>-2523.62</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H12" s="21" t="n">
+      <c r="H12" s="20" t="n">
         <v>1770</v>
       </c>
-      <c r="I12" s="26" t="n">
+      <c r="I12" s="28" t="n">
         <v>1.41</v>
       </c>
-      <c r="J12" s="15" t="inlineStr">
+      <c r="J12" s="14" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr"/>
-      <c r="M12" s="23" t="inlineStr"/>
-      <c r="N12" s="25" t="inlineStr"/>
-      <c r="O12" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P12" s="24" t="inlineStr">
+      <c r="K12" s="17" t="n">
+        <v>1945.09</v>
+      </c>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="n">
+        <v>1945.09</v>
+      </c>
+      <c r="N12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="23" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P12" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1242,68 +1295,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr"/>
-      <c r="L13" s="13" t="inlineStr"/>
-      <c r="M13" s="12" t="inlineStr"/>
-      <c r="N13" s="14" t="inlineStr"/>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="K13" s="7" t="n">
+        <v>1298.54</v>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>1298.54</v>
+      </c>
+      <c r="N13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P13" s="12" t="inlineStr">
+        <is>
+          <t>Detrator Moderado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>10041262</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>1047.81</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>3042.52</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>-1994.71</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>-0.6559999999999999</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>2289</v>
+      </c>
+      <c r="I14" s="21" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K14" s="22" t="inlineStr"/>
+      <c r="L14" s="23" t="inlineStr"/>
+      <c r="M14" s="22" t="inlineStr"/>
+      <c r="N14" s="24" t="inlineStr"/>
+      <c r="O14" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P13" s="13" t="inlineStr">
-        <is>
-          <t>Detrator Moderado</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>10041262</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="n">
-        <v>1047.81</v>
-      </c>
-      <c r="E14" s="18" t="n">
-        <v>3042.52</v>
-      </c>
-      <c r="F14" s="19" t="n">
-        <v>-1994.71</v>
-      </c>
-      <c r="G14" s="20" t="n">
-        <v>-0.6559999999999999</v>
-      </c>
-      <c r="H14" s="21" t="n">
-        <v>2289</v>
-      </c>
-      <c r="I14" s="22" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="J14" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr"/>
-      <c r="M14" s="23" t="inlineStr"/>
-      <c r="N14" s="25" t="inlineStr"/>
-      <c r="O14" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P14" s="24" t="inlineStr">
+      <c r="P14" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1346,68 +1409,68 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K15" s="12" t="inlineStr"/>
-      <c r="L15" s="13" t="inlineStr"/>
-      <c r="M15" s="12" t="inlineStr"/>
-      <c r="N15" s="14" t="inlineStr"/>
-      <c r="O15" s="13" t="inlineStr">
+      <c r="K15" s="26" t="inlineStr"/>
+      <c r="L15" s="12" t="inlineStr"/>
+      <c r="M15" s="26" t="inlineStr"/>
+      <c r="N15" s="27" t="inlineStr"/>
+      <c r="O15" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P15" s="13" t="inlineStr">
+      <c r="P15" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="15" t="n">
+      <c r="A16" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>10052534</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
         </is>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="17" t="n">
         <v>571.85</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="17" t="n">
         <v>1968.69</v>
       </c>
-      <c r="F16" s="19" t="n">
+      <c r="F16" s="18" t="n">
         <v>-1396.84</v>
       </c>
-      <c r="G16" s="20" t="n">
+      <c r="G16" s="19" t="n">
         <v>-0.71</v>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="20" t="n">
         <v>8641</v>
       </c>
-      <c r="I16" s="22" t="n">
+      <c r="I16" s="21" t="n">
         <v>6.86</v>
       </c>
-      <c r="J16" s="15" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr"/>
-      <c r="M16" s="23" t="inlineStr"/>
-      <c r="N16" s="25" t="inlineStr"/>
-      <c r="O16" s="24" t="inlineStr">
+      <c r="K16" s="22" t="inlineStr"/>
+      <c r="L16" s="23" t="inlineStr"/>
+      <c r="M16" s="22" t="inlineStr"/>
+      <c r="N16" s="24" t="inlineStr"/>
+      <c r="O16" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P16" s="24" t="inlineStr">
+      <c r="P16" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1442,7 +1505,7 @@
       <c r="H17" s="10" t="n">
         <v>1277</v>
       </c>
-      <c r="I17" s="27" t="n">
+      <c r="I17" s="30" t="n">
         <v>1.01</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1450,68 +1513,68 @@
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K17" s="12" t="inlineStr"/>
-      <c r="L17" s="13" t="inlineStr"/>
-      <c r="M17" s="12" t="inlineStr"/>
-      <c r="N17" s="14" t="inlineStr"/>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="K17" s="26" t="inlineStr"/>
+      <c r="L17" s="12" t="inlineStr"/>
+      <c r="M17" s="26" t="inlineStr"/>
+      <c r="N17" s="27" t="inlineStr"/>
+      <c r="O17" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P17" s="13" t="inlineStr">
+      <c r="P17" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="15" t="n">
+      <c r="A18" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>10041263</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
         </is>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="17" t="n">
         <v>95.90000000000001</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="17" t="n">
         <v>1409.57</v>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F18" s="18" t="n">
         <v>-1313.67</v>
       </c>
-      <c r="G18" s="20" t="n">
+      <c r="G18" s="19" t="n">
         <v>-0.9320000000000001</v>
       </c>
-      <c r="H18" s="21" t="n">
+      <c r="H18" s="20" t="n">
         <v>3254</v>
       </c>
-      <c r="I18" s="22" t="n">
+      <c r="I18" s="21" t="n">
         <v>2.58</v>
       </c>
-      <c r="J18" s="15" t="inlineStr">
+      <c r="J18" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr"/>
-      <c r="M18" s="23" t="inlineStr"/>
-      <c r="N18" s="25" t="inlineStr"/>
-      <c r="O18" s="24" t="inlineStr">
+      <c r="K18" s="22" t="inlineStr"/>
+      <c r="L18" s="23" t="inlineStr"/>
+      <c r="M18" s="22" t="inlineStr"/>
+      <c r="N18" s="24" t="inlineStr"/>
+      <c r="O18" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P18" s="24" t="inlineStr">
+      <c r="P18" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1554,78 +1617,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K19" s="12" t="inlineStr"/>
-      <c r="L19" s="13" t="inlineStr"/>
-      <c r="M19" s="12" t="inlineStr"/>
-      <c r="N19" s="14" t="inlineStr"/>
-      <c r="O19" s="13" t="inlineStr">
+      <c r="K19" s="26" t="inlineStr"/>
+      <c r="L19" s="12" t="inlineStr"/>
+      <c r="M19" s="26" t="inlineStr"/>
+      <c r="N19" s="27" t="inlineStr"/>
+      <c r="O19" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P19" s="13" t="inlineStr">
+      <c r="P19" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="15" t="n">
+      <c r="A20" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>100016230</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>NEUTROGENA GEL HID FACIAL 50G HYDRO BOOST WATER</t>
         </is>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="17" t="n">
         <v>1205.31</v>
       </c>
-      <c r="F20" s="19" t="n">
+      <c r="F20" s="18" t="n">
         <v>-1205.31</v>
       </c>
-      <c r="G20" s="20" t="n">
+      <c r="G20" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H20" s="21" t="n">
+      <c r="H20" s="20" t="n">
         <v>4849</v>
       </c>
-      <c r="I20" s="22" t="n">
+      <c r="I20" s="21" t="n">
         <v>3.85</v>
       </c>
-      <c r="J20" s="15" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K20" s="18" t="n">
+      <c r="K20" s="17" t="n">
         <v>94.98999999999999</v>
       </c>
-      <c r="L20" s="24" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M20" s="18" t="n">
-        <v>58.99</v>
-      </c>
-      <c r="N20" s="28" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="O20" s="24" t="inlineStr">
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="N20" s="25" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="O20" s="23" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P20" s="24" t="inlineStr">
+      <c r="P20" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1668,68 +1731,68 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K21" s="12" t="inlineStr"/>
-      <c r="L21" s="13" t="inlineStr"/>
-      <c r="M21" s="12" t="inlineStr"/>
-      <c r="N21" s="14" t="inlineStr"/>
-      <c r="O21" s="13" t="inlineStr">
+      <c r="K21" s="26" t="inlineStr"/>
+      <c r="L21" s="12" t="inlineStr"/>
+      <c r="M21" s="26" t="inlineStr"/>
+      <c r="N21" s="27" t="inlineStr"/>
+      <c r="O21" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P21" s="13" t="inlineStr">
+      <c r="P21" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="15" t="n">
+      <c r="A22" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>10042966</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC JUMBO M 148UN</t>
         </is>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="17" t="n">
         <v>766.9299999999999</v>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E22" s="17" t="n">
         <v>1866.75</v>
       </c>
-      <c r="F22" s="19" t="n">
+      <c r="F22" s="18" t="n">
         <v>-1099.82</v>
       </c>
-      <c r="G22" s="20" t="n">
+      <c r="G22" s="19" t="n">
         <v>-0.589</v>
       </c>
-      <c r="H22" s="21" t="n">
+      <c r="H22" s="20" t="n">
         <v>3834</v>
       </c>
-      <c r="I22" s="22" t="n">
+      <c r="I22" s="21" t="n">
         <v>3.05</v>
       </c>
-      <c r="J22" s="15" t="inlineStr">
+      <c r="J22" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr"/>
-      <c r="M22" s="23" t="inlineStr"/>
-      <c r="N22" s="25" t="inlineStr"/>
-      <c r="O22" s="24" t="inlineStr">
+      <c r="K22" s="22" t="inlineStr"/>
+      <c r="L22" s="23" t="inlineStr"/>
+      <c r="M22" s="22" t="inlineStr"/>
+      <c r="N22" s="24" t="inlineStr"/>
+      <c r="O22" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P22" s="24" t="inlineStr">
+      <c r="P22" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1775,7 +1838,7 @@
       <c r="K23" s="7" t="n">
         <v>149.4</v>
       </c>
-      <c r="L23" s="13" t="inlineStr">
+      <c r="L23" s="12" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
@@ -1783,67 +1846,77 @@
       <c r="M23" s="7" t="n">
         <v>107</v>
       </c>
-      <c r="N23" s="29" t="n">
+      <c r="N23" s="31" t="n">
         <v>0.396</v>
       </c>
-      <c r="O23" s="13" t="inlineStr">
+      <c r="O23" s="12" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P23" s="13" t="inlineStr">
+      <c r="P23" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="15" t="n">
+      <c r="A24" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>10050440</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>AMMY 4MG 72CP REV MANTECORP</t>
         </is>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E24" s="17" t="n">
         <v>1030.93</v>
       </c>
-      <c r="F24" s="19" t="n">
+      <c r="F24" s="18" t="n">
         <v>-1030.93</v>
       </c>
-      <c r="G24" s="20" t="n">
+      <c r="G24" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H24" s="21" t="n">
+      <c r="H24" s="20" t="n">
         <v>864</v>
       </c>
-      <c r="I24" s="26" t="n">
+      <c r="I24" s="28" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="J24" s="15" t="inlineStr">
-        <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr"/>
-      <c r="M24" s="23" t="inlineStr"/>
-      <c r="N24" s="25" t="inlineStr"/>
-      <c r="O24" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P24" s="24" t="inlineStr">
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v>315.46</v>
+      </c>
+      <c r="L24" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M24" s="17" t="n">
+        <v>236.6</v>
+      </c>
+      <c r="N24" s="25" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="O24" s="23" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P24" s="23" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
@@ -1889,7 +1962,7 @@
       <c r="K25" s="7" t="n">
         <v>988.22</v>
       </c>
-      <c r="L25" s="13" t="inlineStr">
+      <c r="L25" s="12" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
@@ -1897,67 +1970,73 @@
       <c r="M25" s="7" t="n">
         <v>988.22</v>
       </c>
-      <c r="N25" s="30" t="n">
+      <c r="N25" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O25" s="13" t="inlineStr">
+      <c r="O25" s="12" t="inlineStr">
         <is>
           <t>Preço Alinhado</t>
         </is>
       </c>
-      <c r="P25" s="13" t="inlineStr">
+      <c r="P25" s="12" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="15" t="n">
+      <c r="A26" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>10034724</t>
         </is>
       </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>CONTRAVE 8+90MG 120CP REV LIB PROL MERCK (C1)</t>
         </is>
       </c>
-      <c r="D26" s="18" t="n">
+      <c r="D26" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="18" t="n">
+      <c r="E26" s="17" t="n">
         <v>944.51</v>
       </c>
-      <c r="F26" s="19" t="n">
+      <c r="F26" s="18" t="n">
         <v>-944.51</v>
       </c>
-      <c r="G26" s="20" t="n">
+      <c r="G26" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H26" s="21" t="n">
+      <c r="H26" s="20" t="n">
         <v>2108</v>
       </c>
-      <c r="I26" s="22" t="n">
+      <c r="I26" s="21" t="n">
         <v>1.67</v>
       </c>
-      <c r="J26" s="15" t="inlineStr">
+      <c r="J26" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr"/>
-      <c r="M26" s="23" t="inlineStr"/>
-      <c r="N26" s="25" t="inlineStr"/>
-      <c r="O26" s="24" t="inlineStr">
+      <c r="K26" s="22" t="inlineStr"/>
+      <c r="L26" s="23" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>549.9</v>
+      </c>
+      <c r="N26" s="24" t="inlineStr"/>
+      <c r="O26" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P26" s="24" t="inlineStr">
+      <c r="P26" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2000,68 +2079,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K27" s="12" t="inlineStr"/>
-      <c r="L27" s="13" t="inlineStr"/>
-      <c r="M27" s="12" t="inlineStr"/>
-      <c r="N27" s="14" t="inlineStr"/>
-      <c r="O27" s="13" t="inlineStr">
+      <c r="K27" s="7" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="N27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr">
+        <is>
+          <t>Neutro</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>10052533</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>695.4</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>1568.39</v>
+      </c>
+      <c r="F28" s="18" t="n">
+        <v>-872.99</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>-0.5570000000000001</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v>16250</v>
+      </c>
+      <c r="I28" s="21" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="J28" s="14" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="inlineStr"/>
+      <c r="L28" s="23" t="inlineStr"/>
+      <c r="M28" s="22" t="inlineStr"/>
+      <c r="N28" s="24" t="inlineStr"/>
+      <c r="O28" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P27" s="13" t="inlineStr">
-        <is>
-          <t>Neutro</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>10052533</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="n">
-        <v>695.4</v>
-      </c>
-      <c r="E28" s="18" t="n">
-        <v>1568.39</v>
-      </c>
-      <c r="F28" s="19" t="n">
-        <v>-872.99</v>
-      </c>
-      <c r="G28" s="20" t="n">
-        <v>-0.5570000000000001</v>
-      </c>
-      <c r="H28" s="21" t="n">
-        <v>16250</v>
-      </c>
-      <c r="I28" s="22" t="n">
-        <v>12.91</v>
-      </c>
-      <c r="J28" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr"/>
-      <c r="M28" s="23" t="inlineStr"/>
-      <c r="N28" s="25" t="inlineStr"/>
-      <c r="O28" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P28" s="24" t="inlineStr">
+      <c r="P28" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2096,7 +2185,7 @@
       <c r="H29" s="10" t="n">
         <v>212</v>
       </c>
-      <c r="I29" s="27" t="n">
+      <c r="I29" s="30" t="n">
         <v>0.17</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2104,68 +2193,74 @@
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K29" s="12" t="inlineStr"/>
-      <c r="L29" s="13" t="inlineStr"/>
-      <c r="M29" s="12" t="inlineStr"/>
-      <c r="N29" s="14" t="inlineStr"/>
-      <c r="O29" s="13" t="inlineStr">
+      <c r="K29" s="26" t="inlineStr"/>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="n">
+        <v>1212.9</v>
+      </c>
+      <c r="N29" s="27" t="inlineStr"/>
+      <c r="O29" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P29" s="13" t="inlineStr">
+      <c r="P29" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="15" t="n">
+      <c r="A30" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>10053171</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>OZIVY 0,25MG+0,5MG 1CAN 1,5ML EMS</t>
         </is>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E30" s="17" t="n">
         <v>754.62</v>
       </c>
-      <c r="F30" s="19" t="n">
+      <c r="F30" s="18" t="n">
         <v>-754.62</v>
       </c>
-      <c r="G30" s="20" t="n">
+      <c r="G30" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H30" s="21" t="n">
+      <c r="H30" s="20" t="n">
         <v>1643</v>
       </c>
-      <c r="I30" s="26" t="n">
+      <c r="I30" s="28" t="n">
         <v>1.31</v>
       </c>
-      <c r="J30" s="15" t="inlineStr">
+      <c r="J30" s="14" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr"/>
-      <c r="M30" s="23" t="inlineStr"/>
-      <c r="N30" s="25" t="inlineStr"/>
-      <c r="O30" s="24" t="inlineStr">
+      <c r="K30" s="22" t="inlineStr"/>
+      <c r="L30" s="23" t="inlineStr"/>
+      <c r="M30" s="22" t="inlineStr"/>
+      <c r="N30" s="24" t="inlineStr"/>
+      <c r="O30" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P30" s="24" t="inlineStr">
+      <c r="P30" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2211,7 +2306,7 @@
       <c r="K31" s="7" t="n">
         <v>74.22</v>
       </c>
-      <c r="L31" s="13" t="inlineStr">
+      <c r="L31" s="12" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
@@ -2219,67 +2314,77 @@
       <c r="M31" s="7" t="n">
         <v>55.67</v>
       </c>
-      <c r="N31" s="29" t="n">
+      <c r="N31" s="31" t="n">
         <v>0.333</v>
       </c>
-      <c r="O31" s="13" t="inlineStr">
+      <c r="O31" s="12" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P31" s="13" t="inlineStr">
+      <c r="P31" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="15" t="n">
+      <c r="A32" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>10030120</t>
         </is>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="C32" s="16" t="inlineStr">
         <is>
           <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
         </is>
       </c>
-      <c r="D32" s="18" t="n">
+      <c r="D32" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="18" t="n">
+      <c r="E32" s="17" t="n">
         <v>691.48</v>
       </c>
-      <c r="F32" s="19" t="n">
+      <c r="F32" s="18" t="n">
         <v>-691.48</v>
       </c>
-      <c r="G32" s="20" t="n">
+      <c r="G32" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H32" s="21" t="n">
+      <c r="H32" s="20" t="n">
         <v>2004</v>
       </c>
-      <c r="I32" s="22" t="n">
+      <c r="I32" s="21" t="n">
         <v>1.59</v>
       </c>
-      <c r="J32" s="15" t="inlineStr">
+      <c r="J32" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr"/>
-      <c r="M32" s="23" t="inlineStr"/>
-      <c r="N32" s="25" t="inlineStr"/>
-      <c r="O32" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P32" s="24" t="inlineStr">
+      <c r="K32" s="17" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="L32" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M32" s="17" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="N32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="23" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P32" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2322,68 +2427,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K33" s="12" t="inlineStr"/>
-      <c r="L33" s="13" t="inlineStr"/>
-      <c r="M33" s="12" t="inlineStr"/>
-      <c r="N33" s="14" t="inlineStr"/>
-      <c r="O33" s="13" t="inlineStr">
+      <c r="K33" s="26" t="inlineStr"/>
+      <c r="L33" s="12" t="inlineStr"/>
+      <c r="M33" s="26" t="inlineStr"/>
+      <c r="N33" s="27" t="inlineStr"/>
+      <c r="O33" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P33" s="13" t="inlineStr">
+      <c r="P33" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="15" t="n">
+      <c r="A34" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>10049094</t>
         </is>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
         <is>
           <t>NUSTENDI 180MG/10MG 30CP DAIICHI</t>
         </is>
       </c>
-      <c r="D34" s="18" t="n">
+      <c r="D34" s="17" t="n">
         <v>203.67</v>
       </c>
-      <c r="E34" s="18" t="n">
+      <c r="E34" s="17" t="n">
         <v>860.5700000000001</v>
       </c>
-      <c r="F34" s="19" t="n">
+      <c r="F34" s="18" t="n">
         <v>-656.9</v>
       </c>
-      <c r="G34" s="20" t="n">
+      <c r="G34" s="19" t="n">
         <v>-0.763</v>
       </c>
-      <c r="H34" s="21" t="n">
+      <c r="H34" s="20" t="n">
         <v>2850</v>
       </c>
-      <c r="I34" s="22" t="n">
+      <c r="I34" s="21" t="n">
         <v>2.26</v>
       </c>
-      <c r="J34" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr"/>
-      <c r="L34" s="24" t="inlineStr"/>
-      <c r="M34" s="23" t="inlineStr"/>
-      <c r="N34" s="25" t="inlineStr"/>
-      <c r="O34" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P34" s="24" t="inlineStr">
+      <c r="J34" s="14" t="inlineStr">
+        <is>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="n">
+        <v>218.67</v>
+      </c>
+      <c r="L34" s="23" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M34" s="17" t="n">
+        <v>197.18</v>
+      </c>
+      <c r="N34" s="25" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="O34" s="23" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P34" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2423,81 +2538,91 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K35" s="12" t="inlineStr"/>
-      <c r="L35" s="13" t="inlineStr"/>
-      <c r="M35" s="12" t="inlineStr"/>
-      <c r="N35" s="14" t="inlineStr"/>
-      <c r="O35" s="13" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P35" s="13" t="inlineStr">
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="n">
+        <v>164.09</v>
+      </c>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="n">
+        <v>115.9</v>
+      </c>
+      <c r="N35" s="31" t="n">
+        <v>0.416</v>
+      </c>
+      <c r="O35" s="12" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P35" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="15" t="n">
+      <c r="A36" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t>10097312</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr">
         <is>
           <t>NESTOGENO 2 800G NESTLE</t>
         </is>
       </c>
-      <c r="D36" s="18" t="n">
+      <c r="D36" s="17" t="n">
         <v>271.96</v>
       </c>
-      <c r="E36" s="18" t="n">
+      <c r="E36" s="17" t="n">
         <v>841.95</v>
       </c>
-      <c r="F36" s="19" t="n">
+      <c r="F36" s="18" t="n">
         <v>-569.99</v>
       </c>
-      <c r="G36" s="20" t="n">
+      <c r="G36" s="19" t="n">
         <v>-0.677</v>
       </c>
-      <c r="H36" s="21" t="n">
+      <c r="H36" s="20" t="n">
         <v>13240</v>
       </c>
-      <c r="I36" s="22" t="n">
+      <c r="I36" s="21" t="n">
         <v>10.52</v>
       </c>
-      <c r="J36" s="15" t="inlineStr">
+      <c r="J36" s="14" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K36" s="18" t="n">
+      <c r="K36" s="17" t="n">
         <v>67.98999999999999</v>
       </c>
-      <c r="L36" s="24" t="inlineStr">
+      <c r="L36" s="23" t="inlineStr">
         <is>
           <t>DROGARAIA</t>
         </is>
       </c>
-      <c r="M36" s="18" t="n">
+      <c r="M36" s="17" t="n">
         <v>61.06</v>
       </c>
-      <c r="N36" s="28" t="n">
+      <c r="N36" s="25" t="n">
         <v>0.113</v>
       </c>
-      <c r="O36" s="24" t="inlineStr">
+      <c r="O36" s="23" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P36" s="24" t="inlineStr">
+      <c r="P36" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2540,68 +2665,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K37" s="12" t="inlineStr"/>
-      <c r="L37" s="13" t="inlineStr"/>
-      <c r="M37" s="12" t="inlineStr"/>
-      <c r="N37" s="14" t="inlineStr"/>
-      <c r="O37" s="13" t="inlineStr">
+      <c r="K37" s="26" t="inlineStr"/>
+      <c r="L37" s="12" t="inlineStr"/>
+      <c r="M37" s="26" t="inlineStr"/>
+      <c r="N37" s="27" t="inlineStr"/>
+      <c r="O37" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P37" s="13" t="inlineStr">
+      <c r="P37" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="15" t="n">
+      <c r="A38" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>100011547</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C38" s="16" t="inlineStr">
         <is>
           <t>NAN SUPREME 1 800G NESTLE</t>
         </is>
       </c>
-      <c r="D38" s="18" t="n">
+      <c r="D38" s="17" t="n">
         <v>132.49</v>
       </c>
-      <c r="E38" s="18" t="n">
+      <c r="E38" s="17" t="n">
         <v>685.71</v>
       </c>
-      <c r="F38" s="19" t="n">
+      <c r="F38" s="18" t="n">
         <v>-553.22</v>
       </c>
-      <c r="G38" s="20" t="n">
+      <c r="G38" s="19" t="n">
         <v>-0.8070000000000001</v>
       </c>
-      <c r="H38" s="21" t="n">
+      <c r="H38" s="20" t="n">
         <v>8308</v>
       </c>
-      <c r="I38" s="22" t="n">
+      <c r="I38" s="21" t="n">
         <v>6.6</v>
       </c>
-      <c r="J38" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K38" s="23" t="inlineStr"/>
-      <c r="L38" s="24" t="inlineStr"/>
-      <c r="M38" s="23" t="inlineStr"/>
-      <c r="N38" s="25" t="inlineStr"/>
-      <c r="O38" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P38" s="24" t="inlineStr">
+      <c r="J38" s="14" t="inlineStr">
+        <is>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K38" s="17" t="n">
+        <v>132.49</v>
+      </c>
+      <c r="L38" s="23" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M38" s="17" t="n">
+        <v>124.19</v>
+      </c>
+      <c r="N38" s="25" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="O38" s="23" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P38" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2641,71 +2776,81 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="N39" s="31" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="O39" s="12" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P39" s="12" t="inlineStr">
+        <is>
+          <t>Neutro</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>100011549</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>NAN SUPREME 2 800G NESTLE</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="n">
+        <v>264.98</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <v>806.87</v>
+      </c>
+      <c r="F40" s="18" t="n">
+        <v>-541.89</v>
+      </c>
+      <c r="G40" s="19" t="n">
+        <v>-0.672</v>
+      </c>
+      <c r="H40" s="20" t="n">
+        <v>7821</v>
+      </c>
+      <c r="I40" s="21" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="J40" s="14" t="inlineStr">
+        <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K39" s="12" t="inlineStr"/>
-      <c r="L39" s="13" t="inlineStr"/>
-      <c r="M39" s="12" t="inlineStr"/>
-      <c r="N39" s="14" t="inlineStr"/>
-      <c r="O39" s="13" t="inlineStr">
+      <c r="K40" s="22" t="inlineStr"/>
+      <c r="L40" s="23" t="inlineStr"/>
+      <c r="M40" s="22" t="inlineStr"/>
+      <c r="N40" s="24" t="inlineStr"/>
+      <c r="O40" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P39" s="13" t="inlineStr">
-        <is>
-          <t>Neutro</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="15" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="16" t="inlineStr">
-        <is>
-          <t>100011549</t>
-        </is>
-      </c>
-      <c r="C40" s="17" t="inlineStr">
-        <is>
-          <t>NAN SUPREME 2 800G NESTLE</t>
-        </is>
-      </c>
-      <c r="D40" s="18" t="n">
-        <v>264.98</v>
-      </c>
-      <c r="E40" s="18" t="n">
-        <v>806.87</v>
-      </c>
-      <c r="F40" s="19" t="n">
-        <v>-541.89</v>
-      </c>
-      <c r="G40" s="20" t="n">
-        <v>-0.672</v>
-      </c>
-      <c r="H40" s="21" t="n">
-        <v>7821</v>
-      </c>
-      <c r="I40" s="22" t="n">
-        <v>6.21</v>
-      </c>
-      <c r="J40" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr"/>
-      <c r="L40" s="24" t="inlineStr"/>
-      <c r="M40" s="23" t="inlineStr"/>
-      <c r="N40" s="25" t="inlineStr"/>
-      <c r="O40" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P40" s="24" t="inlineStr">
+      <c r="P40" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2748,78 +2893,84 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K41" s="12" t="inlineStr"/>
-      <c r="L41" s="13" t="inlineStr"/>
-      <c r="M41" s="12" t="inlineStr"/>
-      <c r="N41" s="14" t="inlineStr"/>
-      <c r="O41" s="13" t="inlineStr">
+      <c r="K41" s="26" t="inlineStr"/>
+      <c r="L41" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="n">
+        <v>988.22</v>
+      </c>
+      <c r="N41" s="27" t="inlineStr"/>
+      <c r="O41" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P41" s="13" t="inlineStr">
+      <c r="P41" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="15" t="n">
+      <c r="A42" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>10097311</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C42" s="16" t="inlineStr">
         <is>
           <t>NESTOGENO 1 800G NESTLE</t>
         </is>
       </c>
-      <c r="D42" s="18" t="n">
+      <c r="D42" s="17" t="n">
         <v>407.94</v>
       </c>
-      <c r="E42" s="18" t="n">
+      <c r="E42" s="17" t="n">
         <v>932.3200000000001</v>
       </c>
-      <c r="F42" s="19" t="n">
+      <c r="F42" s="18" t="n">
         <v>-524.38</v>
       </c>
-      <c r="G42" s="20" t="n">
+      <c r="G42" s="19" t="n">
         <v>-0.5620000000000001</v>
       </c>
-      <c r="H42" s="21" t="n">
+      <c r="H42" s="20" t="n">
         <v>10934</v>
       </c>
-      <c r="I42" s="22" t="n">
+      <c r="I42" s="21" t="n">
         <v>8.68</v>
       </c>
-      <c r="J42" s="15" t="inlineStr">
+      <c r="J42" s="14" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K42" s="18" t="n">
+      <c r="K42" s="17" t="n">
         <v>67.98999999999999</v>
       </c>
-      <c r="L42" s="24" t="inlineStr">
+      <c r="L42" s="23" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
       </c>
-      <c r="M42" s="18" t="n">
+      <c r="M42" s="17" t="n">
         <v>62.9</v>
       </c>
-      <c r="N42" s="28" t="n">
+      <c r="N42" s="25" t="n">
         <v>0.081</v>
       </c>
-      <c r="O42" s="24" t="inlineStr">
+      <c r="O42" s="23" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P42" s="24" t="inlineStr">
+      <c r="P42" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2862,68 +3013,74 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K43" s="12" t="inlineStr"/>
-      <c r="L43" s="13" t="inlineStr"/>
-      <c r="M43" s="12" t="inlineStr"/>
-      <c r="N43" s="14" t="inlineStr"/>
-      <c r="O43" s="13" t="inlineStr">
+      <c r="K43" s="26" t="inlineStr"/>
+      <c r="L43" s="12" t="inlineStr"/>
+      <c r="M43" s="26" t="inlineStr"/>
+      <c r="N43" s="27" t="inlineStr"/>
+      <c r="O43" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P43" s="13" t="inlineStr">
+      <c r="P43" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="15" t="n">
+      <c r="A44" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>10034467</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C44" s="16" t="inlineStr">
         <is>
           <t>SLINDA 4MG 72CP+12PLACEBOS EXELTIS</t>
         </is>
       </c>
-      <c r="D44" s="18" t="n">
+      <c r="D44" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E44" s="18" t="n">
+      <c r="E44" s="17" t="n">
         <v>493.16</v>
       </c>
-      <c r="F44" s="19" t="n">
+      <c r="F44" s="18" t="n">
         <v>-493.16</v>
       </c>
-      <c r="G44" s="20" t="n">
+      <c r="G44" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H44" s="21" t="n">
+      <c r="H44" s="20" t="n">
         <v>3854</v>
       </c>
-      <c r="I44" s="22" t="n">
+      <c r="I44" s="21" t="n">
         <v>3.06</v>
       </c>
-      <c r="J44" s="15" t="inlineStr">
+      <c r="J44" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K44" s="23" t="inlineStr"/>
-      <c r="L44" s="24" t="inlineStr"/>
-      <c r="M44" s="23" t="inlineStr"/>
-      <c r="N44" s="25" t="inlineStr"/>
-      <c r="O44" s="24" t="inlineStr">
+      <c r="K44" s="22" t="inlineStr"/>
+      <c r="L44" s="23" t="inlineStr">
+        <is>
+          <t>DROGARAIA</t>
+        </is>
+      </c>
+      <c r="M44" s="17" t="n">
+        <v>234.98</v>
+      </c>
+      <c r="N44" s="24" t="inlineStr"/>
+      <c r="O44" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P44" s="24" t="inlineStr">
+      <c r="P44" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -2958,7 +3115,7 @@
       <c r="H45" s="10" t="n">
         <v>666</v>
       </c>
-      <c r="I45" s="27" t="n">
+      <c r="I45" s="30" t="n">
         <v>0.53</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -2966,68 +3123,68 @@
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K45" s="12" t="inlineStr"/>
-      <c r="L45" s="13" t="inlineStr"/>
-      <c r="M45" s="12" t="inlineStr"/>
-      <c r="N45" s="14" t="inlineStr"/>
-      <c r="O45" s="13" t="inlineStr">
+      <c r="K45" s="26" t="inlineStr"/>
+      <c r="L45" s="12" t="inlineStr"/>
+      <c r="M45" s="26" t="inlineStr"/>
+      <c r="N45" s="27" t="inlineStr"/>
+      <c r="O45" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P45" s="13" t="inlineStr">
+      <c r="P45" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="15" t="n">
+      <c r="A46" s="14" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>10046473</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr">
+      <c r="C46" s="16" t="inlineStr">
         <is>
           <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 32UN</t>
         </is>
       </c>
-      <c r="D46" s="18" t="n">
+      <c r="D46" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E46" s="18" t="n">
+      <c r="E46" s="17" t="n">
         <v>471.47</v>
       </c>
-      <c r="F46" s="19" t="n">
+      <c r="F46" s="18" t="n">
         <v>-471.47</v>
       </c>
-      <c r="G46" s="20" t="n">
+      <c r="G46" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H46" s="21" t="n">
+      <c r="H46" s="20" t="n">
         <v>19751</v>
       </c>
-      <c r="I46" s="22" t="n">
+      <c r="I46" s="21" t="n">
         <v>15.69</v>
       </c>
-      <c r="J46" s="15" t="inlineStr">
+      <c r="J46" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K46" s="23" t="inlineStr"/>
-      <c r="L46" s="24" t="inlineStr"/>
-      <c r="M46" s="23" t="inlineStr"/>
-      <c r="N46" s="25" t="inlineStr"/>
-      <c r="O46" s="24" t="inlineStr">
+      <c r="K46" s="22" t="inlineStr"/>
+      <c r="L46" s="23" t="inlineStr"/>
+      <c r="M46" s="22" t="inlineStr"/>
+      <c r="N46" s="24" t="inlineStr"/>
+      <c r="O46" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P46" s="24" t="inlineStr">
+      <c r="P46" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3073,7 +3230,7 @@
       <c r="K47" s="7" t="n">
         <v>25.9</v>
       </c>
-      <c r="L47" s="13" t="inlineStr">
+      <c r="L47" s="12" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
@@ -3081,77 +3238,77 @@
       <c r="M47" s="7" t="n">
         <v>15.9</v>
       </c>
-      <c r="N47" s="29" t="n">
+      <c r="N47" s="31" t="n">
         <v>0.629</v>
       </c>
-      <c r="O47" s="13" t="inlineStr">
+      <c r="O47" s="12" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P47" s="13" t="inlineStr">
+      <c r="P47" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="15" t="n">
+      <c r="A48" s="14" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="16" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>100013179</t>
         </is>
       </c>
-      <c r="C48" s="17" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
         <is>
           <t>UTROGESTAN 200MG 42CAP BESINS</t>
         </is>
       </c>
-      <c r="D48" s="18" t="n">
+      <c r="D48" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E48" s="18" t="n">
+      <c r="E48" s="17" t="n">
         <v>468.79</v>
       </c>
-      <c r="F48" s="19" t="n">
+      <c r="F48" s="18" t="n">
         <v>-468.79</v>
       </c>
-      <c r="G48" s="20" t="n">
+      <c r="G48" s="19" t="n">
         <v>-1</v>
       </c>
-      <c r="H48" s="21" t="n">
+      <c r="H48" s="20" t="n">
         <v>3370</v>
       </c>
-      <c r="I48" s="22" t="n">
+      <c r="I48" s="21" t="n">
         <v>2.68</v>
       </c>
-      <c r="J48" s="15" t="inlineStr">
+      <c r="J48" s="14" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="K48" s="17" t="n">
         <v>246.91</v>
       </c>
-      <c r="L48" s="24" t="inlineStr">
+      <c r="L48" s="23" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="M48" s="17" t="n">
         <v>209.07</v>
       </c>
-      <c r="N48" s="28" t="n">
+      <c r="N48" s="25" t="n">
         <v>0.181</v>
       </c>
-      <c r="O48" s="24" t="inlineStr">
+      <c r="O48" s="23" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P48" s="24" t="inlineStr">
+      <c r="P48" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3194,68 +3351,78 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K49" s="12" t="inlineStr"/>
-      <c r="L49" s="13" t="inlineStr"/>
-      <c r="M49" s="12" t="inlineStr"/>
-      <c r="N49" s="14" t="inlineStr"/>
-      <c r="O49" s="13" t="inlineStr">
+      <c r="K49" s="7" t="n">
+        <v>1617.66</v>
+      </c>
+      <c r="L49" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M49" s="7" t="n">
+        <v>1617.66</v>
+      </c>
+      <c r="N49" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="12" t="inlineStr">
+        <is>
+          <t>Preço Alinhado</t>
+        </is>
+      </c>
+      <c r="P49" s="12" t="inlineStr">
+        <is>
+          <t>Neutro</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>10052539</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="n">
+        <v>727.24</v>
+      </c>
+      <c r="E50" s="17" t="n">
+        <v>1174.13</v>
+      </c>
+      <c r="F50" s="18" t="n">
+        <v>-446.89</v>
+      </c>
+      <c r="G50" s="19" t="n">
+        <v>-0.381</v>
+      </c>
+      <c r="H50" s="20" t="n">
+        <v>5078</v>
+      </c>
+      <c r="I50" s="21" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="J50" s="14" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K50" s="22" t="inlineStr"/>
+      <c r="L50" s="23" t="inlineStr"/>
+      <c r="M50" s="22" t="inlineStr"/>
+      <c r="N50" s="24" t="inlineStr"/>
+      <c r="O50" s="23" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P49" s="13" t="inlineStr">
-        <is>
-          <t>Neutro</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="15" t="n">
-        <v>46</v>
-      </c>
-      <c r="B50" s="16" t="inlineStr">
-        <is>
-          <t>10052539</t>
-        </is>
-      </c>
-      <c r="C50" s="17" t="inlineStr">
-        <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
-        </is>
-      </c>
-      <c r="D50" s="18" t="n">
-        <v>727.24</v>
-      </c>
-      <c r="E50" s="18" t="n">
-        <v>1174.13</v>
-      </c>
-      <c r="F50" s="19" t="n">
-        <v>-446.89</v>
-      </c>
-      <c r="G50" s="20" t="n">
-        <v>-0.381</v>
-      </c>
-      <c r="H50" s="21" t="n">
-        <v>5078</v>
-      </c>
-      <c r="I50" s="22" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="J50" s="15" t="inlineStr">
-        <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="inlineStr"/>
-      <c r="L50" s="24" t="inlineStr"/>
-      <c r="M50" s="23" t="inlineStr"/>
-      <c r="N50" s="25" t="inlineStr"/>
-      <c r="O50" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P50" s="24" t="inlineStr">
+      <c r="P50" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3301,7 +3468,7 @@
       <c r="K51" s="7" t="n">
         <v>170.87</v>
       </c>
-      <c r="L51" s="13" t="inlineStr">
+      <c r="L51" s="12" t="inlineStr">
         <is>
           <t>DROGARAIA</t>
         </is>
@@ -3309,67 +3476,77 @@
       <c r="M51" s="7" t="n">
         <v>125.98</v>
       </c>
-      <c r="N51" s="29" t="n">
+      <c r="N51" s="31" t="n">
         <v>0.356</v>
       </c>
-      <c r="O51" s="13" t="inlineStr">
+      <c r="O51" s="12" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P51" s="13" t="inlineStr">
+      <c r="P51" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="15" t="n">
+      <c r="A52" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="16" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>10022882</t>
         </is>
       </c>
-      <c r="C52" s="17" t="inlineStr">
+      <c r="C52" s="16" t="inlineStr">
         <is>
           <t>ACICLOVIR 400MG 30CP GEN PRATI</t>
         </is>
       </c>
-      <c r="D52" s="18" t="n">
+      <c r="D52" s="17" t="n">
         <v>214.47</v>
       </c>
-      <c r="E52" s="18" t="n">
+      <c r="E52" s="17" t="n">
         <v>646.23</v>
       </c>
-      <c r="F52" s="19" t="n">
+      <c r="F52" s="18" t="n">
         <v>-431.76</v>
       </c>
-      <c r="G52" s="20" t="n">
+      <c r="G52" s="19" t="n">
         <v>-0.6679999999999999</v>
       </c>
-      <c r="H52" s="21" t="n">
+      <c r="H52" s="20" t="n">
         <v>5328</v>
       </c>
-      <c r="I52" s="22" t="n">
+      <c r="I52" s="21" t="n">
         <v>4.23</v>
       </c>
-      <c r="J52" s="15" t="inlineStr">
+      <c r="J52" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K52" s="23" t="inlineStr"/>
-      <c r="L52" s="24" t="inlineStr"/>
-      <c r="M52" s="23" t="inlineStr"/>
-      <c r="N52" s="25" t="inlineStr"/>
-      <c r="O52" s="24" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P52" s="24" t="inlineStr">
+      <c r="K52" s="17" t="n">
+        <v>71.48999999999999</v>
+      </c>
+      <c r="L52" s="23" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M52" s="17" t="n">
+        <v>72.98999999999999</v>
+      </c>
+      <c r="N52" s="29" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="O52" s="23" t="inlineStr">
+        <is>
+          <t>Líder de Preço</t>
+        </is>
+      </c>
+      <c r="P52" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
@@ -3404,127 +3581,137 @@
       <c r="H53" s="10" t="n">
         <v>1755</v>
       </c>
-      <c r="I53" s="27" t="n">
+      <c r="I53" s="30" t="n">
         <v>1.39</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K53" s="12" t="inlineStr"/>
-      <c r="L53" s="13" t="inlineStr"/>
-      <c r="M53" s="12" t="inlineStr"/>
-      <c r="N53" s="14" t="inlineStr"/>
-      <c r="O53" s="13" t="inlineStr">
-        <is>
-          <t>Não Monitorado</t>
-        </is>
-      </c>
-      <c r="P53" s="13" t="inlineStr">
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="n">
+        <v>210.44</v>
+      </c>
+      <c r="L53" s="12" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M53" s="7" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="N53" s="31" t="n">
+        <v>0.403</v>
+      </c>
+      <c r="O53" s="12" t="inlineStr">
+        <is>
+          <t>São João Mais Cara</t>
+        </is>
+      </c>
+      <c r="P53" s="12" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="15" t="n">
+      <c r="A54" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="16" t="inlineStr">
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t>100011848</t>
         </is>
       </c>
-      <c r="C54" s="17" t="inlineStr">
+      <c r="C54" s="16" t="inlineStr">
         <is>
           <t>DES AXE AERO 150ML APOLLO</t>
         </is>
       </c>
-      <c r="D54" s="18" t="n">
+      <c r="D54" s="17" t="n">
         <v>74.3</v>
       </c>
-      <c r="E54" s="18" t="n">
+      <c r="E54" s="17" t="n">
         <v>459.59</v>
       </c>
-      <c r="F54" s="19" t="n">
+      <c r="F54" s="18" t="n">
         <v>-385.29</v>
       </c>
-      <c r="G54" s="20" t="n">
+      <c r="G54" s="19" t="n">
         <v>-0.838</v>
       </c>
-      <c r="H54" s="21" t="n">
+      <c r="H54" s="20" t="n">
         <v>58984</v>
       </c>
-      <c r="I54" s="22" t="n">
+      <c r="I54" s="21" t="n">
         <v>46.85</v>
       </c>
-      <c r="J54" s="15" t="inlineStr">
+      <c r="J54" s="14" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K54" s="18" t="n">
+      <c r="K54" s="17" t="n">
         <v>10.9</v>
       </c>
-      <c r="L54" s="24" t="inlineStr">
+      <c r="L54" s="23" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
       </c>
-      <c r="M54" s="18" t="n">
+      <c r="M54" s="17" t="n">
         <v>8.98</v>
       </c>
-      <c r="N54" s="28" t="n">
+      <c r="N54" s="25" t="n">
         <v>0.214</v>
       </c>
-      <c r="O54" s="24" t="inlineStr">
+      <c r="O54" s="23" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P54" s="24" t="inlineStr">
+      <c r="P54" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
     </row>
     <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="31" t="inlineStr">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t>TOTAL TOP 50</t>
         </is>
       </c>
-      <c r="B55" s="32" t="n"/>
-      <c r="C55" s="32" t="n"/>
-      <c r="D55" s="33">
+      <c r="B55" s="33" t="n"/>
+      <c r="C55" s="33" t="n"/>
+      <c r="D55" s="34">
         <f>SUM(D5:D54)</f>
         <v/>
       </c>
-      <c r="E55" s="33">
+      <c r="E55" s="34">
         <f>SUM(E5:E54)</f>
         <v/>
       </c>
-      <c r="F55" s="34">
+      <c r="F55" s="35">
         <f>SUM(F5:F54)</f>
         <v/>
       </c>
-      <c r="G55" s="35">
+      <c r="G55" s="36">
         <f>(D55-E55)/E55</f>
         <v/>
       </c>
-      <c r="H55" s="36">
+      <c r="H55" s="37">
         <f>SUM(H5:H54)</f>
         <v/>
       </c>
-      <c r="I55" s="37" t="inlineStr"/>
-      <c r="J55" s="37" t="inlineStr"/>
-      <c r="K55" s="37" t="inlineStr"/>
-      <c r="L55" s="37" t="inlineStr"/>
-      <c r="M55" s="37" t="inlineStr"/>
-      <c r="N55" s="37" t="inlineStr"/>
-      <c r="O55" s="37" t="inlineStr"/>
-      <c r="P55" s="37" t="inlineStr"/>
+      <c r="I55" s="38" t="inlineStr"/>
+      <c r="J55" s="38" t="inlineStr"/>
+      <c r="K55" s="38" t="inlineStr"/>
+      <c r="L55" s="38" t="inlineStr"/>
+      <c r="M55" s="38" t="inlineStr"/>
+      <c r="N55" s="38" t="inlineStr"/>
+      <c r="O55" s="38" t="inlineStr"/>
+      <c r="P55" s="38" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat: radar de acao imediata & alertas de preco, ruptura real e explicacao GLP-1
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -209,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -246,6 +246,9 @@
     <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -279,6 +282,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="167" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -304,10 +310,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="10" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -674,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -693,6 +698,7 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -791,6 +797,11 @@
           <t>Classificação</t>
         </is>
       </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Ação Recomendada</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -853,56 +864,66 @@
           <t>Detrator Crítico</t>
         </is>
       </c>
+      <c r="Q5" s="14" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>10042969</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC JUMBO XXG 112UN</t>
         </is>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="18" t="n">
         <v>4012.69</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="18" t="n">
         <v>12516.41</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>-8503.719999999999</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="20" t="n">
         <v>-0.679</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="21" t="n">
         <v>10635</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="22" t="n">
         <v>8.449999999999999</v>
       </c>
-      <c r="J6" s="14" t="inlineStr">
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K6" s="22" t="inlineStr"/>
-      <c r="L6" s="23" t="inlineStr"/>
-      <c r="M6" s="22" t="inlineStr"/>
-      <c r="N6" s="24" t="inlineStr"/>
-      <c r="O6" s="23" t="inlineStr">
+      <c r="K6" s="23" t="inlineStr"/>
+      <c r="L6" s="24" t="inlineStr"/>
+      <c r="M6" s="23" t="inlineStr"/>
+      <c r="N6" s="25" t="inlineStr"/>
+      <c r="O6" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P6" s="23" t="inlineStr">
+      <c r="P6" s="24" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
+        </is>
+      </c>
+      <c r="Q6" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -967,56 +988,66 @@
           <t>Detrator Crítico</t>
         </is>
       </c>
+      <c r="Q7" s="14" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="14" t="n">
+      <c r="A8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>10053130</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>OZIVY 1MG 1CAN 3ML EMS</t>
         </is>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="18" t="n">
         <v>4925.62</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="18" t="n">
         <v>11345.16</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>-6419.54</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="20" t="n">
         <v>-0.5660000000000001</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="21" t="n">
         <v>12111</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="22" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="J8" s="14" t="inlineStr">
+      <c r="J8" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K8" s="22" t="inlineStr"/>
-      <c r="L8" s="23" t="inlineStr"/>
-      <c r="M8" s="22" t="inlineStr"/>
-      <c r="N8" s="24" t="inlineStr"/>
-      <c r="O8" s="23" t="inlineStr">
+      <c r="K8" s="23" t="inlineStr"/>
+      <c r="L8" s="24" t="inlineStr"/>
+      <c r="M8" s="23" t="inlineStr"/>
+      <c r="N8" s="25" t="inlineStr"/>
+      <c r="O8" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P8" s="23" t="inlineStr">
+      <c r="P8" s="24" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
+        </is>
+      </c>
+      <c r="Q8" s="26" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -1081,66 +1112,76 @@
           <t>Detrator Crítico</t>
         </is>
       </c>
+      <c r="Q9" s="14" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="14" t="n">
+      <c r="A10" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>10042968</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC JUMBO XG 116UN</t>
         </is>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="18" t="n">
         <v>2720.52</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="18" t="n">
         <v>7721.22</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>-5000.7</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="20" t="n">
         <v>-0.648</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="21" t="n">
         <v>2116</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="22" t="n">
         <v>1.68</v>
       </c>
-      <c r="J10" s="14" t="inlineStr">
+      <c r="J10" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="K10" s="18" t="n">
         <v>159.9</v>
       </c>
-      <c r="L10" s="23" t="inlineStr">
+      <c r="L10" s="24" t="inlineStr">
         <is>
           <t>PANVEL</t>
         </is>
       </c>
-      <c r="M10" s="17" t="n">
+      <c r="M10" s="18" t="n">
         <v>149.9</v>
       </c>
-      <c r="N10" s="25" t="n">
+      <c r="N10" s="27" t="n">
         <v>0.067</v>
       </c>
-      <c r="O10" s="23" t="inlineStr">
+      <c r="O10" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P10" s="23" t="inlineStr">
+      <c r="P10" s="24" t="inlineStr">
         <is>
           <t>Detrator Crítico</t>
+        </is>
+      </c>
+      <c r="Q10" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Panvel R$ 149.90)</t>
         </is>
       </c>
     </row>
@@ -1181,10 +1222,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K11" s="26" t="inlineStr"/>
+      <c r="K11" s="28" t="inlineStr"/>
       <c r="L11" s="12" t="inlineStr"/>
-      <c r="M11" s="26" t="inlineStr"/>
-      <c r="N11" s="27" t="inlineStr"/>
+      <c r="M11" s="28" t="inlineStr"/>
+      <c r="N11" s="29" t="inlineStr"/>
       <c r="O11" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1195,66 +1236,76 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q11" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="14" t="n">
+      <c r="A12" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>10040801</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>WEGOVY 1,7MG 3ML NOVO NORDISK</t>
         </is>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="18" t="n">
         <v>2523.62</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <v>-2523.62</v>
       </c>
-      <c r="G12" s="19" t="n">
+      <c r="G12" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="H12" s="21" t="n">
         <v>1770</v>
       </c>
-      <c r="I12" s="28" t="n">
+      <c r="I12" s="30" t="n">
         <v>1.41</v>
       </c>
-      <c r="J12" s="14" t="inlineStr">
+      <c r="J12" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K12" s="17" t="n">
+      <c r="K12" s="18" t="n">
         <v>1945.09</v>
       </c>
-      <c r="L12" s="23" t="inlineStr">
+      <c r="L12" s="24" t="inlineStr">
         <is>
           <t>PANVEL</t>
         </is>
       </c>
-      <c r="M12" s="17" t="n">
+      <c r="M12" s="18" t="n">
         <v>1945.09</v>
       </c>
-      <c r="N12" s="29" t="n">
+      <c r="N12" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="O12" s="23" t="inlineStr">
+      <c r="O12" s="24" t="inlineStr">
         <is>
           <t>Preço Alinhado</t>
         </is>
       </c>
-      <c r="P12" s="23" t="inlineStr">
+      <c r="P12" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q12" s="26" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -1319,56 +1370,66 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q13" s="14" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="14" t="n">
+      <c r="A14" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>10041262</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
         </is>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="18" t="n">
         <v>1047.81</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="18" t="n">
         <v>3042.52</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>-1994.71</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="20" t="n">
         <v>-0.6559999999999999</v>
       </c>
-      <c r="H14" s="20" t="n">
+      <c r="H14" s="21" t="n">
         <v>2289</v>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="22" t="n">
         <v>1.82</v>
       </c>
-      <c r="J14" s="14" t="inlineStr">
+      <c r="J14" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K14" s="22" t="inlineStr"/>
-      <c r="L14" s="23" t="inlineStr"/>
-      <c r="M14" s="22" t="inlineStr"/>
-      <c r="N14" s="24" t="inlineStr"/>
-      <c r="O14" s="23" t="inlineStr">
+      <c r="K14" s="23" t="inlineStr"/>
+      <c r="L14" s="24" t="inlineStr"/>
+      <c r="M14" s="23" t="inlineStr"/>
+      <c r="N14" s="25" t="inlineStr"/>
+      <c r="O14" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P14" s="23" t="inlineStr">
+      <c r="P14" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q14" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1409,10 +1470,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K15" s="26" t="inlineStr"/>
+      <c r="K15" s="28" t="inlineStr"/>
       <c r="L15" s="12" t="inlineStr"/>
-      <c r="M15" s="26" t="inlineStr"/>
-      <c r="N15" s="27" t="inlineStr"/>
+      <c r="M15" s="28" t="inlineStr"/>
+      <c r="N15" s="29" t="inlineStr"/>
       <c r="O15" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1423,56 +1484,66 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q15" s="14" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="14" t="n">
+      <c r="A16" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>10052534</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
         </is>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="18" t="n">
         <v>571.85</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="18" t="n">
         <v>1968.69</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <v>-1396.84</v>
       </c>
-      <c r="G16" s="19" t="n">
+      <c r="G16" s="20" t="n">
         <v>-0.71</v>
       </c>
-      <c r="H16" s="20" t="n">
+      <c r="H16" s="21" t="n">
         <v>8641</v>
       </c>
-      <c r="I16" s="21" t="n">
+      <c r="I16" s="22" t="n">
         <v>6.86</v>
       </c>
-      <c r="J16" s="14" t="inlineStr">
+      <c r="J16" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K16" s="22" t="inlineStr"/>
-      <c r="L16" s="23" t="inlineStr"/>
-      <c r="M16" s="22" t="inlineStr"/>
-      <c r="N16" s="24" t="inlineStr"/>
-      <c r="O16" s="23" t="inlineStr">
+      <c r="K16" s="23" t="inlineStr"/>
+      <c r="L16" s="24" t="inlineStr"/>
+      <c r="M16" s="23" t="inlineStr"/>
+      <c r="N16" s="25" t="inlineStr"/>
+      <c r="O16" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P16" s="23" t="inlineStr">
+      <c r="P16" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q16" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1576,7 @@
       <c r="H17" s="10" t="n">
         <v>1277</v>
       </c>
-      <c r="I17" s="30" t="n">
+      <c r="I17" s="32" t="n">
         <v>1.01</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1513,10 +1584,10 @@
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K17" s="26" t="inlineStr"/>
+      <c r="K17" s="28" t="inlineStr"/>
       <c r="L17" s="12" t="inlineStr"/>
-      <c r="M17" s="26" t="inlineStr"/>
-      <c r="N17" s="27" t="inlineStr"/>
+      <c r="M17" s="28" t="inlineStr"/>
+      <c r="N17" s="29" t="inlineStr"/>
       <c r="O17" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1527,56 +1598,66 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q17" s="14" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="14" t="n">
+      <c r="A18" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>10041263</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
         </is>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="18" t="n">
         <v>95.90000000000001</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="18" t="n">
         <v>1409.57</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="19" t="n">
         <v>-1313.67</v>
       </c>
-      <c r="G18" s="19" t="n">
+      <c r="G18" s="20" t="n">
         <v>-0.9320000000000001</v>
       </c>
-      <c r="H18" s="20" t="n">
+      <c r="H18" s="21" t="n">
         <v>3254</v>
       </c>
-      <c r="I18" s="21" t="n">
+      <c r="I18" s="22" t="n">
         <v>2.58</v>
       </c>
-      <c r="J18" s="14" t="inlineStr">
+      <c r="J18" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K18" s="22" t="inlineStr"/>
-      <c r="L18" s="23" t="inlineStr"/>
-      <c r="M18" s="22" t="inlineStr"/>
-      <c r="N18" s="24" t="inlineStr"/>
-      <c r="O18" s="23" t="inlineStr">
+      <c r="K18" s="23" t="inlineStr"/>
+      <c r="L18" s="24" t="inlineStr"/>
+      <c r="M18" s="23" t="inlineStr"/>
+      <c r="N18" s="25" t="inlineStr"/>
+      <c r="O18" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P18" s="23" t="inlineStr">
+      <c r="P18" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q18" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1617,10 +1698,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K19" s="26" t="inlineStr"/>
+      <c r="K19" s="28" t="inlineStr"/>
       <c r="L19" s="12" t="inlineStr"/>
-      <c r="M19" s="26" t="inlineStr"/>
-      <c r="N19" s="27" t="inlineStr"/>
+      <c r="M19" s="28" t="inlineStr"/>
+      <c r="N19" s="29" t="inlineStr"/>
       <c r="O19" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1631,66 +1712,76 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q19" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="14" t="n">
+      <c r="A20" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>100016230</t>
         </is>
       </c>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>NEUTROGENA GEL HID FACIAL 50G HYDRO BOOST WATER</t>
         </is>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="17" t="n">
+      <c r="E20" s="18" t="n">
         <v>1205.31</v>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="19" t="n">
         <v>-1205.31</v>
       </c>
-      <c r="G20" s="19" t="n">
+      <c r="G20" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H20" s="20" t="n">
+      <c r="H20" s="21" t="n">
         <v>4849</v>
       </c>
-      <c r="I20" s="21" t="n">
+      <c r="I20" s="22" t="n">
         <v>3.85</v>
       </c>
-      <c r="J20" s="14" t="inlineStr">
+      <c r="J20" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K20" s="17" t="n">
+      <c r="K20" s="18" t="n">
         <v>94.98999999999999</v>
       </c>
-      <c r="L20" s="23" t="inlineStr">
+      <c r="L20" s="24" t="inlineStr">
         <is>
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="M20" s="17" t="n">
+      <c r="M20" s="18" t="n">
         <v>49.9</v>
       </c>
-      <c r="N20" s="25" t="n">
+      <c r="N20" s="27" t="n">
         <v>0.904</v>
       </c>
-      <c r="O20" s="23" t="inlineStr">
+      <c r="O20" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P20" s="23" t="inlineStr">
+      <c r="P20" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q20" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 49.90)</t>
         </is>
       </c>
     </row>
@@ -1731,10 +1822,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K21" s="26" t="inlineStr"/>
+      <c r="K21" s="28" t="inlineStr"/>
       <c r="L21" s="12" t="inlineStr"/>
-      <c r="M21" s="26" t="inlineStr"/>
-      <c r="N21" s="27" t="inlineStr"/>
+      <c r="M21" s="28" t="inlineStr"/>
+      <c r="N21" s="29" t="inlineStr"/>
       <c r="O21" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1745,56 +1836,66 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q21" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="14" t="n">
+      <c r="A22" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>10042966</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC JUMBO M 148UN</t>
         </is>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="18" t="n">
         <v>766.9299999999999</v>
       </c>
-      <c r="E22" s="17" t="n">
+      <c r="E22" s="18" t="n">
         <v>1866.75</v>
       </c>
-      <c r="F22" s="18" t="n">
+      <c r="F22" s="19" t="n">
         <v>-1099.82</v>
       </c>
-      <c r="G22" s="19" t="n">
+      <c r="G22" s="20" t="n">
         <v>-0.589</v>
       </c>
-      <c r="H22" s="20" t="n">
+      <c r="H22" s="21" t="n">
         <v>3834</v>
       </c>
-      <c r="I22" s="21" t="n">
+      <c r="I22" s="22" t="n">
         <v>3.05</v>
       </c>
-      <c r="J22" s="14" t="inlineStr">
+      <c r="J22" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K22" s="22" t="inlineStr"/>
-      <c r="L22" s="23" t="inlineStr"/>
-      <c r="M22" s="22" t="inlineStr"/>
-      <c r="N22" s="24" t="inlineStr"/>
-      <c r="O22" s="23" t="inlineStr">
+      <c r="K22" s="23" t="inlineStr"/>
+      <c r="L22" s="24" t="inlineStr"/>
+      <c r="M22" s="23" t="inlineStr"/>
+      <c r="N22" s="25" t="inlineStr"/>
+      <c r="O22" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P22" s="23" t="inlineStr">
+      <c r="P22" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q22" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1947,7 @@
       <c r="M23" s="7" t="n">
         <v>107</v>
       </c>
-      <c r="N23" s="31" t="n">
+      <c r="N23" s="33" t="n">
         <v>0.396</v>
       </c>
       <c r="O23" s="12" t="inlineStr">
@@ -1859,66 +1960,76 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q23" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 107.00)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="14" t="n">
+      <c r="A24" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>10050440</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>AMMY 4MG 72CP REV MANTECORP</t>
         </is>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="17" t="n">
+      <c r="E24" s="18" t="n">
         <v>1030.93</v>
       </c>
-      <c r="F24" s="18" t="n">
+      <c r="F24" s="19" t="n">
         <v>-1030.93</v>
       </c>
-      <c r="G24" s="19" t="n">
+      <c r="G24" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H24" s="20" t="n">
+      <c r="H24" s="21" t="n">
         <v>864</v>
       </c>
-      <c r="I24" s="28" t="n">
+      <c r="I24" s="30" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="J24" s="14" t="inlineStr">
+      <c r="J24" s="15" t="inlineStr">
         <is>
           <t>⚠️ Duplo Detrator</t>
         </is>
       </c>
-      <c r="K24" s="17" t="n">
+      <c r="K24" s="18" t="n">
         <v>315.46</v>
       </c>
-      <c r="L24" s="23" t="inlineStr">
+      <c r="L24" s="24" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
       </c>
-      <c r="M24" s="17" t="n">
+      <c r="M24" s="18" t="n">
         <v>236.6</v>
       </c>
-      <c r="N24" s="25" t="n">
+      <c r="N24" s="27" t="n">
         <v>0.333</v>
       </c>
-      <c r="O24" s="23" t="inlineStr">
+      <c r="O24" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P24" s="23" t="inlineStr">
+      <c r="P24" s="24" t="inlineStr">
         <is>
           <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q24" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar e Remanejar (Precopopular R$ 236.60)</t>
         </is>
       </c>
     </row>
@@ -1983,62 +2094,72 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
+      <c r="Q25" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="14" t="n">
+      <c r="A26" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>10034724</t>
         </is>
       </c>
-      <c r="C26" s="16" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>CONTRAVE 8+90MG 120CP REV LIB PROL MERCK (C1)</t>
         </is>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="17" t="n">
+      <c r="E26" s="18" t="n">
         <v>944.51</v>
       </c>
-      <c r="F26" s="18" t="n">
+      <c r="F26" s="19" t="n">
         <v>-944.51</v>
       </c>
-      <c r="G26" s="19" t="n">
+      <c r="G26" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H26" s="20" t="n">
+      <c r="H26" s="21" t="n">
         <v>2108</v>
       </c>
-      <c r="I26" s="21" t="n">
+      <c r="I26" s="22" t="n">
         <v>1.67</v>
       </c>
-      <c r="J26" s="14" t="inlineStr">
+      <c r="J26" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K26" s="22" t="inlineStr"/>
-      <c r="L26" s="23" t="inlineStr">
+      <c r="K26" s="23" t="inlineStr"/>
+      <c r="L26" s="24" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
       </c>
-      <c r="M26" s="17" t="n">
+      <c r="M26" s="18" t="n">
         <v>549.9</v>
       </c>
-      <c r="N26" s="24" t="inlineStr"/>
-      <c r="O26" s="23" t="inlineStr">
+      <c r="N26" s="25" t="inlineStr"/>
+      <c r="O26" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P26" s="23" t="inlineStr">
+      <c r="P26" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q26" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2103,56 +2224,66 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q27" s="14" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="14" t="n">
+      <c r="A28" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>10052533</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
         </is>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <v>695.4</v>
       </c>
-      <c r="E28" s="17" t="n">
+      <c r="E28" s="18" t="n">
         <v>1568.39</v>
       </c>
-      <c r="F28" s="18" t="n">
+      <c r="F28" s="19" t="n">
         <v>-872.99</v>
       </c>
-      <c r="G28" s="19" t="n">
+      <c r="G28" s="20" t="n">
         <v>-0.5570000000000001</v>
       </c>
-      <c r="H28" s="20" t="n">
+      <c r="H28" s="21" t="n">
         <v>16250</v>
       </c>
-      <c r="I28" s="21" t="n">
+      <c r="I28" s="22" t="n">
         <v>12.91</v>
       </c>
-      <c r="J28" s="14" t="inlineStr">
+      <c r="J28" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K28" s="22" t="inlineStr"/>
-      <c r="L28" s="23" t="inlineStr"/>
-      <c r="M28" s="22" t="inlineStr"/>
-      <c r="N28" s="24" t="inlineStr"/>
-      <c r="O28" s="23" t="inlineStr">
+      <c r="K28" s="23" t="inlineStr"/>
+      <c r="L28" s="24" t="inlineStr"/>
+      <c r="M28" s="23" t="inlineStr"/>
+      <c r="N28" s="25" t="inlineStr"/>
+      <c r="O28" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P28" s="23" t="inlineStr">
+      <c r="P28" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q28" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2316,7 @@
       <c r="H29" s="10" t="n">
         <v>212</v>
       </c>
-      <c r="I29" s="30" t="n">
+      <c r="I29" s="32" t="n">
         <v>0.17</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2193,7 +2324,7 @@
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K29" s="26" t="inlineStr"/>
+      <c r="K29" s="28" t="inlineStr"/>
       <c r="L29" s="12" t="inlineStr">
         <is>
           <t>PANVEL</t>
@@ -2202,7 +2333,7 @@
       <c r="M29" s="7" t="n">
         <v>1212.9</v>
       </c>
-      <c r="N29" s="27" t="inlineStr"/>
+      <c r="N29" s="29" t="inlineStr"/>
       <c r="O29" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -2213,56 +2344,66 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q29" s="14" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="14" t="n">
+      <c r="A30" s="15" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>10053171</t>
         </is>
       </c>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>OZIVY 0,25MG+0,5MG 1CAN 1,5ML EMS</t>
         </is>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="17" t="n">
+      <c r="E30" s="18" t="n">
         <v>754.62</v>
       </c>
-      <c r="F30" s="18" t="n">
+      <c r="F30" s="19" t="n">
         <v>-754.62</v>
       </c>
-      <c r="G30" s="19" t="n">
+      <c r="G30" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H30" s="20" t="n">
+      <c r="H30" s="21" t="n">
         <v>1643</v>
       </c>
-      <c r="I30" s="28" t="n">
+      <c r="I30" s="30" t="n">
         <v>1.31</v>
       </c>
-      <c r="J30" s="14" t="inlineStr">
+      <c r="J30" s="15" t="inlineStr">
         <is>
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K30" s="22" t="inlineStr"/>
-      <c r="L30" s="23" t="inlineStr"/>
-      <c r="M30" s="22" t="inlineStr"/>
-      <c r="N30" s="24" t="inlineStr"/>
-      <c r="O30" s="23" t="inlineStr">
+      <c r="K30" s="23" t="inlineStr"/>
+      <c r="L30" s="24" t="inlineStr"/>
+      <c r="M30" s="23" t="inlineStr"/>
+      <c r="N30" s="25" t="inlineStr"/>
+      <c r="O30" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P30" s="23" t="inlineStr">
+      <c r="P30" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q30" s="26" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2455,7 @@
       <c r="M31" s="7" t="n">
         <v>55.67</v>
       </c>
-      <c r="N31" s="31" t="n">
+      <c r="N31" s="33" t="n">
         <v>0.333</v>
       </c>
       <c r="O31" s="12" t="inlineStr">
@@ -2327,66 +2468,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q31" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 55.67)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="14" t="n">
+      <c r="A32" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="15" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>10030120</t>
         </is>
       </c>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
         <is>
           <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
         </is>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D32" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="17" t="n">
+      <c r="E32" s="18" t="n">
         <v>691.48</v>
       </c>
-      <c r="F32" s="18" t="n">
+      <c r="F32" s="19" t="n">
         <v>-691.48</v>
       </c>
-      <c r="G32" s="19" t="n">
+      <c r="G32" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H32" s="20" t="n">
+      <c r="H32" s="21" t="n">
         <v>2004</v>
       </c>
-      <c r="I32" s="21" t="n">
+      <c r="I32" s="22" t="n">
         <v>1.59</v>
       </c>
-      <c r="J32" s="14" t="inlineStr">
+      <c r="J32" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K32" s="17" t="n">
+      <c r="K32" s="18" t="n">
         <v>1301.17</v>
       </c>
-      <c r="L32" s="23" t="inlineStr">
+      <c r="L32" s="24" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
       </c>
-      <c r="M32" s="17" t="n">
+      <c r="M32" s="18" t="n">
         <v>1301.17</v>
       </c>
-      <c r="N32" s="29" t="n">
+      <c r="N32" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="O32" s="23" t="inlineStr">
+      <c r="O32" s="24" t="inlineStr">
         <is>
           <t>Preço Alinhado</t>
         </is>
       </c>
-      <c r="P32" s="23" t="inlineStr">
+      <c r="P32" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q32" s="26" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -2427,10 +2578,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K33" s="26" t="inlineStr"/>
+      <c r="K33" s="28" t="inlineStr"/>
       <c r="L33" s="12" t="inlineStr"/>
-      <c r="M33" s="26" t="inlineStr"/>
-      <c r="N33" s="27" t="inlineStr"/>
+      <c r="M33" s="28" t="inlineStr"/>
+      <c r="N33" s="29" t="inlineStr"/>
       <c r="O33" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -2441,66 +2592,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q33" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="14" t="n">
+      <c r="A34" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="15" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>10049094</t>
         </is>
       </c>
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C34" s="17" t="inlineStr">
         <is>
           <t>NUSTENDI 180MG/10MG 30CP DAIICHI</t>
         </is>
       </c>
-      <c r="D34" s="17" t="n">
+      <c r="D34" s="18" t="n">
         <v>203.67</v>
       </c>
-      <c r="E34" s="17" t="n">
+      <c r="E34" s="18" t="n">
         <v>860.5700000000001</v>
       </c>
-      <c r="F34" s="18" t="n">
+      <c r="F34" s="19" t="n">
         <v>-656.9</v>
       </c>
-      <c r="G34" s="19" t="n">
+      <c r="G34" s="20" t="n">
         <v>-0.763</v>
       </c>
-      <c r="H34" s="20" t="n">
+      <c r="H34" s="21" t="n">
         <v>2850</v>
       </c>
-      <c r="I34" s="21" t="n">
+      <c r="I34" s="22" t="n">
         <v>2.26</v>
       </c>
-      <c r="J34" s="14" t="inlineStr">
+      <c r="J34" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K34" s="17" t="n">
+      <c r="K34" s="18" t="n">
         <v>218.67</v>
       </c>
-      <c r="L34" s="23" t="inlineStr">
+      <c r="L34" s="24" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
       </c>
-      <c r="M34" s="17" t="n">
+      <c r="M34" s="18" t="n">
         <v>197.18</v>
       </c>
-      <c r="N34" s="25" t="n">
+      <c r="N34" s="27" t="n">
         <v>0.109</v>
       </c>
-      <c r="O34" s="23" t="inlineStr">
+      <c r="O34" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P34" s="23" t="inlineStr">
+      <c r="P34" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q34" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 197.18)</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2713,7 @@
       <c r="M35" s="7" t="n">
         <v>115.9</v>
       </c>
-      <c r="N35" s="31" t="n">
+      <c r="N35" s="33" t="n">
         <v>0.416</v>
       </c>
       <c r="O35" s="12" t="inlineStr">
@@ -2565,66 +2726,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q35" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 115.90)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="14" t="n">
+      <c r="A36" s="15" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="15" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>10097312</t>
         </is>
       </c>
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>NESTOGENO 2 800G NESTLE</t>
         </is>
       </c>
-      <c r="D36" s="17" t="n">
+      <c r="D36" s="18" t="n">
         <v>271.96</v>
       </c>
-      <c r="E36" s="17" t="n">
+      <c r="E36" s="18" t="n">
         <v>841.95</v>
       </c>
-      <c r="F36" s="18" t="n">
+      <c r="F36" s="19" t="n">
         <v>-569.99</v>
       </c>
-      <c r="G36" s="19" t="n">
+      <c r="G36" s="20" t="n">
         <v>-0.677</v>
       </c>
-      <c r="H36" s="20" t="n">
+      <c r="H36" s="21" t="n">
         <v>13240</v>
       </c>
-      <c r="I36" s="21" t="n">
+      <c r="I36" s="22" t="n">
         <v>10.52</v>
       </c>
-      <c r="J36" s="14" t="inlineStr">
+      <c r="J36" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K36" s="17" t="n">
+      <c r="K36" s="18" t="n">
         <v>67.98999999999999</v>
       </c>
-      <c r="L36" s="23" t="inlineStr">
+      <c r="L36" s="24" t="inlineStr">
         <is>
           <t>DROGARAIA</t>
         </is>
       </c>
-      <c r="M36" s="17" t="n">
+      <c r="M36" s="18" t="n">
         <v>61.06</v>
       </c>
-      <c r="N36" s="25" t="n">
+      <c r="N36" s="27" t="n">
         <v>0.113</v>
       </c>
-      <c r="O36" s="23" t="inlineStr">
+      <c r="O36" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P36" s="23" t="inlineStr">
+      <c r="P36" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q36" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Drogaraia R$ 61.06)</t>
         </is>
       </c>
     </row>
@@ -2665,10 +2836,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K37" s="26" t="inlineStr"/>
+      <c r="K37" s="28" t="inlineStr"/>
       <c r="L37" s="12" t="inlineStr"/>
-      <c r="M37" s="26" t="inlineStr"/>
-      <c r="N37" s="27" t="inlineStr"/>
+      <c r="M37" s="28" t="inlineStr"/>
+      <c r="N37" s="29" t="inlineStr"/>
       <c r="O37" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -2679,66 +2850,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q37" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="14" t="n">
+      <c r="A38" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>100011547</t>
         </is>
       </c>
-      <c r="C38" s="16" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
         <is>
           <t>NAN SUPREME 1 800G NESTLE</t>
         </is>
       </c>
-      <c r="D38" s="17" t="n">
+      <c r="D38" s="18" t="n">
         <v>132.49</v>
       </c>
-      <c r="E38" s="17" t="n">
+      <c r="E38" s="18" t="n">
         <v>685.71</v>
       </c>
-      <c r="F38" s="18" t="n">
+      <c r="F38" s="19" t="n">
         <v>-553.22</v>
       </c>
-      <c r="G38" s="19" t="n">
+      <c r="G38" s="20" t="n">
         <v>-0.8070000000000001</v>
       </c>
-      <c r="H38" s="20" t="n">
+      <c r="H38" s="21" t="n">
         <v>8308</v>
       </c>
-      <c r="I38" s="21" t="n">
+      <c r="I38" s="22" t="n">
         <v>6.6</v>
       </c>
-      <c r="J38" s="14" t="inlineStr">
+      <c r="J38" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K38" s="17" t="n">
+      <c r="K38" s="18" t="n">
         <v>132.49</v>
       </c>
-      <c r="L38" s="23" t="inlineStr">
+      <c r="L38" s="24" t="inlineStr">
         <is>
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="M38" s="17" t="n">
+      <c r="M38" s="18" t="n">
         <v>124.19</v>
       </c>
-      <c r="N38" s="25" t="n">
+      <c r="N38" s="27" t="n">
         <v>0.067</v>
       </c>
-      <c r="O38" s="23" t="inlineStr">
+      <c r="O38" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P38" s="23" t="inlineStr">
+      <c r="P38" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q38" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 124.19)</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2971,7 @@
       <c r="M39" s="7" t="n">
         <v>59.9</v>
       </c>
-      <c r="N39" s="31" t="n">
+      <c r="N39" s="33" t="n">
         <v>0.167</v>
       </c>
       <c r="O39" s="12" t="inlineStr">
@@ -2803,56 +2984,66 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q39" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 59.90)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="14" t="n">
+      <c r="A40" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B40" s="16" t="inlineStr">
         <is>
           <t>100011549</t>
         </is>
       </c>
-      <c r="C40" s="16" t="inlineStr">
+      <c r="C40" s="17" t="inlineStr">
         <is>
           <t>NAN SUPREME 2 800G NESTLE</t>
         </is>
       </c>
-      <c r="D40" s="17" t="n">
+      <c r="D40" s="18" t="n">
         <v>264.98</v>
       </c>
-      <c r="E40" s="17" t="n">
+      <c r="E40" s="18" t="n">
         <v>806.87</v>
       </c>
-      <c r="F40" s="18" t="n">
+      <c r="F40" s="19" t="n">
         <v>-541.89</v>
       </c>
-      <c r="G40" s="19" t="n">
+      <c r="G40" s="20" t="n">
         <v>-0.672</v>
       </c>
-      <c r="H40" s="20" t="n">
+      <c r="H40" s="21" t="n">
         <v>7821</v>
       </c>
-      <c r="I40" s="21" t="n">
+      <c r="I40" s="22" t="n">
         <v>6.21</v>
       </c>
-      <c r="J40" s="14" t="inlineStr">
+      <c r="J40" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K40" s="22" t="inlineStr"/>
-      <c r="L40" s="23" t="inlineStr"/>
-      <c r="M40" s="22" t="inlineStr"/>
-      <c r="N40" s="24" t="inlineStr"/>
-      <c r="O40" s="23" t="inlineStr">
+      <c r="K40" s="23" t="inlineStr"/>
+      <c r="L40" s="24" t="inlineStr"/>
+      <c r="M40" s="23" t="inlineStr"/>
+      <c r="N40" s="25" t="inlineStr"/>
+      <c r="O40" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P40" s="23" t="inlineStr">
+      <c r="P40" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q40" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2893,7 +3084,7 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K41" s="26" t="inlineStr"/>
+      <c r="K41" s="28" t="inlineStr"/>
       <c r="L41" s="12" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
@@ -2902,7 +3093,7 @@
       <c r="M41" s="7" t="n">
         <v>988.22</v>
       </c>
-      <c r="N41" s="27" t="inlineStr"/>
+      <c r="N41" s="29" t="inlineStr"/>
       <c r="O41" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -2913,66 +3104,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q41" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="14" t="n">
+      <c r="A42" s="15" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t>10097311</t>
         </is>
       </c>
-      <c r="C42" s="16" t="inlineStr">
+      <c r="C42" s="17" t="inlineStr">
         <is>
           <t>NESTOGENO 1 800G NESTLE</t>
         </is>
       </c>
-      <c r="D42" s="17" t="n">
+      <c r="D42" s="18" t="n">
         <v>407.94</v>
       </c>
-      <c r="E42" s="17" t="n">
+      <c r="E42" s="18" t="n">
         <v>932.3200000000001</v>
       </c>
-      <c r="F42" s="18" t="n">
+      <c r="F42" s="19" t="n">
         <v>-524.38</v>
       </c>
-      <c r="G42" s="19" t="n">
+      <c r="G42" s="20" t="n">
         <v>-0.5620000000000001</v>
       </c>
-      <c r="H42" s="20" t="n">
+      <c r="H42" s="21" t="n">
         <v>10934</v>
       </c>
-      <c r="I42" s="21" t="n">
+      <c r="I42" s="22" t="n">
         <v>8.68</v>
       </c>
-      <c r="J42" s="14" t="inlineStr">
+      <c r="J42" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K42" s="17" t="n">
+      <c r="K42" s="18" t="n">
         <v>67.98999999999999</v>
       </c>
-      <c r="L42" s="23" t="inlineStr">
+      <c r="L42" s="24" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
       </c>
-      <c r="M42" s="17" t="n">
+      <c r="M42" s="18" t="n">
         <v>62.9</v>
       </c>
-      <c r="N42" s="25" t="n">
+      <c r="N42" s="27" t="n">
         <v>0.081</v>
       </c>
-      <c r="O42" s="23" t="inlineStr">
+      <c r="O42" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P42" s="23" t="inlineStr">
+      <c r="P42" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q42" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 62.90)</t>
         </is>
       </c>
     </row>
@@ -3013,10 +3214,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K43" s="26" t="inlineStr"/>
+      <c r="K43" s="28" t="inlineStr"/>
       <c r="L43" s="12" t="inlineStr"/>
-      <c r="M43" s="26" t="inlineStr"/>
-      <c r="N43" s="27" t="inlineStr"/>
+      <c r="M43" s="28" t="inlineStr"/>
+      <c r="N43" s="29" t="inlineStr"/>
       <c r="O43" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -3027,62 +3228,72 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q43" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="14" t="n">
+      <c r="A44" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="15" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>10034467</t>
         </is>
       </c>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>SLINDA 4MG 72CP+12PLACEBOS EXELTIS</t>
         </is>
       </c>
-      <c r="D44" s="17" t="n">
+      <c r="D44" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E44" s="17" t="n">
+      <c r="E44" s="18" t="n">
         <v>493.16</v>
       </c>
-      <c r="F44" s="18" t="n">
+      <c r="F44" s="19" t="n">
         <v>-493.16</v>
       </c>
-      <c r="G44" s="19" t="n">
+      <c r="G44" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H44" s="20" t="n">
+      <c r="H44" s="21" t="n">
         <v>3854</v>
       </c>
-      <c r="I44" s="21" t="n">
+      <c r="I44" s="22" t="n">
         <v>3.06</v>
       </c>
-      <c r="J44" s="14" t="inlineStr">
+      <c r="J44" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K44" s="22" t="inlineStr"/>
-      <c r="L44" s="23" t="inlineStr">
+      <c r="K44" s="23" t="inlineStr"/>
+      <c r="L44" s="24" t="inlineStr">
         <is>
           <t>DROGARAIA</t>
         </is>
       </c>
-      <c r="M44" s="17" t="n">
+      <c r="M44" s="18" t="n">
         <v>234.98</v>
       </c>
-      <c r="N44" s="24" t="inlineStr"/>
-      <c r="O44" s="23" t="inlineStr">
+      <c r="N44" s="25" t="inlineStr"/>
+      <c r="O44" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P44" s="23" t="inlineStr">
+      <c r="P44" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q44" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3326,7 @@
       <c r="H45" s="10" t="n">
         <v>666</v>
       </c>
-      <c r="I45" s="30" t="n">
+      <c r="I45" s="32" t="n">
         <v>0.53</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3123,10 +3334,10 @@
           <t>🚨 Ruptura Logística</t>
         </is>
       </c>
-      <c r="K45" s="26" t="inlineStr"/>
+      <c r="K45" s="28" t="inlineStr"/>
       <c r="L45" s="12" t="inlineStr"/>
-      <c r="M45" s="26" t="inlineStr"/>
-      <c r="N45" s="27" t="inlineStr"/>
+      <c r="M45" s="28" t="inlineStr"/>
+      <c r="N45" s="29" t="inlineStr"/>
       <c r="O45" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -3137,56 +3348,66 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q45" s="14" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="14" t="n">
+      <c r="A46" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B46" s="16" t="inlineStr">
         <is>
           <t>10046473</t>
         </is>
       </c>
-      <c r="C46" s="16" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr">
         <is>
           <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 32UN</t>
         </is>
       </c>
-      <c r="D46" s="17" t="n">
+      <c r="D46" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E46" s="17" t="n">
+      <c r="E46" s="18" t="n">
         <v>471.47</v>
       </c>
-      <c r="F46" s="18" t="n">
+      <c r="F46" s="19" t="n">
         <v>-471.47</v>
       </c>
-      <c r="G46" s="19" t="n">
+      <c r="G46" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H46" s="20" t="n">
+      <c r="H46" s="21" t="n">
         <v>19751</v>
       </c>
-      <c r="I46" s="21" t="n">
+      <c r="I46" s="22" t="n">
         <v>15.69</v>
       </c>
-      <c r="J46" s="14" t="inlineStr">
+      <c r="J46" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K46" s="22" t="inlineStr"/>
-      <c r="L46" s="23" t="inlineStr"/>
-      <c r="M46" s="22" t="inlineStr"/>
-      <c r="N46" s="24" t="inlineStr"/>
-      <c r="O46" s="23" t="inlineStr">
+      <c r="K46" s="23" t="inlineStr"/>
+      <c r="L46" s="24" t="inlineStr"/>
+      <c r="M46" s="23" t="inlineStr"/>
+      <c r="N46" s="25" t="inlineStr"/>
+      <c r="O46" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P46" s="23" t="inlineStr">
+      <c r="P46" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q46" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3459,7 @@
       <c r="M47" s="7" t="n">
         <v>15.9</v>
       </c>
-      <c r="N47" s="31" t="n">
+      <c r="N47" s="33" t="n">
         <v>0.629</v>
       </c>
       <c r="O47" s="12" t="inlineStr">
@@ -3251,66 +3472,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q47" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 15.90)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="14" t="n">
+      <c r="A48" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>100013179</t>
         </is>
       </c>
-      <c r="C48" s="16" t="inlineStr">
+      <c r="C48" s="17" t="inlineStr">
         <is>
           <t>UTROGESTAN 200MG 42CAP BESINS</t>
         </is>
       </c>
-      <c r="D48" s="17" t="n">
+      <c r="D48" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E48" s="17" t="n">
+      <c r="E48" s="18" t="n">
         <v>468.79</v>
       </c>
-      <c r="F48" s="18" t="n">
+      <c r="F48" s="19" t="n">
         <v>-468.79</v>
       </c>
-      <c r="G48" s="19" t="n">
+      <c r="G48" s="20" t="n">
         <v>-1</v>
       </c>
-      <c r="H48" s="20" t="n">
+      <c r="H48" s="21" t="n">
         <v>3370</v>
       </c>
-      <c r="I48" s="21" t="n">
+      <c r="I48" s="22" t="n">
         <v>2.68</v>
       </c>
-      <c r="J48" s="14" t="inlineStr">
+      <c r="J48" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K48" s="17" t="n">
+      <c r="K48" s="18" t="n">
         <v>246.91</v>
       </c>
-      <c r="L48" s="23" t="inlineStr">
+      <c r="L48" s="24" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
       </c>
-      <c r="M48" s="17" t="n">
+      <c r="M48" s="18" t="n">
         <v>209.07</v>
       </c>
-      <c r="N48" s="25" t="n">
+      <c r="N48" s="27" t="n">
         <v>0.181</v>
       </c>
-      <c r="O48" s="23" t="inlineStr">
+      <c r="O48" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P48" s="23" t="inlineStr">
+      <c r="P48" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q48" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 209.07)</t>
         </is>
       </c>
     </row>
@@ -3375,56 +3606,66 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q49" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="14" t="n">
+      <c r="A50" s="15" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B50" s="16" t="inlineStr">
         <is>
           <t>10052539</t>
         </is>
       </c>
-      <c r="C50" s="16" t="inlineStr">
+      <c r="C50" s="17" t="inlineStr">
         <is>
           <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
         </is>
       </c>
-      <c r="D50" s="17" t="n">
+      <c r="D50" s="18" t="n">
         <v>727.24</v>
       </c>
-      <c r="E50" s="17" t="n">
+      <c r="E50" s="18" t="n">
         <v>1174.13</v>
       </c>
-      <c r="F50" s="18" t="n">
+      <c r="F50" s="19" t="n">
         <v>-446.89</v>
       </c>
-      <c r="G50" s="19" t="n">
+      <c r="G50" s="20" t="n">
         <v>-0.381</v>
       </c>
-      <c r="H50" s="20" t="n">
+      <c r="H50" s="21" t="n">
         <v>5078</v>
       </c>
-      <c r="I50" s="21" t="n">
+      <c r="I50" s="22" t="n">
         <v>4.03</v>
       </c>
-      <c r="J50" s="14" t="inlineStr">
+      <c r="J50" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K50" s="22" t="inlineStr"/>
-      <c r="L50" s="23" t="inlineStr"/>
-      <c r="M50" s="22" t="inlineStr"/>
-      <c r="N50" s="24" t="inlineStr"/>
-      <c r="O50" s="23" t="inlineStr">
+      <c r="K50" s="23" t="inlineStr"/>
+      <c r="L50" s="24" t="inlineStr"/>
+      <c r="M50" s="23" t="inlineStr"/>
+      <c r="N50" s="25" t="inlineStr"/>
+      <c r="O50" s="24" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
         </is>
       </c>
-      <c r="P50" s="23" t="inlineStr">
+      <c r="P50" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q50" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3717,7 @@
       <c r="M51" s="7" t="n">
         <v>125.98</v>
       </c>
-      <c r="N51" s="31" t="n">
+      <c r="N51" s="33" t="n">
         <v>0.356</v>
       </c>
       <c r="O51" s="12" t="inlineStr">
@@ -3489,66 +3730,76 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q51" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Drogaraia R$ 125.98)</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="14" t="n">
+      <c r="A52" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="15" t="inlineStr">
+      <c r="B52" s="16" t="inlineStr">
         <is>
           <t>10022882</t>
         </is>
       </c>
-      <c r="C52" s="16" t="inlineStr">
+      <c r="C52" s="17" t="inlineStr">
         <is>
           <t>ACICLOVIR 400MG 30CP GEN PRATI</t>
         </is>
       </c>
-      <c r="D52" s="17" t="n">
+      <c r="D52" s="18" t="n">
         <v>214.47</v>
       </c>
-      <c r="E52" s="17" t="n">
+      <c r="E52" s="18" t="n">
         <v>646.23</v>
       </c>
-      <c r="F52" s="18" t="n">
+      <c r="F52" s="19" t="n">
         <v>-431.76</v>
       </c>
-      <c r="G52" s="19" t="n">
+      <c r="G52" s="20" t="n">
         <v>-0.6679999999999999</v>
       </c>
-      <c r="H52" s="20" t="n">
+      <c r="H52" s="21" t="n">
         <v>5328</v>
       </c>
-      <c r="I52" s="21" t="n">
+      <c r="I52" s="22" t="n">
         <v>4.23</v>
       </c>
-      <c r="J52" s="14" t="inlineStr">
+      <c r="J52" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K52" s="17" t="n">
+      <c r="K52" s="18" t="n">
         <v>71.48999999999999</v>
       </c>
-      <c r="L52" s="23" t="inlineStr">
+      <c r="L52" s="24" t="inlineStr">
         <is>
           <t>PANVEL</t>
         </is>
       </c>
-      <c r="M52" s="17" t="n">
+      <c r="M52" s="18" t="n">
         <v>72.98999999999999</v>
       </c>
-      <c r="N52" s="29" t="n">
+      <c r="N52" s="31" t="n">
         <v>-0.021</v>
       </c>
-      <c r="O52" s="23" t="inlineStr">
+      <c r="O52" s="24" t="inlineStr">
         <is>
           <t>Líder de Preço</t>
         </is>
       </c>
-      <c r="P52" s="23" t="inlineStr">
+      <c r="P52" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
+        </is>
+      </c>
+      <c r="Q52" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3832,7 @@
       <c r="H53" s="10" t="n">
         <v>1755</v>
       </c>
-      <c r="I53" s="30" t="n">
+      <c r="I53" s="32" t="n">
         <v>1.39</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -3600,7 +3851,7 @@
       <c r="M53" s="7" t="n">
         <v>149.99</v>
       </c>
-      <c r="N53" s="31" t="n">
+      <c r="N53" s="33" t="n">
         <v>0.403</v>
       </c>
       <c r="O53" s="12" t="inlineStr">
@@ -3613,105 +3864,113 @@
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q53" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar e Remanejar (Amazon R$ 149.99)</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="14" t="n">
+      <c r="A54" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="15" t="inlineStr">
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>100011848</t>
         </is>
       </c>
-      <c r="C54" s="16" t="inlineStr">
+      <c r="C54" s="17" t="inlineStr">
         <is>
           <t>DES AXE AERO 150ML APOLLO</t>
         </is>
       </c>
-      <c r="D54" s="17" t="n">
+      <c r="D54" s="18" t="n">
         <v>74.3</v>
       </c>
-      <c r="E54" s="17" t="n">
+      <c r="E54" s="18" t="n">
         <v>459.59</v>
       </c>
-      <c r="F54" s="18" t="n">
+      <c r="F54" s="19" t="n">
         <v>-385.29</v>
       </c>
-      <c r="G54" s="19" t="n">
+      <c r="G54" s="20" t="n">
         <v>-0.838</v>
       </c>
-      <c r="H54" s="20" t="n">
+      <c r="H54" s="21" t="n">
         <v>58984</v>
       </c>
-      <c r="I54" s="21" t="n">
+      <c r="I54" s="22" t="n">
         <v>46.85</v>
       </c>
-      <c r="J54" s="14" t="inlineStr">
+      <c r="J54" s="15" t="inlineStr">
         <is>
           <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
-      <c r="K54" s="17" t="n">
+      <c r="K54" s="18" t="n">
         <v>10.9</v>
       </c>
-      <c r="L54" s="23" t="inlineStr">
+      <c r="L54" s="24" t="inlineStr">
         <is>
           <t>NISSEI</t>
         </is>
       </c>
-      <c r="M54" s="17" t="n">
+      <c r="M54" s="18" t="n">
         <v>8.98</v>
       </c>
-      <c r="N54" s="25" t="n">
+      <c r="N54" s="27" t="n">
         <v>0.214</v>
       </c>
-      <c r="O54" s="23" t="inlineStr">
+      <c r="O54" s="24" t="inlineStr">
         <is>
           <t>São João Mais Cara</t>
         </is>
       </c>
-      <c r="P54" s="23" t="inlineStr">
+      <c r="P54" s="24" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
+      <c r="Q54" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 8.98)</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="32" t="inlineStr">
+      <c r="A55" s="34" t="inlineStr">
         <is>
           <t>TOTAL TOP 50</t>
         </is>
       </c>
-      <c r="B55" s="33" t="n"/>
-      <c r="C55" s="33" t="n"/>
-      <c r="D55" s="34">
+      <c r="B55" s="35" t="n"/>
+      <c r="C55" s="35" t="n"/>
+      <c r="D55" s="36">
         <f>SUM(D5:D54)</f>
         <v/>
       </c>
-      <c r="E55" s="34">
+      <c r="E55" s="36">
         <f>SUM(E5:E54)</f>
         <v/>
       </c>
-      <c r="F55" s="35">
+      <c r="F55" s="37">
         <f>SUM(F5:F54)</f>
         <v/>
       </c>
-      <c r="G55" s="36">
+      <c r="G55" s="38">
         <f>(D55-E55)/E55</f>
         <v/>
       </c>
-      <c r="H55" s="37">
-        <f>SUM(H5:H54)</f>
-        <v/>
-      </c>
-      <c r="I55" s="38" t="inlineStr"/>
-      <c r="J55" s="38" t="inlineStr"/>
-      <c r="K55" s="38" t="inlineStr"/>
-      <c r="L55" s="38" t="inlineStr"/>
-      <c r="M55" s="38" t="inlineStr"/>
-      <c r="N55" s="38" t="inlineStr"/>
-      <c r="O55" s="38" t="inlineStr"/>
-      <c r="P55" s="38" t="inlineStr"/>
+      <c r="H55" s="39" t="n"/>
+      <c r="I55" s="39" t="inlineStr"/>
+      <c r="J55" s="39" t="inlineStr"/>
+      <c r="K55" s="39" t="inlineStr"/>
+      <c r="L55" s="39" t="inlineStr"/>
+      <c r="M55" s="39" t="inlineStr"/>
+      <c r="N55" s="39" t="inlineStr"/>
+      <c r="O55" s="39" t="inlineStr"/>
+      <c r="P55" s="39" t="inlineStr"/>
+      <c r="Q55" s="39" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Fix: timeout de extracao noturna e atualizacao intraday (21:53 - R$ 2.03M)
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -297,13 +297,13 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="167" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -711,7 +711,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: 11/09/2026 19:53:03 (19:53) • Tríade Estoque x Preço x Demanda</t>
+          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: 11/09/2026 21:53:02 (21:53) • Tríade Estoque x Preço x Demanda</t>
         </is>
       </c>
     </row>
@@ -818,16 +818,16 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>101518.51</v>
+        <v>114915.66</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>137384.03</v>
+        <v>157518.16</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>-35865.52</v>
+        <v>-42602.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>-0.261</v>
+        <v>-0.27</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>11112</v>
@@ -885,16 +885,16 @@
         </is>
       </c>
       <c r="D6" s="18" t="n">
-        <v>18250.52</v>
+        <v>22050.48</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>51110.17</v>
+        <v>58600.55</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>-32859.65</v>
+        <v>-36550.07</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>-0.643</v>
+        <v>-0.624</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>56877</v>
@@ -952,16 +952,16 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>71228.28</v>
+        <v>77150.8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>92575.7</v>
+        <v>106143</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-21347.42</v>
+        <v>-28992.2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-0.231</v>
+        <v>-0.273</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>9213</v>
@@ -1019,16 +1019,16 @@
         </is>
       </c>
       <c r="D8" s="18" t="n">
-        <v>18151.2</v>
+        <v>24148.2</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>38280.55</v>
+        <v>43890.7</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>-20129.35</v>
+        <v>-19742.5</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>-0.526</v>
+        <v>-0.45</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>3102</v>
@@ -1086,16 +1086,16 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>6996</v>
+        <v>8745</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>21507.39</v>
+        <v>24659.37</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-14511.39</v>
+        <v>-15914.37</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>-0.675</v>
+        <v>-0.645</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>3675</v>
@@ -1153,16 +1153,16 @@
         </is>
       </c>
       <c r="D10" s="18" t="n">
-        <v>3063.09</v>
+        <v>3289.89</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>15360.7</v>
+        <v>17611.86</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>-12297.61</v>
+        <v>-14321.97</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>-0.8009999999999999</v>
+        <v>-0.8129999999999999</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>12375</v>
@@ -1201,31 +1201,31 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>10053130</t>
+          <t>10052533</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>OZIVY 1MG 1CAN 3ML EMS</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>13777.86</v>
+        <v>2616.61</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>25947.45</v>
+        <v>15379.95</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-12169.59</v>
+        <v>-12763.34</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>-0.469</v>
+        <v>-0.83</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>10373</v>
+        <v>16217</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>8.24</v>
+        <v>12.88</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="Q11" s="14" t="inlineStr">
         <is>
-          <t>Push CRM / Recompra 30d no App</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1258,31 +1258,31 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>10052533</t>
+          <t>10053130</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXG 82UN</t>
+          <t>OZIVY 1MG 1CAN 3ML EMS</t>
         </is>
       </c>
       <c r="D12" s="18" t="n">
-        <v>2384.81</v>
+        <v>17170.29</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>13414.07</v>
+        <v>29750.14</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>-11029.26</v>
+        <v>-12579.85</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-0.8220000000000001</v>
+        <v>-0.423</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>16217</v>
+        <v>10373</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>12.88</v>
+        <v>8.24</v>
       </c>
       <c r="J12" s="15" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="Q12" s="26" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -1327,13 +1327,13 @@
         <v>2144.73</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>8378.370000000001</v>
+        <v>9606.25</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-6233.64</v>
+        <v>-7461.52</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>-0.7440000000000001</v>
+        <v>-0.777</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>13285</v>
@@ -1372,31 +1372,31 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>10041257</t>
+          <t>10052532</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT MAX XXG 80UN</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XXXG 70UN</t>
         </is>
       </c>
       <c r="D14" s="18" t="n">
-        <v>13622.65</v>
+        <v>10761.29</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>18796.87</v>
+        <v>16533.49</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>-5174.22</v>
+        <v>-5772.2</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>-0.275</v>
+        <v>-0.349</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>5905</v>
+        <v>18268</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>4.69</v>
+        <v>14.51</v>
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
@@ -1429,31 +1429,31 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>10052532</t>
+          <t>10053816</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XXXG 70UN</t>
+          <t>SEMAVY 1MG 1CAN 3ML HYPERA PHARMA</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>9623.15</v>
+        <v>929.62</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>14420.16</v>
+        <v>5777.15</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-4797.01</v>
+        <v>-4847.53</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>-0.333</v>
+        <v>-0.8390000000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>18268</v>
+        <v>6648</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>14.51</v>
+        <v>5.28</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1486,31 +1486,31 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>10053816</t>
+          <t>10041257</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>SEMAVY 1MG 1CAN 3ML HYPERA PHARMA</t>
+          <t>FR HUGGIES MAXIMA PROT MAX XXG 80UN</t>
         </is>
       </c>
       <c r="D16" s="18" t="n">
-        <v>929.62</v>
+        <v>16720.74</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>5038.71</v>
+        <v>21551.62</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>-4109.09</v>
+        <v>-4830.88</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>-0.8159999999999999</v>
+        <v>-0.224</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>6648</v>
+        <v>5905</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>5.28</v>
+        <v>4.69</v>
       </c>
       <c r="J16" s="15" t="inlineStr">
         <is>
@@ -1543,44 +1543,54 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>10041258</t>
+          <t>100011507</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT MAX XG 82UN</t>
+          <t>CR DENT ORAL B 70G LV3 PG2 3D WHITE</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>12370.97</v>
+        <v>472.01</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>15952.73</v>
+        <v>4325.99</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-3581.76</v>
+        <v>-3853.98</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>-0.225</v>
+        <v>-0.8909999999999999</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>11779</v>
+        <v>86300</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>9.359999999999999</v>
+        <v>68.55</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K17" s="29" t="inlineStr"/>
-      <c r="L17" s="12" t="inlineStr"/>
-      <c r="M17" s="29" t="inlineStr"/>
-      <c r="N17" s="30" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="N17" s="31" t="n">
+        <v>0.388</v>
+      </c>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P17" s="12" t="inlineStr">
@@ -1588,9 +1598,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q17" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q17" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Panvel R$ 12.90)</t>
         </is>
       </c>
     </row>
@@ -1600,54 +1610,44 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>100011507</t>
+          <t>10041258</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>CR DENT ORAL B 70G LV3 PG2 3D WHITE</t>
+          <t>FR HUGGIES MAXIMA PROT MAX XG 82UN</t>
         </is>
       </c>
       <c r="D18" s="18" t="n">
-        <v>436.21</v>
+        <v>14455.39</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>3773.04</v>
+        <v>18290.66</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>-3336.83</v>
+        <v>-3835.27</v>
       </c>
       <c r="G18" s="20" t="n">
-        <v>-0.884</v>
+        <v>-0.21</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>86300</v>
+        <v>11779</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>68.55</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="J18" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K18" s="18" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="L18" s="23" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M18" s="18" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="N18" s="24" t="n">
-        <v>0.388</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K18" s="27" t="inlineStr"/>
+      <c r="L18" s="23" t="inlineStr"/>
+      <c r="M18" s="27" t="inlineStr"/>
+      <c r="N18" s="28" t="inlineStr"/>
       <c r="O18" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P18" s="23" t="inlineStr">
@@ -1655,9 +1655,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q18" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Panvel R$ 12.90)</t>
+      <c r="Q18" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1667,44 +1667,54 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>10028708</t>
+          <t>10050648</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
+          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>517.9299999999999</v>
+        <v>10915</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>3683.09</v>
+        <v>14710.81</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-3165.16</v>
+        <v>-3795.81</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.8590000000000001</v>
+        <v>-0.258</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>43876</v>
+        <v>9407</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>34.85</v>
+        <v>7.47</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K19" s="29" t="inlineStr"/>
-      <c r="L19" s="12" t="inlineStr"/>
-      <c r="M19" s="29" t="inlineStr"/>
-      <c r="N19" s="30" t="inlineStr"/>
+      <c r="K19" s="7" t="n">
+        <v>988.22</v>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>988.22</v>
+      </c>
+      <c r="N19" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O19" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P19" s="12" t="inlineStr">
@@ -1724,46 +1734,40 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>100007235</t>
+          <t>10028708</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>GENOTROPIN 12MG 36UI 1CANETA PFIZER (C5)</t>
+          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
         </is>
       </c>
       <c r="D20" s="18" t="n">
-        <v>0</v>
+        <v>517.9299999999999</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>3067.86</v>
+        <v>4222.86</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>-3067.86</v>
+        <v>-3704.93</v>
       </c>
       <c r="G20" s="20" t="n">
-        <v>-1</v>
+        <v>-0.877</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>362</v>
-      </c>
-      <c r="I20" s="31" t="n">
-        <v>0.29</v>
+        <v>43876</v>
+      </c>
+      <c r="I20" s="22" t="n">
+        <v>34.85</v>
       </c>
       <c r="J20" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K20" s="27" t="inlineStr"/>
-      <c r="L20" s="23" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M20" s="18" t="n">
-        <v>719.99</v>
-      </c>
+      <c r="L20" s="23" t="inlineStr"/>
+      <c r="M20" s="27" t="inlineStr"/>
       <c r="N20" s="28" t="inlineStr"/>
       <c r="O20" s="23" t="inlineStr">
         <is>
@@ -1777,7 +1781,7 @@
       </c>
       <c r="Q20" s="26" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1787,54 +1791,50 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>10050648</t>
+          <t>100007235</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
+          <t>GENOTROPIN 12MG 36UI 1CANETA PFIZER (C5)</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>10116</v>
+        <v>0</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>12830.46</v>
+        <v>3517.47</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-2714.46</v>
+        <v>-3517.47</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>-0.212</v>
+        <v>-1</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>9407</v>
-      </c>
-      <c r="I21" s="11" t="n">
-        <v>7.47</v>
+        <v>362</v>
+      </c>
+      <c r="I21" s="32" t="n">
+        <v>0.29</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="n">
-        <v>988.22</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K21" s="29" t="inlineStr"/>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M21" s="7" t="n">
-        <v>988.22</v>
-      </c>
-      <c r="N21" s="13" t="n">
-        <v>0</v>
-      </c>
+        <v>719.99</v>
+      </c>
+      <c r="N21" s="30" t="inlineStr"/>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P21" s="12" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="Q21" s="14" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -1854,31 +1854,31 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>10026927</t>
+          <t>10097312</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>NANLAC SUPREME 800G NESTLE</t>
+          <t>NESTOGENO 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>1322.34</v>
+        <v>1189.4</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>3959.77</v>
+        <v>4198.47</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>-2637.43</v>
+        <v>-3009.07</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>-0.6659999999999999</v>
+        <v>-0.7170000000000001</v>
       </c>
       <c r="H22" s="21" t="n">
-        <v>8852</v>
+        <v>12553</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>7.03</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J22" s="15" t="inlineStr">
         <is>
@@ -1886,18 +1886,18 @@
         </is>
       </c>
       <c r="K22" s="18" t="n">
-        <v>108.49</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="L22" s="23" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>DROGARAIA</t>
         </is>
       </c>
       <c r="M22" s="18" t="n">
-        <v>97.69</v>
+        <v>61.06</v>
       </c>
       <c r="N22" s="24" t="n">
-        <v>0.111</v>
+        <v>0.113</v>
       </c>
       <c r="O22" s="23" t="inlineStr">
         <is>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="Q22" s="17" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Precopopular R$ 97.69)</t>
+          <t>Reprecificar no Digital (Drogaraia R$ 61.06)</t>
         </is>
       </c>
     </row>
@@ -1921,31 +1921,31 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>10097312</t>
+          <t>10026927</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>NESTOGENO 2 800G NESTLE</t>
+          <t>NANLAC SUPREME 800G NESTLE</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>1121.41</v>
+        <v>1641.21</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>3661.82</v>
+        <v>4540.09</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-2540.41</v>
+        <v>-2898.88</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>-0.6940000000000001</v>
+        <v>-0.639</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>12553</v>
+        <v>8852</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>9.970000000000001</v>
+        <v>7.03</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -1953,18 +1953,18 @@
         </is>
       </c>
       <c r="K23" s="7" t="n">
-        <v>67.98999999999999</v>
+        <v>108.49</v>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>DROGARAIA</t>
+          <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M23" s="7" t="n">
-        <v>61.06</v>
-      </c>
-      <c r="N23" s="32" t="n">
-        <v>0.113</v>
+        <v>97.69</v>
+      </c>
+      <c r="N23" s="31" t="n">
+        <v>0.111</v>
       </c>
       <c r="O23" s="12" t="inlineStr">
         <is>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Drogaraia R$ 61.06)</t>
+          <t>Reprecificar no Digital (Precopopular R$ 97.69)</t>
         </is>
       </c>
     </row>
@@ -2000,13 +2000,13 @@
         <v>834.16</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>3177.18</v>
+        <v>3642.8</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>-2343.02</v>
+        <v>-2808.64</v>
       </c>
       <c r="G24" s="20" t="n">
-        <v>-0.737</v>
+        <v>-0.7709999999999999</v>
       </c>
       <c r="H24" s="21" t="n">
         <v>26082</v>
@@ -2045,54 +2045,44 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>10097311</t>
+          <t>10052538</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>NESTOGENO 1 800G NESTLE</t>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XXG 74</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>1080.27</v>
+        <v>3263.08</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>3368.38</v>
+        <v>6071.35</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-2288.11</v>
+        <v>-2808.27</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>-0.679</v>
+        <v>-0.463</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>10275</v>
+        <v>4774</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>8.16</v>
+        <v>3.79</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K25" s="7" t="n">
-        <v>67.98999999999999</v>
-      </c>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M25" s="7" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="N25" s="32" t="n">
-        <v>0.081</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K25" s="29" t="inlineStr"/>
+      <c r="L25" s="12" t="inlineStr"/>
+      <c r="M25" s="29" t="inlineStr"/>
+      <c r="N25" s="30" t="inlineStr"/>
       <c r="O25" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P25" s="12" t="inlineStr">
@@ -2100,9 +2090,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q25" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 62.90)</t>
+      <c r="Q25" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2112,44 +2102,54 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>10052536</t>
+          <t>10097311</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX M 108UN</t>
+          <t>NESTOGENO 1 800G NESTLE</t>
         </is>
       </c>
       <c r="D26" s="18" t="n">
-        <v>550.36</v>
+        <v>1080.27</v>
       </c>
       <c r="E26" s="18" t="n">
-        <v>2786.64</v>
+        <v>3862.02</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>-2236.28</v>
+        <v>-2781.75</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>-0.8029999999999999</v>
+        <v>-0.72</v>
       </c>
       <c r="H26" s="21" t="n">
-        <v>6345</v>
+        <v>10275</v>
       </c>
       <c r="I26" s="22" t="n">
-        <v>5.04</v>
+        <v>8.16</v>
       </c>
       <c r="J26" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K26" s="27" t="inlineStr"/>
-      <c r="L26" s="23" t="inlineStr"/>
-      <c r="M26" s="27" t="inlineStr"/>
-      <c r="N26" s="28" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K26" s="18" t="n">
+        <v>67.98999999999999</v>
+      </c>
+      <c r="L26" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M26" s="18" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="N26" s="24" t="n">
+        <v>0.081</v>
+      </c>
       <c r="O26" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P26" s="23" t="inlineStr">
@@ -2157,9 +2157,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q26" s="26" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q26" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 62.90)</t>
         </is>
       </c>
     </row>
@@ -2169,50 +2169,54 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>10025098</t>
+          <t>10040750</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
+          <t>WEGOVY 1MG 3ML NOVO NORDISK</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
+        <v>2996.54</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>5777.15</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>-2780.61</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>-0.481</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>3277</v>
+      </c>
+      <c r="I27" s="11" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>1298.54</v>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>1298.54</v>
+      </c>
+      <c r="N27" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="7" t="n">
-        <v>2187.89</v>
-      </c>
-      <c r="F27" s="8" t="n">
-        <v>-2187.89</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H27" s="10" t="n">
-        <v>192</v>
-      </c>
-      <c r="I27" s="33" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K27" s="29" t="inlineStr"/>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M27" s="7" t="n">
-        <v>1212.9</v>
-      </c>
-      <c r="N27" s="30" t="inlineStr"/>
       <c r="O27" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P27" s="12" t="inlineStr">
@@ -2222,7 +2226,7 @@
       </c>
       <c r="Q27" s="14" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -2244,13 +2248,13 @@
         <v>1725</v>
       </c>
       <c r="E28" s="18" t="n">
-        <v>3866.87</v>
+        <v>4433.58</v>
       </c>
       <c r="F28" s="19" t="n">
-        <v>-2141.87</v>
+        <v>-2708.58</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>-0.5539999999999999</v>
+        <v>-0.611</v>
       </c>
       <c r="H28" s="21" t="n">
         <v>1954</v>
@@ -2299,31 +2303,31 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>10052538</t>
+          <t>10052536</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XXG 74</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX M 108UN</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>3153.81</v>
+        <v>550.36</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>5295.31</v>
+        <v>3195.03</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-2141.5</v>
+        <v>-2644.67</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>-0.404</v>
+        <v>-0.828</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>4774</v>
+        <v>6345</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>3.79</v>
+        <v>5.04</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -2356,40 +2360,46 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>10042967</t>
+          <t>10025098</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC JUMBO G 128UN</t>
+          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
         </is>
       </c>
       <c r="D30" s="18" t="n">
-        <v>13103.08</v>
+        <v>0</v>
       </c>
       <c r="E30" s="18" t="n">
-        <v>15114.29</v>
+        <v>2508.54</v>
       </c>
       <c r="F30" s="19" t="n">
-        <v>-2011.21</v>
+        <v>-2508.54</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>-0.133</v>
+        <v>-1</v>
       </c>
       <c r="H30" s="21" t="n">
-        <v>9721</v>
-      </c>
-      <c r="I30" s="22" t="n">
-        <v>7.72</v>
+        <v>192</v>
+      </c>
+      <c r="I30" s="33" t="n">
+        <v>0.15</v>
       </c>
       <c r="J30" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K30" s="27" t="inlineStr"/>
-      <c r="L30" s="23" t="inlineStr"/>
-      <c r="M30" s="27" t="inlineStr"/>
+      <c r="L30" s="23" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M30" s="18" t="n">
+        <v>1212.9</v>
+      </c>
       <c r="N30" s="28" t="inlineStr"/>
       <c r="O30" s="23" t="inlineStr">
         <is>
@@ -2403,7 +2413,7 @@
       </c>
       <c r="Q30" s="26" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2413,44 +2423,54 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>10046656</t>
+          <t>10033757</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>MOUNJARO 12,5MG 4CAN APLIC LILLY</t>
+          <t>FR HUGGIES MAXIMA PROT HIPER XXG 54UN</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>0</v>
+        <v>1165.53</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>1932.6</v>
+        <v>3320.67</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-1932.6</v>
+        <v>-2155.14</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>-1</v>
+        <v>-0.649</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>511</v>
-      </c>
-      <c r="I31" s="33" t="n">
-        <v>0.41</v>
+        <v>23876</v>
+      </c>
+      <c r="I31" s="11" t="n">
+        <v>18.96</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K31" s="29" t="inlineStr"/>
-      <c r="L31" s="12" t="inlineStr"/>
-      <c r="M31" s="29" t="inlineStr"/>
-      <c r="N31" s="30" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="N31" s="31" t="n">
+        <v>0.165</v>
+      </c>
       <c r="O31" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P31" s="12" t="inlineStr">
@@ -2458,9 +2478,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q31" s="14" t="inlineStr">
-        <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+      <c r="Q31" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 72.90)</t>
         </is>
       </c>
     </row>
@@ -2470,54 +2490,44 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>10033463</t>
+          <t>10004981</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
+          <t>GLYXAMBI 25+5MG 30CP REV BOEHRINGER</t>
         </is>
       </c>
       <c r="D32" s="18" t="n">
-        <v>2892.23</v>
+        <v>1999.2</v>
       </c>
       <c r="E32" s="18" t="n">
-        <v>4697.36</v>
+        <v>4094.73</v>
       </c>
       <c r="F32" s="19" t="n">
-        <v>-1805.13</v>
+        <v>-2095.53</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>-0.384</v>
+        <v>-0.512</v>
       </c>
       <c r="H32" s="21" t="n">
-        <v>11439</v>
+        <v>7514</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>9.09</v>
+        <v>5.97</v>
       </c>
       <c r="J32" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K32" s="18" t="n">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M32" s="18" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="N32" s="24" t="n">
-        <v>0.167</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K32" s="27" t="inlineStr"/>
+      <c r="L32" s="23" t="inlineStr"/>
+      <c r="M32" s="27" t="inlineStr"/>
+      <c r="N32" s="28" t="inlineStr"/>
       <c r="O32" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P32" s="23" t="inlineStr">
@@ -2525,9 +2535,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q32" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 59.90)</t>
+      <c r="Q32" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2537,44 +2547,54 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>10004981</t>
+          <t>10101654</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>GLYXAMBI 25+5MG 30CP REV BOEHRINGER</t>
+          <t>NAN COMFOR 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>1799.28</v>
+        <v>1508.65</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>3571.34</v>
+        <v>3526.27</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-1772.06</v>
+        <v>-2017.62</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>-0.496</v>
+        <v>-0.5720000000000001</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>7514</v>
+        <v>13224</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>5.97</v>
+        <v>10.5</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K33" s="29" t="inlineStr"/>
-      <c r="L33" s="12" t="inlineStr"/>
-      <c r="M33" s="29" t="inlineStr"/>
-      <c r="N33" s="30" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>87.48999999999999</v>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="N33" s="31" t="n">
+        <v>0.094</v>
+      </c>
       <c r="O33" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P33" s="12" t="inlineStr">
@@ -2582,9 +2602,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q33" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q33" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 79.99)</t>
         </is>
       </c>
     </row>
@@ -2594,54 +2614,44 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>10101654</t>
+          <t>10042967</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>NAN COMFOR 2 800G NESTLE</t>
+          <t>FR PAMPERS CONFORTSEC JUMBO G 128UN</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
-        <v>1333.67</v>
+        <v>15319.4</v>
       </c>
       <c r="E34" s="18" t="n">
-        <v>3075.54</v>
+        <v>17329.35</v>
       </c>
       <c r="F34" s="19" t="n">
-        <v>-1741.87</v>
+        <v>-2009.95</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>-0.5660000000000001</v>
+        <v>-0.116</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>13224</v>
+        <v>9721</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>10.5</v>
+        <v>7.72</v>
       </c>
       <c r="J34" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K34" s="18" t="n">
-        <v>87.48999999999999</v>
-      </c>
-      <c r="L34" s="23" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="M34" s="18" t="n">
-        <v>79.98999999999999</v>
-      </c>
-      <c r="N34" s="24" t="n">
-        <v>0.094</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K34" s="27" t="inlineStr"/>
+      <c r="L34" s="23" t="inlineStr"/>
+      <c r="M34" s="27" t="inlineStr"/>
+      <c r="N34" s="28" t="inlineStr"/>
       <c r="O34" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P34" s="23" t="inlineStr">
@@ -2649,9 +2659,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q34" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 79.99)</t>
+      <c r="Q34" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2661,31 +2671,31 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>10034724</t>
+          <t>10028706</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>CONTRAVE 8+90MG 120CP REV LIB PROL MERCK (C1)</t>
+          <t>FR SAO JOAO BABY BAG XG 58UN</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>0</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>1738.08</v>
+        <v>2063.99</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>-1738.08</v>
+        <v>-1990</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>-1</v>
+        <v>-0.9640000000000001</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>2052</v>
+        <v>33174</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>1.63</v>
+        <v>26.35</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
@@ -2693,14 +2703,8 @@
         </is>
       </c>
       <c r="K35" s="29" t="inlineStr"/>
-      <c r="L35" s="12" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M35" s="7" t="n">
-        <v>549.9</v>
-      </c>
+      <c r="L35" s="12" t="inlineStr"/>
+      <c r="M35" s="29" t="inlineStr"/>
       <c r="N35" s="30" t="inlineStr"/>
       <c r="O35" s="12" t="inlineStr">
         <is>
@@ -2724,54 +2728,44 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>10033757</t>
+          <t>100011549</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT HIPER XXG 54UN</t>
+          <t>NAN SUPREME 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
-        <v>1163.03</v>
+        <v>647.45</v>
       </c>
       <c r="E36" s="18" t="n">
-        <v>2896.22</v>
+        <v>2524.56</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>-1733.19</v>
+        <v>-1877.11</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>-0.598</v>
+        <v>-0.7440000000000001</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>23876</v>
+        <v>7332</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>18.96</v>
+        <v>5.82</v>
       </c>
       <c r="J36" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K36" s="18" t="n">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="L36" s="23" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M36" s="18" t="n">
-        <v>72.90000000000001</v>
-      </c>
-      <c r="N36" s="24" t="n">
-        <v>0.165</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K36" s="27" t="inlineStr"/>
+      <c r="L36" s="23" t="inlineStr"/>
+      <c r="M36" s="27" t="inlineStr"/>
+      <c r="N36" s="28" t="inlineStr"/>
       <c r="O36" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P36" s="23" t="inlineStr">
@@ -2779,9 +2773,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q36" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 72.90)</t>
+      <c r="Q36" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2791,44 +2785,54 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>10028706</t>
+          <t>100020215</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XG 58UN</t>
+          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>73.98999999999999</v>
+        <v>259</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>1800.16</v>
+        <v>2121.31</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-1726.17</v>
+        <v>-1862.31</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>-0.9590000000000001</v>
+        <v>-0.878</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>33174</v>
+        <v>23100</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>26.35</v>
+        <v>18.35</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K37" s="29" t="inlineStr"/>
-      <c r="L37" s="12" t="inlineStr"/>
-      <c r="M37" s="29" t="inlineStr"/>
-      <c r="N37" s="30" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="N37" s="31" t="n">
+        <v>0.629</v>
+      </c>
       <c r="O37" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P37" s="12" t="inlineStr">
@@ -2836,9 +2840,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q37" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q37" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 15.90)</t>
         </is>
       </c>
     </row>
@@ -2848,54 +2852,44 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>100020215</t>
+          <t>10046475</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
+          <t>CHOCO MILKA HAZELNUT AO LEITE 90G</t>
         </is>
       </c>
       <c r="D38" s="18" t="n">
-        <v>129.5</v>
+        <v>224.38</v>
       </c>
       <c r="E38" s="18" t="n">
-        <v>1850.16</v>
+        <v>1963.65</v>
       </c>
       <c r="F38" s="19" t="n">
-        <v>-1720.66</v>
+        <v>-1739.27</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>-0.93</v>
+        <v>-0.8859999999999999</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>23100</v>
+        <v>12641</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>18.35</v>
+        <v>10.04</v>
       </c>
       <c r="J38" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K38" s="18" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="L38" s="23" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M38" s="18" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="N38" s="24" t="n">
-        <v>0.629</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K38" s="27" t="inlineStr"/>
+      <c r="L38" s="23" t="inlineStr"/>
+      <c r="M38" s="27" t="inlineStr"/>
+      <c r="N38" s="28" t="inlineStr"/>
       <c r="O38" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P38" s="23" t="inlineStr">
@@ -2903,9 +2897,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q38" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Farmaciasnissei R$ 15.90)</t>
+      <c r="Q38" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2915,44 +2909,54 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>10046475</t>
+          <t>10040738</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>CHOCO MILKA HAZELNUT AO LEITE 90G</t>
+          <t>LYBERDIA 40MG 50ML GOTAS EMS (A3)</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>150.92</v>
+        <v>453.61</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>1712.66</v>
+        <v>2186</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-1561.74</v>
+        <v>-1732.39</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>-0.912</v>
+        <v>-0.792</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>12641</v>
+        <v>2478</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>10.04</v>
+        <v>1.97</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K39" s="29" t="inlineStr"/>
-      <c r="L39" s="12" t="inlineStr"/>
-      <c r="M39" s="29" t="inlineStr"/>
-      <c r="N39" s="30" t="inlineStr"/>
+      <c r="K39" s="7" t="n">
+        <v>567.02</v>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="n">
+        <v>567.02</v>
+      </c>
+      <c r="N39" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O39" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P39" s="12" t="inlineStr">
@@ -2972,54 +2976,44 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>100011547</t>
+          <t>10033461</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>NAN SUPREME 1 800G NESTLE</t>
+          <t>FR BABYSEC ULTRA HIPER G 60UN</t>
         </is>
       </c>
       <c r="D40" s="18" t="n">
-        <v>255.16</v>
+        <v>2068.22</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>1718.09</v>
+        <v>3787.62</v>
       </c>
       <c r="F40" s="19" t="n">
-        <v>-1462.93</v>
+        <v>-1719.4</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>-0.851</v>
+        <v>-0.454</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>7879</v>
+        <v>11727</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>6.26</v>
+        <v>9.31</v>
       </c>
       <c r="J40" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K40" s="18" t="n">
-        <v>132.49</v>
-      </c>
-      <c r="L40" s="23" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="M40" s="18" t="n">
-        <v>124.19</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>0.067</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K40" s="27" t="inlineStr"/>
+      <c r="L40" s="23" t="inlineStr"/>
+      <c r="M40" s="27" t="inlineStr"/>
+      <c r="N40" s="28" t="inlineStr"/>
       <c r="O40" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P40" s="23" t="inlineStr">
@@ -3027,9 +3021,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q40" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 124.19)</t>
+      <c r="Q40" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3039,44 +3033,54 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>10006600</t>
+          <t>10102163</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>LEITE NINHO 800G 1+PREBIO 20% DESC 2ªUN</t>
+          <t>QLAIRA 26CP+2CP REV BIOLAB</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>0</v>
+        <v>2346.08</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>1456.2</v>
+        <v>4010.56</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-1456.2</v>
+        <v>-1664.48</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>-1</v>
+        <v>-0.415</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>11466</v>
+        <v>16459</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>9.109999999999999</v>
+        <v>13.07</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K41" s="29" t="inlineStr"/>
-      <c r="L41" s="12" t="inlineStr"/>
-      <c r="M41" s="29" t="inlineStr"/>
-      <c r="N41" s="30" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>74.22</v>
+      </c>
+      <c r="L41" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="N41" s="31" t="n">
+        <v>0.333</v>
+      </c>
       <c r="O41" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P41" s="12" t="inlineStr">
@@ -3084,9 +3088,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q41" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q41" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 55.67)</t>
         </is>
       </c>
     </row>
@@ -3096,54 +3100,54 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>10040738</t>
+          <t>100010322</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>LYBERDIA 40MG 50ML GOTAS EMS (A3)</t>
+          <t>NESLAC COMFOR 800GR NESTLE</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
-        <v>453.61</v>
+        <v>761.24</v>
       </c>
       <c r="E42" s="18" t="n">
-        <v>1906.58</v>
+        <v>2370.43</v>
       </c>
       <c r="F42" s="19" t="n">
-        <v>-1452.97</v>
+        <v>-1609.19</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>-0.762</v>
+        <v>-0.679</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>2478</v>
+        <v>7668</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>1.97</v>
+        <v>6.09</v>
       </c>
       <c r="J42" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K42" s="18" t="n">
-        <v>567.02</v>
+        <v>72.48999999999999</v>
       </c>
       <c r="L42" s="23" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>AMAZON</t>
         </is>
       </c>
       <c r="M42" s="18" t="n">
-        <v>567.02</v>
-      </c>
-      <c r="N42" s="25" t="n">
-        <v>0</v>
+        <v>54.94</v>
+      </c>
+      <c r="N42" s="24" t="n">
+        <v>0.319</v>
       </c>
       <c r="O42" s="23" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P42" s="23" t="inlineStr">
@@ -3151,9 +3155,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q42" s="26" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q42" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 54.94)</t>
         </is>
       </c>
     </row>
@@ -3163,31 +3167,31 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>100010322</t>
+          <t>10033463</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>NESLAC COMFOR 800GR NESTLE</t>
+          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>635.46</v>
+        <v>3784.58</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>2067.44</v>
+        <v>5385.78</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-1431.98</v>
+        <v>-1601.2</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>-0.6929999999999999</v>
+        <v>-0.297</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>7668</v>
+        <v>11439</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>6.09</v>
+        <v>9.09</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
@@ -3195,18 +3199,18 @@
         </is>
       </c>
       <c r="K43" s="7" t="n">
-        <v>72.48999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="L43" s="12" t="inlineStr">
         <is>
-          <t>AMAZON</t>
+          <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M43" s="7" t="n">
-        <v>54.94</v>
-      </c>
-      <c r="N43" s="32" t="n">
-        <v>0.319</v>
+        <v>59.9</v>
+      </c>
+      <c r="N43" s="31" t="n">
+        <v>0.167</v>
       </c>
       <c r="O43" s="12" t="inlineStr">
         <is>
@@ -3220,7 +3224,7 @@
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Amazon R$ 54.94)</t>
+          <t>Reprecificar no Digital (Precopopular R$ 59.90)</t>
         </is>
       </c>
     </row>
@@ -3230,31 +3234,31 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>10033461</t>
+          <t>10006600</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER G 60UN</t>
+          <t>LEITE NINHO 800G 1+PREBIO 20% DESC 2ªUN</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>1875.3</v>
+        <v>105.99</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>3303.48</v>
+        <v>1669.61</v>
       </c>
       <c r="F44" s="19" t="n">
-        <v>-1428.18</v>
+        <v>-1563.62</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>-0.4320000000000001</v>
+        <v>-0.9370000000000001</v>
       </c>
       <c r="H44" s="21" t="n">
-        <v>11727</v>
+        <v>11466</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>9.31</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
@@ -3287,31 +3291,31 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>10102163</t>
+          <t>100005474</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>QLAIRA 26CP+2CP REV BIOLAB</t>
+          <t>NANLAC COMFOR 3 800G NESTLE</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>2096.93</v>
+        <v>9024.290000000001</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>3497.92</v>
+        <v>10568.65</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-1400.99</v>
+        <v>-1544.36</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>-0.401</v>
+        <v>-0.146</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>16459</v>
+        <v>15223</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>13.07</v>
+        <v>12.09</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
@@ -3319,7 +3323,7 @@
         </is>
       </c>
       <c r="K45" s="7" t="n">
-        <v>74.22</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="L45" s="12" t="inlineStr">
         <is>
@@ -3327,10 +3331,10 @@
         </is>
       </c>
       <c r="M45" s="7" t="n">
-        <v>55.67</v>
-      </c>
-      <c r="N45" s="32" t="n">
-        <v>0.333</v>
+        <v>59.99</v>
+      </c>
+      <c r="N45" s="31" t="n">
+        <v>0.342</v>
       </c>
       <c r="O45" s="12" t="inlineStr">
         <is>
@@ -3344,7 +3348,7 @@
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Precopopular R$ 55.67)</t>
+          <t>Reprecificar no Digital (Precopopular R$ 59.99)</t>
         </is>
       </c>
     </row>
@@ -3354,39 +3358,39 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>100001748</t>
+          <t>10050029</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>ELANI CICLO 3MG+30MCG 3X21CP REV LIBBS</t>
+          <t>HEPARINOX 40MG 0,4ML 10SER CRISTALIA</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
-        <v>1297.1</v>
+        <v>384.82</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>2611.92</v>
+        <v>1919.84</v>
       </c>
       <c r="F46" s="19" t="n">
-        <v>-1314.82</v>
+        <v>-1535.02</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>-0.503</v>
+        <v>-0.8</v>
       </c>
       <c r="H46" s="21" t="n">
-        <v>4495</v>
-      </c>
-      <c r="I46" s="22" t="n">
-        <v>3.57</v>
+        <v>634</v>
+      </c>
+      <c r="I46" s="33" t="n">
+        <v>0.5</v>
       </c>
       <c r="J46" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>⚠️ Duplo Detrator</t>
         </is>
       </c>
       <c r="K46" s="18" t="n">
-        <v>113.72</v>
+        <v>867.88</v>
       </c>
       <c r="L46" s="23" t="inlineStr">
         <is>
@@ -3394,14 +3398,14 @@
         </is>
       </c>
       <c r="M46" s="18" t="n">
-        <v>122.49</v>
-      </c>
-      <c r="N46" s="25" t="n">
-        <v>-0.07200000000000001</v>
+        <v>412.88</v>
+      </c>
+      <c r="N46" s="24" t="n">
+        <v>1.102</v>
       </c>
       <c r="O46" s="23" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P46" s="23" t="inlineStr">
@@ -3409,9 +3413,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q46" s="26" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q46" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar e Remanejar (Drogaraia R$ 412.88)</t>
         </is>
       </c>
     </row>
@@ -3421,39 +3425,39 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>10050029</t>
+          <t>100001748</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>HEPARINOX 40MG 0,4ML 10SER CRISTALIA</t>
+          <t>ELANI CICLO 3MG+30MCG 3X21CP REV LIBBS</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>384.82</v>
+        <v>1516.54</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>1674.44</v>
+        <v>2994.71</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-1289.62</v>
+        <v>-1478.17</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>-0.77</v>
+        <v>-0.494</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>634</v>
-      </c>
-      <c r="I47" s="33" t="n">
-        <v>0.5</v>
+        <v>4495</v>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>3.57</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K47" s="7" t="n">
-        <v>867.88</v>
+        <v>113.72</v>
       </c>
       <c r="L47" s="12" t="inlineStr">
         <is>
@@ -3461,14 +3465,14 @@
         </is>
       </c>
       <c r="M47" s="7" t="n">
-        <v>412.88</v>
-      </c>
-      <c r="N47" s="32" t="n">
-        <v>1.102</v>
+        <v>122.49</v>
+      </c>
+      <c r="N47" s="13" t="n">
+        <v>-0.07200000000000001</v>
       </c>
       <c r="O47" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P47" s="12" t="inlineStr">
@@ -3476,9 +3480,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q47" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar e Remanejar (Drogaraia R$ 412.88)</t>
+      <c r="Q47" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3488,44 +3492,54 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>100011549</t>
+          <t>100011547</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>NAN SUPREME 2 800G NESTLE</t>
+          <t>NAN SUPREME 1 800G NESTLE</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
-        <v>912.4299999999999</v>
+        <v>500.13</v>
       </c>
       <c r="E48" s="18" t="n">
-        <v>2201.87</v>
+        <v>1969.89</v>
       </c>
       <c r="F48" s="19" t="n">
-        <v>-1289.44</v>
+        <v>-1469.76</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>-0.586</v>
+        <v>-0.746</v>
       </c>
       <c r="H48" s="21" t="n">
-        <v>7332</v>
+        <v>7879</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>5.82</v>
+        <v>6.26</v>
       </c>
       <c r="J48" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K48" s="27" t="inlineStr"/>
-      <c r="L48" s="23" t="inlineStr"/>
-      <c r="M48" s="27" t="inlineStr"/>
-      <c r="N48" s="28" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K48" s="18" t="n">
+        <v>132.49</v>
+      </c>
+      <c r="L48" s="23" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M48" s="18" t="n">
+        <v>124.19</v>
+      </c>
+      <c r="N48" s="24" t="n">
+        <v>0.067</v>
+      </c>
       <c r="O48" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P48" s="23" t="inlineStr">
@@ -3533,9 +3547,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q48" s="26" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q48" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 124.19)</t>
         </is>
       </c>
     </row>
@@ -3545,54 +3559,44 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>10007354</t>
+          <t>77912</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>ITRACONAZOL 100MG 15CAP GEN GEOLAB</t>
+          <t>DES REXONA AERO 150ML POWDER</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>679.5599999999999</v>
+        <v>903.91</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>1931.81</v>
+        <v>2355.16</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-1252.25</v>
+        <v>-1451.25</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>-0.648</v>
+        <v>-0.616</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>4930</v>
+        <v>21567</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>3.92</v>
+        <v>17.13</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K49" s="7" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="L49" s="12" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
-        </is>
-      </c>
-      <c r="M49" s="7" t="n">
-        <v>75.98999999999999</v>
-      </c>
-      <c r="N49" s="13" t="n">
-        <v>-0.343</v>
-      </c>
+      <c r="K49" s="29" t="inlineStr"/>
+      <c r="L49" s="12" t="inlineStr"/>
+      <c r="M49" s="29" t="inlineStr"/>
+      <c r="N49" s="30" t="inlineStr"/>
       <c r="O49" s="12" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P49" s="12" t="inlineStr">
@@ -3612,54 +3616,54 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>100005474</t>
+          <t>10007354</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>NANLAC COMFOR 3 800G NESTLE</t>
+          <t>ITRACONAZOL 100MG 15CAP GEN GEOLAB</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
-        <v>7967.13</v>
+        <v>779.36</v>
       </c>
       <c r="E50" s="18" t="n">
-        <v>9217.75</v>
+        <v>2214.93</v>
       </c>
       <c r="F50" s="19" t="n">
-        <v>-1250.62</v>
+        <v>-1435.57</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>-0.136</v>
+        <v>-0.648</v>
       </c>
       <c r="H50" s="21" t="n">
-        <v>15223</v>
+        <v>4930</v>
       </c>
       <c r="I50" s="22" t="n">
-        <v>12.09</v>
+        <v>3.92</v>
       </c>
       <c r="J50" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K50" s="18" t="n">
-        <v>80.48999999999999</v>
+        <v>49.9</v>
       </c>
       <c r="L50" s="23" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>DROGARAIA</t>
         </is>
       </c>
       <c r="M50" s="18" t="n">
-        <v>59.99</v>
-      </c>
-      <c r="N50" s="24" t="n">
-        <v>0.342</v>
+        <v>75.98999999999999</v>
+      </c>
+      <c r="N50" s="25" t="n">
+        <v>-0.343</v>
       </c>
       <c r="O50" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P50" s="23" t="inlineStr">
@@ -3667,9 +3671,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q50" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 59.99)</t>
+      <c r="Q50" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3679,44 +3683,54 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>10045392</t>
+          <t>100015009</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>CHOCO MILKA BUBBLY WHITE 95G</t>
+          <t>SAB DOVE 90G LV+ PG- 6UN ORIGINAL</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>113.94</v>
+        <v>1841.1</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>1353.87</v>
+        <v>3275.98</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-1239.93</v>
+        <v>-1434.88</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>-0.9159999999999999</v>
+        <v>-0.4379999999999999</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>6708</v>
+        <v>60400</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>5.33</v>
+        <v>47.97</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K51" s="29" t="inlineStr"/>
-      <c r="L51" s="12" t="inlineStr"/>
-      <c r="M51" s="29" t="inlineStr"/>
-      <c r="N51" s="30" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="L51" s="12" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="N51" s="31" t="n">
+        <v>0.12</v>
+      </c>
       <c r="O51" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P51" s="12" t="inlineStr">
@@ -3724,9 +3738,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q51" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q51" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Panvel R$ 24.90)</t>
         </is>
       </c>
     </row>
@@ -3736,44 +3750,54 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>10041263</t>
+          <t>100015212</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
+          <t>ANORO 62,5+25MCG 30DOSES GSK</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
-        <v>612.1799999999999</v>
+        <v>342.69</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>1840.05</v>
+        <v>1776.76</v>
       </c>
       <c r="F52" s="19" t="n">
-        <v>-1227.87</v>
+        <v>-1434.07</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>-0.667</v>
+        <v>-0.8070000000000001</v>
       </c>
       <c r="H52" s="21" t="n">
-        <v>3206</v>
+        <v>2013</v>
       </c>
       <c r="I52" s="22" t="n">
-        <v>2.55</v>
+        <v>1.6</v>
       </c>
       <c r="J52" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K52" s="27" t="inlineStr"/>
-      <c r="L52" s="23" t="inlineStr"/>
-      <c r="M52" s="27" t="inlineStr"/>
-      <c r="N52" s="28" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K52" s="18" t="n">
+        <v>423.51</v>
+      </c>
+      <c r="L52" s="23" t="inlineStr">
+        <is>
+          <t>NISSEI</t>
+        </is>
+      </c>
+      <c r="M52" s="18" t="n">
+        <v>360.25</v>
+      </c>
+      <c r="N52" s="24" t="n">
+        <v>0.176</v>
+      </c>
       <c r="O52" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P52" s="23" t="inlineStr">
@@ -3781,9 +3805,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q52" s="26" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q52" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 360.25)</t>
         </is>
       </c>
     </row>
@@ -3793,31 +3817,31 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>77912</t>
+          <t>10045392</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>DES REXONA AERO 150ML POWDER</t>
+          <t>CHOCO MILKA BUBBLY WHITE 95G</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>844.3099999999999</v>
+        <v>151.92</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>2054.12</v>
+        <v>1552.28</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-1209.81</v>
+        <v>-1400.36</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>-0.589</v>
+        <v>-0.902</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>21567</v>
+        <v>6708</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>17.13</v>
+        <v>5.33</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
@@ -3850,54 +3874,44 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>100015212</t>
+          <t>10041263</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>ANORO 62,5+25MCG 30DOSES GSK</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
         </is>
       </c>
       <c r="D54" s="18" t="n">
-        <v>342.69</v>
+        <v>718.08</v>
       </c>
       <c r="E54" s="18" t="n">
-        <v>1549.65</v>
+        <v>2109.72</v>
       </c>
       <c r="F54" s="19" t="n">
-        <v>-1206.96</v>
+        <v>-1391.64</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>-0.779</v>
+        <v>-0.66</v>
       </c>
       <c r="H54" s="21" t="n">
-        <v>2013</v>
+        <v>3206</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>1.6</v>
+        <v>2.55</v>
       </c>
       <c r="J54" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K54" s="18" t="n">
-        <v>423.51</v>
-      </c>
-      <c r="L54" s="23" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M54" s="18" t="n">
-        <v>360.25</v>
-      </c>
-      <c r="N54" s="24" t="n">
-        <v>0.176</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K54" s="27" t="inlineStr"/>
+      <c r="L54" s="23" t="inlineStr"/>
+      <c r="M54" s="27" t="inlineStr"/>
+      <c r="N54" s="28" t="inlineStr"/>
       <c r="O54" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P54" s="23" t="inlineStr">
@@ -3905,9 +3919,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q54" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Farmaciasnissei R$ 360.25)</t>
+      <c r="Q54" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adicionar aba Visão Regional & Lojas, ranking de perda por concorrente Precifica e alertas executivos
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -267,7 +267,7 @@
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -282,9 +282,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -294,7 +291,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -303,7 +300,10 @@
     <xf numFmtId="167" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -711,7 +711,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: - (15:53) • Tríade Estoque x Preço x Demanda</t>
+          <t>Canais Digitais (App, Site, Marketplace) • Horário de Corte: - (16:53) • Tríade Estoque x Preço x Demanda</t>
         </is>
       </c>
     </row>
@@ -818,16 +818,16 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>10373.64</v>
+        <v>11284.33</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>32484.14</v>
+        <v>36207.57</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>-22110.5</v>
+        <v>-24923.24</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>-0.6809999999999999</v>
+        <v>-0.6879999999999999</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>58027</v>
@@ -876,35 +876,35 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>10053130</t>
+          <t>10046657</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>OZIVY 1MG 1CAN 3ML EMS</t>
+          <t>MOUNJARO 15MG 4CAN APLIC LILLY</t>
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>2788.86</v>
+        <v>0</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>13715.17</v>
+        <v>11035.72</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>-10926.31</v>
+        <v>-11035.72</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>-0.797</v>
+        <v>-1</v>
       </c>
       <c r="H6" s="20" t="n">
-        <v>10648</v>
+        <v>1174</v>
       </c>
       <c r="I6" s="21" t="n">
-        <v>8.460000000000001</v>
+        <v>0.93</v>
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K6" s="22" t="inlineStr"/>
@@ -923,7 +923,7 @@
       </c>
       <c r="Q6" s="25" t="inlineStr">
         <is>
-          <t>Push CRM / Recompra 30d no App</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -933,41 +933,41 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>10046657</t>
+          <t>10053130</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>MOUNJARO 15MG 4CAN APLIC LILLY</t>
+          <t>OZIVY 1MG 1CAN 3ML EMS</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0</v>
+        <v>4786.86</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>9900.860000000001</v>
+        <v>15287.25</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-9900.860000000001</v>
+        <v>-10500.39</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-1</v>
+        <v>-0.6870000000000001</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1174</v>
-      </c>
-      <c r="I7" s="26" t="n">
-        <v>0.93</v>
+        <v>10648</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>8.460000000000001</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K7" s="27" t="inlineStr"/>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K7" s="26" t="inlineStr"/>
       <c r="L7" s="12" t="inlineStr"/>
-      <c r="M7" s="27" t="inlineStr"/>
-      <c r="N7" s="28" t="inlineStr"/>
+      <c r="M7" s="26" t="inlineStr"/>
+      <c r="N7" s="27" t="inlineStr"/>
       <c r="O7" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -978,9 +978,9 @@
           <t>Detrator Crítico</t>
         </is>
       </c>
-      <c r="Q7" s="29" t="inlineStr">
-        <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+      <c r="Q7" s="28" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -1002,18 +1002,18 @@
         <v>1246.38</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>8124.43</v>
+        <v>9055.67</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>-6878.05</v>
+        <v>-7809.29</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>-0.847</v>
+        <v>-0.862</v>
       </c>
       <c r="H8" s="20" t="n">
         <v>16204</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="29" t="n">
         <v>12.87</v>
       </c>
       <c r="J8" s="14" t="inlineStr">
@@ -1047,44 +1047,54 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>10052534</t>
+          <t>10046655</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
+          <t>MOUNJARO 10MG 4CAN APLIC LILLY</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>1481.47</v>
+        <v>3998</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7069.57</v>
+        <v>10652.19</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-5588.1</v>
+        <v>-6654.19</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>-0.79</v>
+        <v>-0.625</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>9137</v>
+        <v>3130</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>7.26</v>
+        <v>2.49</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K9" s="27" t="inlineStr"/>
-      <c r="L9" s="12" t="inlineStr"/>
-      <c r="M9" s="27" t="inlineStr"/>
-      <c r="N9" s="28" t="inlineStr"/>
+      <c r="K9" s="7" t="n">
+        <v>3210.85</v>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>3210.85</v>
+      </c>
+      <c r="N9" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="O9" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P9" s="12" t="inlineStr">
@@ -1092,9 +1102,9 @@
           <t>Detrator Crítico</t>
         </is>
       </c>
-      <c r="Q9" s="29" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q9" s="28" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -1104,54 +1114,44 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>10046655</t>
+          <t>10052534</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>MOUNJARO 10MG 4CAN APLIC LILLY</t>
+          <t>FR PAMPERS CONFORTSEC BAG MAX XG 86UN</t>
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>3998</v>
+        <v>1703.38</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>9556.76</v>
+        <v>7879.9</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>-5558.76</v>
+        <v>-6176.52</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>-0.5820000000000001</v>
+        <v>-0.784</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>3130</v>
-      </c>
-      <c r="I10" s="21" t="n">
-        <v>2.49</v>
+        <v>9137</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>7.26</v>
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K10" s="17" t="n">
-        <v>3210.85</v>
-      </c>
-      <c r="L10" s="23" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M10" s="17" t="n">
-        <v>3210.85</v>
-      </c>
-      <c r="N10" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="K10" s="22" t="inlineStr"/>
+      <c r="L10" s="23" t="inlineStr"/>
+      <c r="M10" s="22" t="inlineStr"/>
+      <c r="N10" s="24" t="inlineStr"/>
       <c r="O10" s="23" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P10" s="23" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="Q10" s="25" t="inlineStr">
         <is>
-          <t>Push CRM / Recompra 30d no App</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1180,16 +1180,16 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>5357.66</v>
+        <v>5705.36</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>9271.309999999999</v>
+        <v>10334.01</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-3913.65</v>
+        <v>-4628.65</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>-0.422</v>
+        <v>-0.448</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>17809</v>
@@ -1202,10 +1202,10 @@
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K11" s="27" t="inlineStr"/>
+      <c r="K11" s="26" t="inlineStr"/>
       <c r="L11" s="12" t="inlineStr"/>
-      <c r="M11" s="27" t="inlineStr"/>
-      <c r="N11" s="28" t="inlineStr"/>
+      <c r="M11" s="26" t="inlineStr"/>
+      <c r="N11" s="27" t="inlineStr"/>
       <c r="O11" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1216,7 +1216,7 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q11" s="29" t="inlineStr">
+      <c r="Q11" s="28" t="inlineStr">
         <is>
           <t>Ação Promocional / Destaque Home</t>
         </is>
@@ -1237,21 +1237,21 @@
         </is>
       </c>
       <c r="D12" s="17" t="n">
-        <v>1022.69</v>
+        <v>1138.59</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>4013.95</v>
+        <v>4474.05</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>-2991.26</v>
+        <v>-3335.46</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>-0.745</v>
+        <v>-0.746</v>
       </c>
       <c r="H12" s="20" t="n">
         <v>13911</v>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="29" t="n">
         <v>11.05</v>
       </c>
       <c r="J12" s="14" t="inlineStr">
@@ -1285,54 +1285,44 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>10046654</t>
+          <t>10041258</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>MOUNJARO 7,5MG 4CAN APLIC LILLY</t>
+          <t>FR HUGGIES MAXIMA PROT MAX XG 82UN</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>12134.2</v>
+        <v>9392.219999999999</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>14936.31</v>
+        <v>12212.63</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-2802.11</v>
+        <v>-2820.41</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>-0.188</v>
+        <v>-0.231</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>4321</v>
+        <v>11643</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>3.43</v>
+        <v>9.25</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K13" s="7" t="n">
-        <v>2766.26</v>
-      </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>2766.26</v>
-      </c>
-      <c r="N13" s="31" t="n">
-        <v>0</v>
-      </c>
+      <c r="K13" s="26" t="inlineStr"/>
+      <c r="L13" s="12" t="inlineStr"/>
+      <c r="M13" s="26" t="inlineStr"/>
+      <c r="N13" s="27" t="inlineStr"/>
       <c r="O13" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P13" s="12" t="inlineStr">
@@ -1340,9 +1330,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q13" s="29" t="inlineStr">
-        <is>
-          <t>Push CRM / Recompra 30d no App</t>
+      <c r="Q13" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1352,44 +1342,54 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>10041258</t>
+          <t>100005474</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT MAX XG 82UN</t>
+          <t>NANLAC COMFOR 3 800G NESTLE</t>
         </is>
       </c>
       <c r="D14" s="17" t="n">
-        <v>8565.030000000001</v>
+        <v>4268.64</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>10956.74</v>
+        <v>6349.31</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>-2391.71</v>
+        <v>-2080.67</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>-0.218</v>
+        <v>-0.328</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>11643</v>
-      </c>
-      <c r="I14" s="21" t="n">
-        <v>9.25</v>
+        <v>17876</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>14.2</v>
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K14" s="22" t="inlineStr"/>
-      <c r="L14" s="23" t="inlineStr"/>
-      <c r="M14" s="22" t="inlineStr"/>
-      <c r="N14" s="24" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K14" s="17" t="n">
+        <v>80.48999999999999</v>
+      </c>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="N14" s="31" t="n">
+        <v>0.342</v>
+      </c>
       <c r="O14" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P14" s="23" t="inlineStr">
@@ -1397,9 +1397,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q14" s="25" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q14" s="16" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 59.99)</t>
         </is>
       </c>
     </row>
@@ -1409,54 +1409,54 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>10050654</t>
+          <t>10101654</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>POVIZTRA 2,4MG 3ML EUROFARMA</t>
+          <t>NAN COMFOR 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>3507</v>
+        <v>666.11</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>5669.25</v>
+        <v>2625.37</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-2162.25</v>
+        <v>-1959.26</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>-0.381</v>
+        <v>-0.746</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>4049</v>
+        <v>13256</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>3.22</v>
+        <v>10.53</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K15" s="7" t="n">
-        <v>1617.66</v>
+        <v>87.48999999999999</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>AMAZON</t>
         </is>
       </c>
       <c r="M15" s="7" t="n">
-        <v>1617.66</v>
-      </c>
-      <c r="N15" s="31" t="n">
-        <v>0</v>
+        <v>79.98999999999999</v>
+      </c>
+      <c r="N15" s="13" t="n">
+        <v>0.094</v>
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P15" s="12" t="inlineStr">
@@ -1464,9 +1464,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q15" s="29" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q15" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 79.99)</t>
         </is>
       </c>
     </row>
@@ -1476,54 +1476,44 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>100005474</t>
+          <t>10028708</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>NANLAC COMFOR 3 800G NESTLE</t>
+          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
         </is>
       </c>
       <c r="D16" s="17" t="n">
-        <v>3578.56</v>
+        <v>502.14</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>5696.37</v>
+        <v>2407.39</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>-2117.81</v>
+        <v>-1905.25</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>-0.3720000000000001</v>
+        <v>-0.7909999999999999</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>17876</v>
-      </c>
-      <c r="I16" s="21" t="n">
-        <v>14.2</v>
+        <v>43780</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>34.77</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K16" s="17" t="n">
-        <v>80.48999999999999</v>
-      </c>
-      <c r="L16" s="23" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>59.99</v>
-      </c>
-      <c r="N16" s="32" t="n">
-        <v>0.342</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K16" s="22" t="inlineStr"/>
+      <c r="L16" s="23" t="inlineStr"/>
+      <c r="M16" s="22" t="inlineStr"/>
+      <c r="N16" s="24" t="inlineStr"/>
       <c r="O16" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P16" s="23" t="inlineStr">
@@ -1531,9 +1521,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q16" s="16" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 59.99)</t>
+      <c r="Q16" s="25" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1543,41 +1533,41 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>10004419</t>
+          <t>10041257</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>OZEMPIC 1MG 4AGULHAS NOVOFINE 4MM NOVO NORDISK</t>
+          <t>FR HUGGIES MAXIMA PROT MAX XXG 80UN</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>0</v>
+        <v>10390.45</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>2116.09</v>
+        <v>12177.1</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-2116.09</v>
+        <v>-1786.65</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>-1</v>
+        <v>-0.147</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>2468</v>
+        <v>7889</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>1.96</v>
+        <v>6.27</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K17" s="27" t="inlineStr"/>
+      <c r="K17" s="26" t="inlineStr"/>
       <c r="L17" s="12" t="inlineStr"/>
-      <c r="M17" s="27" t="inlineStr"/>
-      <c r="N17" s="28" t="inlineStr"/>
+      <c r="M17" s="26" t="inlineStr"/>
+      <c r="N17" s="27" t="inlineStr"/>
       <c r="O17" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1588,9 +1578,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q17" s="29" t="inlineStr">
-        <is>
-          <t>Push CRM / Recompra 30d no App</t>
+      <c r="Q17" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1600,31 +1590,31 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>10028708</t>
+          <t>10028706</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XXG 56UN</t>
+          <t>FR SAO JOAO BABY BAG XG 58UN</t>
         </is>
       </c>
       <c r="D18" s="17" t="n">
-        <v>428.15</v>
+        <v>221.97</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>2159.82</v>
+        <v>1941.2</v>
       </c>
       <c r="F18" s="18" t="n">
-        <v>-1731.67</v>
+        <v>-1719.23</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>-0.802</v>
+        <v>-0.8859999999999999</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>43780</v>
-      </c>
-      <c r="I18" s="21" t="n">
-        <v>34.77</v>
+        <v>33174</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>26.35</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
@@ -1657,41 +1647,41 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>10041257</t>
+          <t>100001402</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT MAX XXG 80UN</t>
+          <t>SERVICO DOMICILIO</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>9225.549999999999</v>
+        <v>7989.51</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>10924.86</v>
+        <v>9702.299999999999</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-1699.31</v>
+        <v>-1712.79</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.156</v>
+        <v>-0.177</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>7889</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>6.27</v>
+        <v>0</v>
+      </c>
+      <c r="I19" s="32" t="n">
+        <v>0</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K19" s="27" t="inlineStr"/>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K19" s="26" t="inlineStr"/>
       <c r="L19" s="12" t="inlineStr"/>
-      <c r="M19" s="27" t="inlineStr"/>
-      <c r="N19" s="28" t="inlineStr"/>
+      <c r="M19" s="26" t="inlineStr"/>
+      <c r="N19" s="27" t="inlineStr"/>
       <c r="O19" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -1702,9 +1692,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q19" s="29" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q19" s="28" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -1714,31 +1704,31 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>10101654</t>
+          <t>100011507</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>NAN COMFOR 2 800G NESTLE</t>
+          <t>CR DENT ORAL B 70G LV3 PG2 3D WHITE</t>
         </is>
       </c>
       <c r="D20" s="17" t="n">
-        <v>666.11</v>
+        <v>213.42</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>2355.39</v>
+        <v>1897.2</v>
       </c>
       <c r="F20" s="18" t="n">
-        <v>-1689.28</v>
+        <v>-1683.78</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>-0.7170000000000001</v>
+        <v>-0.888</v>
       </c>
       <c r="H20" s="20" t="n">
-        <v>13256</v>
-      </c>
-      <c r="I20" s="21" t="n">
-        <v>10.53</v>
+        <v>86250</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>68.51000000000001</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
@@ -1746,18 +1736,18 @@
         </is>
       </c>
       <c r="K20" s="17" t="n">
-        <v>87.48999999999999</v>
+        <v>17.9</v>
       </c>
       <c r="L20" s="23" t="inlineStr">
         <is>
-          <t>AMAZON</t>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M20" s="17" t="n">
-        <v>79.98999999999999</v>
-      </c>
-      <c r="N20" s="32" t="n">
-        <v>0.094</v>
+        <v>12.9</v>
+      </c>
+      <c r="N20" s="31" t="n">
+        <v>0.388</v>
       </c>
       <c r="O20" s="23" t="inlineStr">
         <is>
@@ -1771,7 +1761,7 @@
       </c>
       <c r="Q20" s="16" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Amazon R$ 79.99)</t>
+          <t>Reprecificar no Digital (Panvel R$ 12.90)</t>
         </is>
       </c>
     </row>
@@ -1781,44 +1771,54 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>100001402</t>
+          <t>10030120</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>SERVICO DOMICILIO</t>
+          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>7122.64</v>
+        <v>0</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>8704.559999999999</v>
+        <v>1467.77</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-1581.92</v>
+        <v>-1467.77</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>-0.182</v>
+        <v>-1</v>
       </c>
       <c r="H21" s="10" t="n">
+        <v>1930</v>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="N21" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K21" s="27" t="inlineStr"/>
-      <c r="L21" s="12" t="inlineStr"/>
-      <c r="M21" s="27" t="inlineStr"/>
-      <c r="N21" s="28" t="inlineStr"/>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P21" s="12" t="inlineStr">
@@ -1826,9 +1826,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q21" s="29" t="inlineStr">
-        <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+      <c r="Q21" s="28" t="inlineStr">
+        <is>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -1838,44 +1838,54 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>10028706</t>
+          <t>10050654</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG XG 58UN</t>
+          <t>POVIZTRA 2,4MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D22" s="17" t="n">
-        <v>221.97</v>
+        <v>4951</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>1741.57</v>
+        <v>6319.07</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>-1519.6</v>
+        <v>-1368.07</v>
       </c>
       <c r="G22" s="19" t="n">
-        <v>-0.873</v>
+        <v>-0.216</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>33174</v>
-      </c>
-      <c r="I22" s="21" t="n">
-        <v>26.35</v>
+        <v>4049</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>3.22</v>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K22" s="22" t="inlineStr"/>
-      <c r="L22" s="23" t="inlineStr"/>
-      <c r="M22" s="22" t="inlineStr"/>
-      <c r="N22" s="24" t="inlineStr"/>
+      <c r="K22" s="17" t="n">
+        <v>1617.66</v>
+      </c>
+      <c r="L22" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>1617.66</v>
+      </c>
+      <c r="N22" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="O22" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P22" s="23" t="inlineStr">
@@ -1895,54 +1905,54 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>100011507</t>
+          <t>10026836</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>CR DENT ORAL B 70G LV3 PG2 3D WHITE</t>
+          <t>IUMI ES 3MG+20MCG 120CP REV LIBBS</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>213.42</v>
+        <v>2075.77</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>1702.1</v>
+        <v>3437.99</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-1488.68</v>
+        <v>-1362.22</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>-0.875</v>
+        <v>-0.396</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>86250</v>
+        <v>3355</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>68.51000000000001</v>
+        <v>2.66</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K23" s="7" t="n">
-        <v>17.9</v>
+        <v>153.23</v>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>DROGARAIA</t>
         </is>
       </c>
       <c r="M23" s="7" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="N23" s="13" t="n">
-        <v>0.388</v>
+        <v>173.71</v>
+      </c>
+      <c r="N23" s="30" t="n">
+        <v>-0.118</v>
       </c>
       <c r="O23" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P23" s="12" t="inlineStr">
@@ -1950,9 +1960,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q23" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Panvel R$ 12.90)</t>
+      <c r="Q23" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1962,39 +1972,39 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>10026836</t>
+          <t>100014678</t>
         </is>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>IUMI ES 3MG+20MCG 120CP REV LIBBS</t>
+          <t>TADALAFILA 5MG 30CP REV GEN EMS</t>
         </is>
       </c>
       <c r="D24" s="17" t="n">
-        <v>1626.08</v>
+        <v>2364.03</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>3084.44</v>
+        <v>3647.51</v>
       </c>
       <c r="F24" s="18" t="n">
-        <v>-1458.36</v>
+        <v>-1283.48</v>
       </c>
       <c r="G24" s="19" t="n">
-        <v>-0.473</v>
+        <v>-0.352</v>
       </c>
       <c r="H24" s="20" t="n">
-        <v>3355</v>
-      </c>
-      <c r="I24" s="21" t="n">
-        <v>2.66</v>
+        <v>54758</v>
+      </c>
+      <c r="I24" s="29" t="n">
+        <v>43.49</v>
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K24" s="17" t="n">
-        <v>153.23</v>
+        <v>18.09</v>
       </c>
       <c r="L24" s="23" t="inlineStr">
         <is>
@@ -2002,14 +2012,14 @@
         </is>
       </c>
       <c r="M24" s="17" t="n">
-        <v>173.71</v>
-      </c>
-      <c r="N24" s="30" t="n">
-        <v>-0.118</v>
+        <v>14.68</v>
+      </c>
+      <c r="N24" s="31" t="n">
+        <v>0.232</v>
       </c>
       <c r="O24" s="23" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P24" s="23" t="inlineStr">
@@ -2017,9 +2027,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q24" s="25" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q24" s="16" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Drogaraia R$ 14.68)</t>
         </is>
       </c>
     </row>
@@ -2029,54 +2039,54 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>10030120</t>
+          <t>100020215</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
+          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>0</v>
+        <v>306.82</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>1316.83</v>
+        <v>1579.27</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-1316.83</v>
+        <v>-1272.45</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>-1</v>
+        <v>-0.8059999999999999</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>1930</v>
+        <v>23281</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>1.53</v>
+        <v>18.49</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K25" s="7" t="n">
-        <v>1301.17</v>
+        <v>25.9</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M25" s="7" t="n">
-        <v>1301.17</v>
-      </c>
-      <c r="N25" s="31" t="n">
-        <v>0</v>
+        <v>15.9</v>
+      </c>
+      <c r="N25" s="13" t="n">
+        <v>0.629</v>
       </c>
       <c r="O25" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P25" s="12" t="inlineStr">
@@ -2084,9 +2094,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q25" s="29" t="inlineStr">
-        <is>
-          <t>Push CRM / Recompra 30d no App</t>
+      <c r="Q25" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 15.90)</t>
         </is>
       </c>
     </row>
@@ -2096,54 +2106,44 @@
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>100014678</t>
+          <t>10033758</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>TADALAFILA 5MG 30CP REV GEN EMS</t>
+          <t>FR HUGGIES MAXIMA PROT HIPER XG 56UN</t>
         </is>
       </c>
       <c r="D26" s="17" t="n">
-        <v>2038.41</v>
+        <v>676.7</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>3272.41</v>
+        <v>1903.3</v>
       </c>
       <c r="F26" s="18" t="n">
-        <v>-1234</v>
+        <v>-1226.6</v>
       </c>
       <c r="G26" s="19" t="n">
-        <v>-0.377</v>
+        <v>-0.644</v>
       </c>
       <c r="H26" s="20" t="n">
-        <v>54758</v>
-      </c>
-      <c r="I26" s="21" t="n">
-        <v>43.49</v>
+        <v>26408</v>
+      </c>
+      <c r="I26" s="29" t="n">
+        <v>20.98</v>
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="n">
-        <v>18.09</v>
-      </c>
-      <c r="L26" s="23" t="inlineStr">
-        <is>
-          <t>DROGARAIA</t>
-        </is>
-      </c>
-      <c r="M26" s="17" t="n">
-        <v>14.68</v>
-      </c>
-      <c r="N26" s="32" t="n">
-        <v>0.232</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K26" s="22" t="inlineStr"/>
+      <c r="L26" s="23" t="inlineStr"/>
+      <c r="M26" s="22" t="inlineStr"/>
+      <c r="N26" s="24" t="inlineStr"/>
       <c r="O26" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P26" s="23" t="inlineStr">
@@ -2151,9 +2151,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q26" s="16" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Drogaraia R$ 14.68)</t>
+      <c r="Q26" s="25" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2163,54 +2163,44 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>10050640</t>
+          <t>10033461</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>POVIZTRA 0,25MG 1,5ML EUROFARMA</t>
+          <t>FR BABYSEC ULTRA HIPER G 60UN</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>885</v>
+        <v>1509.4</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>2026.78</v>
+        <v>2705.01</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>-1141.78</v>
+        <v>-1195.61</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.442</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>6229</v>
+        <v>11699</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>4.95</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K27" s="7" t="n">
-        <v>831.76</v>
-      </c>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M27" s="7" t="n">
-        <v>831.76</v>
-      </c>
-      <c r="N27" s="31" t="n">
-        <v>0</v>
-      </c>
+      <c r="K27" s="26" t="inlineStr"/>
+      <c r="L27" s="12" t="inlineStr"/>
+      <c r="M27" s="26" t="inlineStr"/>
+      <c r="N27" s="27" t="inlineStr"/>
       <c r="O27" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P27" s="12" t="inlineStr">
@@ -2218,7 +2208,7 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q27" s="29" t="inlineStr">
+      <c r="Q27" s="28" t="inlineStr">
         <is>
           <t>Ação Promocional / Destaque Home</t>
         </is>
@@ -2230,31 +2220,31 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>100020215</t>
+          <t>10097312</t>
         </is>
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>DES DOVE AERO 150ML REGULAR ORIGINAL</t>
+          <t>NESTOGENO 2 800G NESTLE</t>
         </is>
       </c>
       <c r="D28" s="17" t="n">
-        <v>280.92</v>
+        <v>995.11</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>1416.87</v>
+        <v>2178.03</v>
       </c>
       <c r="F28" s="18" t="n">
-        <v>-1135.95</v>
+        <v>-1182.92</v>
       </c>
       <c r="G28" s="19" t="n">
-        <v>-0.802</v>
+        <v>-0.5429999999999999</v>
       </c>
       <c r="H28" s="20" t="n">
-        <v>23281</v>
-      </c>
-      <c r="I28" s="21" t="n">
-        <v>18.49</v>
+        <v>12677</v>
+      </c>
+      <c r="I28" s="29" t="n">
+        <v>10.07</v>
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
@@ -2262,18 +2252,18 @@
         </is>
       </c>
       <c r="K28" s="17" t="n">
-        <v>25.9</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="L28" s="23" t="inlineStr">
         <is>
-          <t>NISSEI</t>
+          <t>DROGARAIA</t>
         </is>
       </c>
       <c r="M28" s="17" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="N28" s="32" t="n">
-        <v>0.629</v>
+        <v>61.06</v>
+      </c>
+      <c r="N28" s="31" t="n">
+        <v>0.113</v>
       </c>
       <c r="O28" s="23" t="inlineStr">
         <is>
@@ -2287,7 +2277,7 @@
       </c>
       <c r="Q28" s="16" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Farmaciasnissei R$ 15.90)</t>
+          <t>Reprecificar no Digital (Drogaraia R$ 61.06)</t>
         </is>
       </c>
     </row>
@@ -2297,44 +2287,54 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>10033758</t>
+          <t>10023627</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES MAXIMA PROT HIPER XG 56UN</t>
+          <t>APTANUTRI PROFUTURA 3 800G DANONE</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>591.8</v>
+        <v>958.8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>1707.57</v>
+        <v>2067.83</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-1115.77</v>
+        <v>-1109.03</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>-0.653</v>
+        <v>-0.536</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>26408</v>
+        <v>8301</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>20.98</v>
+        <v>6.59</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K29" s="27" t="inlineStr"/>
-      <c r="L29" s="12" t="inlineStr"/>
-      <c r="M29" s="27" t="inlineStr"/>
-      <c r="N29" s="28" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="n">
+        <v>106.99</v>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="n">
+        <v>79.79000000000001</v>
+      </c>
+      <c r="N29" s="13" t="n">
+        <v>0.341</v>
+      </c>
       <c r="O29" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P29" s="12" t="inlineStr">
@@ -2342,9 +2342,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q29" s="29" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q29" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 79.79)</t>
         </is>
       </c>
     </row>
@@ -2354,44 +2354,54 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>10033461</t>
+          <t>100014681</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER G 60UN</t>
+          <t>TADALAFILA 20MG 4CP REV GEN EMS</t>
         </is>
       </c>
       <c r="D30" s="17" t="n">
-        <v>1369.6</v>
+        <v>1284.48</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>2426.84</v>
+        <v>2387.23</v>
       </c>
       <c r="F30" s="18" t="n">
-        <v>-1057.24</v>
+        <v>-1102.75</v>
       </c>
       <c r="G30" s="19" t="n">
-        <v>-0.436</v>
+        <v>-0.462</v>
       </c>
       <c r="H30" s="20" t="n">
-        <v>11699</v>
-      </c>
-      <c r="I30" s="21" t="n">
-        <v>9.289999999999999</v>
+        <v>25510</v>
+      </c>
+      <c r="I30" s="29" t="n">
+        <v>20.26</v>
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K30" s="22" t="inlineStr"/>
-      <c r="L30" s="23" t="inlineStr"/>
-      <c r="M30" s="22" t="inlineStr"/>
-      <c r="N30" s="24" t="inlineStr"/>
+      <c r="K30" s="17" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="L30" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M30" s="17" t="n">
+        <v>13.57</v>
+      </c>
+      <c r="N30" s="33" t="n">
+        <v>-0.139</v>
+      </c>
       <c r="O30" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P30" s="23" t="inlineStr">
@@ -2411,54 +2421,44 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>10023627</t>
+          <t>10028705</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>APTANUTRI PROFUTURA 3 800G DANONE</t>
+          <t>FR SAO JOAO BABY BAG G 60UN</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>807.8200000000001</v>
+        <v>0</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>1855.19</v>
+        <v>1080.96</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-1047.37</v>
+        <v>-1080.96</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>-0.5649999999999999</v>
+        <v>-1</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>8301</v>
+        <v>28997</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>6.59</v>
+        <v>23.03</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="n">
-        <v>106.99</v>
-      </c>
-      <c r="L31" s="12" t="inlineStr">
-        <is>
-          <t>AMAZON</t>
-        </is>
-      </c>
-      <c r="M31" s="7" t="n">
-        <v>79.79000000000001</v>
-      </c>
-      <c r="N31" s="13" t="n">
-        <v>0.341</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K31" s="26" t="inlineStr"/>
+      <c r="L31" s="12" t="inlineStr"/>
+      <c r="M31" s="26" t="inlineStr"/>
+      <c r="N31" s="27" t="inlineStr"/>
       <c r="O31" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P31" s="12" t="inlineStr">
@@ -2466,9 +2466,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q31" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 79.79)</t>
+      <c r="Q31" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2478,54 +2478,54 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>100010706</t>
+          <t>10050640</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>IUMI 3MG+20MCG 72CP REV LIBBS</t>
+          <t>POVIZTRA 0,25MG 1,5ML EUROFARMA</t>
         </is>
       </c>
       <c r="D32" s="17" t="n">
-        <v>909.35</v>
+        <v>1180</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>1929.16</v>
+        <v>2259.09</v>
       </c>
       <c r="F32" s="18" t="n">
-        <v>-1019.81</v>
+        <v>-1079.09</v>
       </c>
       <c r="G32" s="19" t="n">
-        <v>-0.529</v>
+        <v>-0.478</v>
       </c>
       <c r="H32" s="20" t="n">
-        <v>5921</v>
-      </c>
-      <c r="I32" s="21" t="n">
-        <v>4.7</v>
+        <v>6229</v>
+      </c>
+      <c r="I32" s="29" t="n">
+        <v>4.95</v>
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K32" s="17" t="n">
-        <v>120.64</v>
+        <v>831.76</v>
       </c>
       <c r="L32" s="23" t="inlineStr">
         <is>
-          <t>NISSEI</t>
+          <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M32" s="17" t="n">
-        <v>114.9</v>
-      </c>
-      <c r="N32" s="32" t="n">
-        <v>0.05</v>
+        <v>831.76</v>
+      </c>
+      <c r="N32" s="33" t="n">
+        <v>0</v>
       </c>
       <c r="O32" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P32" s="23" t="inlineStr">
@@ -2533,9 +2533,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q32" s="16" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Farmaciasnissei R$ 114.90)</t>
+      <c r="Q32" s="25" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2545,41 +2545,41 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>10028705</t>
+          <t>10052067</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>FR SAO JOAO BABY BAG G 60UN</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XXXG 64UN</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>0</v>
+        <v>415.32</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>969.79</v>
+        <v>1489.4</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-969.79</v>
+        <v>-1074.08</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>-1</v>
+        <v>-0.721</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>28997</v>
-      </c>
-      <c r="I33" s="11" t="n">
-        <v>23.03</v>
+        <v>1360</v>
+      </c>
+      <c r="I33" s="32" t="n">
+        <v>1.08</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K33" s="27" t="inlineStr"/>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K33" s="26" t="inlineStr"/>
       <c r="L33" s="12" t="inlineStr"/>
-      <c r="M33" s="27" t="inlineStr"/>
-      <c r="N33" s="28" t="inlineStr"/>
+      <c r="M33" s="26" t="inlineStr"/>
+      <c r="N33" s="27" t="inlineStr"/>
       <c r="O33" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -2587,12 +2587,12 @@
       </c>
       <c r="P33" s="12" t="inlineStr">
         <is>
-          <t>Neutro</t>
-        </is>
-      </c>
-      <c r="Q33" s="29" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q33" s="28" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2602,54 +2602,64 @@
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>10052539</t>
+          <t>10030119</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
+          <t>RYBELSUS 14MG 30CP NOVO NORDISK</t>
         </is>
       </c>
       <c r="D34" s="17" t="n">
-        <v>1760.22</v>
+        <v>1150</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>2724.42</v>
+        <v>2201.66</v>
       </c>
       <c r="F34" s="18" t="n">
-        <v>-964.2</v>
+        <v>-1051.66</v>
       </c>
       <c r="G34" s="19" t="n">
-        <v>-0.354</v>
+        <v>-0.478</v>
       </c>
       <c r="H34" s="20" t="n">
-        <v>4720</v>
-      </c>
-      <c r="I34" s="21" t="n">
-        <v>3.75</v>
+        <v>2755</v>
+      </c>
+      <c r="I34" s="29" t="n">
+        <v>2.19</v>
       </c>
       <c r="J34" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K34" s="22" t="inlineStr"/>
-      <c r="L34" s="23" t="inlineStr"/>
-      <c r="M34" s="22" t="inlineStr"/>
-      <c r="N34" s="24" t="inlineStr"/>
+      <c r="K34" s="17" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="L34" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M34" s="17" t="n">
+        <v>1301.17</v>
+      </c>
+      <c r="N34" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="O34" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P34" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Detrator Moderado</t>
         </is>
       </c>
       <c r="Q34" s="25" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Push CRM / Recompra 30d no App</t>
         </is>
       </c>
     </row>
@@ -2659,64 +2669,64 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>10097312</t>
+          <t>10024521</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>NESTOGENO 2 800G NESTLE</t>
+          <t>XIFAXAN 550MG 28CP REV BIOLAB</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>995.11</v>
+        <v>0</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>1954.05</v>
+        <v>1015.86</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>-958.9400000000001</v>
+        <v>-1015.86</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>-0.491</v>
+        <v>-1</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>12677</v>
-      </c>
-      <c r="I35" s="11" t="n">
-        <v>10.07</v>
+        <v>541</v>
+      </c>
+      <c r="I35" s="32" t="n">
+        <v>0.43</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K35" s="7" t="n">
-        <v>67.98999999999999</v>
+        <v>799.9</v>
       </c>
       <c r="L35" s="12" t="inlineStr">
         <is>
-          <t>DROGARAIA</t>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M35" s="7" t="n">
-        <v>61.06</v>
-      </c>
-      <c r="N35" s="13" t="n">
-        <v>0.113</v>
+        <v>814.9</v>
+      </c>
+      <c r="N35" s="30" t="n">
+        <v>-0.018</v>
       </c>
       <c r="O35" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P35" s="12" t="inlineStr">
         <is>
-          <t>Neutro</t>
-        </is>
-      </c>
-      <c r="Q35" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Drogaraia R$ 61.06)</t>
+          <t>Detrator Moderado</t>
+        </is>
+      </c>
+      <c r="Q35" s="28" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2726,54 +2736,44 @@
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>100014681</t>
+          <t>10052539</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>TADALAFILA 20MG 4CP REV GEN EMS</t>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
         </is>
       </c>
       <c r="D36" s="17" t="n">
-        <v>1202.65</v>
+        <v>2110.08</v>
       </c>
       <c r="E36" s="17" t="n">
-        <v>2141.74</v>
+        <v>3036.7</v>
       </c>
       <c r="F36" s="18" t="n">
-        <v>-939.09</v>
+        <v>-926.62</v>
       </c>
       <c r="G36" s="19" t="n">
-        <v>-0.4379999999999999</v>
+        <v>-0.305</v>
       </c>
       <c r="H36" s="20" t="n">
-        <v>25510</v>
-      </c>
-      <c r="I36" s="21" t="n">
-        <v>20.26</v>
+        <v>4720</v>
+      </c>
+      <c r="I36" s="29" t="n">
+        <v>3.75</v>
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K36" s="17" t="n">
-        <v>11.69</v>
-      </c>
-      <c r="L36" s="23" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M36" s="17" t="n">
-        <v>13.57</v>
-      </c>
-      <c r="N36" s="30" t="n">
-        <v>-0.139</v>
-      </c>
+      <c r="K36" s="22" t="inlineStr"/>
+      <c r="L36" s="23" t="inlineStr"/>
+      <c r="M36" s="22" t="inlineStr"/>
+      <c r="N36" s="24" t="inlineStr"/>
       <c r="O36" s="23" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P36" s="23" t="inlineStr">
@@ -2793,41 +2793,41 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>10052067</t>
+          <t>10023713</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XXXG 64UN</t>
+          <t>KIT PANTENE SH 350+COND 175ML LISO</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>415.32</v>
+        <v>118.93</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>1336.24</v>
+        <v>1036.15</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-920.92</v>
+        <v>-917.22</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>-0.6890000000000001</v>
+        <v>-0.885</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1360</v>
-      </c>
-      <c r="I37" s="26" t="n">
-        <v>1.08</v>
+        <v>17139</v>
+      </c>
+      <c r="I37" s="11" t="n">
+        <v>13.61</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K37" s="27" t="inlineStr"/>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K37" s="26" t="inlineStr"/>
       <c r="L37" s="12" t="inlineStr"/>
-      <c r="M37" s="27" t="inlineStr"/>
-      <c r="N37" s="28" t="inlineStr"/>
+      <c r="M37" s="26" t="inlineStr"/>
+      <c r="N37" s="27" t="inlineStr"/>
       <c r="O37" s="12" t="inlineStr">
         <is>
           <t>Não Monitorado</t>
@@ -2838,9 +2838,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q37" s="29" t="inlineStr">
-        <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+      <c r="Q37" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2850,54 +2850,44 @@
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>10024521</t>
+          <t>10001098</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>XIFAXAN 550MG 28CP REV BIOLAB</t>
+          <t>TOALHAS UMED HUGGIES 192UN HIDRATACAO</t>
         </is>
       </c>
       <c r="D38" s="17" t="n">
-        <v>0</v>
+        <v>1071.56</v>
       </c>
       <c r="E38" s="17" t="n">
-        <v>911.39</v>
+        <v>1976.07</v>
       </c>
       <c r="F38" s="18" t="n">
-        <v>-911.39</v>
+        <v>-904.51</v>
       </c>
       <c r="G38" s="19" t="n">
-        <v>-1</v>
+        <v>-0.458</v>
       </c>
       <c r="H38" s="20" t="n">
-        <v>541</v>
-      </c>
-      <c r="I38" s="33" t="n">
-        <v>0.43</v>
+        <v>8108</v>
+      </c>
+      <c r="I38" s="29" t="n">
+        <v>6.44</v>
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K38" s="17" t="n">
-        <v>799.9</v>
-      </c>
-      <c r="L38" s="23" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M38" s="17" t="n">
-        <v>814.9</v>
-      </c>
-      <c r="N38" s="30" t="n">
-        <v>-0.018</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K38" s="22" t="inlineStr"/>
+      <c r="L38" s="23" t="inlineStr"/>
+      <c r="M38" s="22" t="inlineStr"/>
+      <c r="N38" s="24" t="inlineStr"/>
       <c r="O38" s="23" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P38" s="23" t="inlineStr">
@@ -2907,7 +2897,7 @@
       </c>
       <c r="Q38" s="25" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2926,16 +2916,16 @@
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>1144.93</v>
+        <v>1341.25</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>1993.86</v>
+        <v>2222.4</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-848.9299999999999</v>
+        <v>-881.15</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>-0.426</v>
+        <v>-0.396</v>
       </c>
       <c r="H39" s="10" t="n">
         <v>10260</v>
@@ -2993,21 +2983,21 @@
         </is>
       </c>
       <c r="D40" s="17" t="n">
-        <v>388.6</v>
+        <v>521.09</v>
       </c>
       <c r="E40" s="17" t="n">
-        <v>1232.66</v>
+        <v>1373.95</v>
       </c>
       <c r="F40" s="18" t="n">
-        <v>-844.0599999999999</v>
+        <v>-852.86</v>
       </c>
       <c r="G40" s="19" t="n">
-        <v>-0.6850000000000001</v>
+        <v>-0.621</v>
       </c>
       <c r="H40" s="20" t="n">
         <v>7950</v>
       </c>
-      <c r="I40" s="21" t="n">
+      <c r="I40" s="29" t="n">
         <v>6.31</v>
       </c>
       <c r="J40" s="14" t="inlineStr">
@@ -3026,7 +3016,7 @@
       <c r="M40" s="17" t="n">
         <v>124.19</v>
       </c>
-      <c r="N40" s="32" t="n">
+      <c r="N40" s="31" t="n">
         <v>0.067</v>
       </c>
       <c r="O40" s="23" t="inlineStr">
@@ -3051,54 +3041,44 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>10030119</t>
+          <t>10052538</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>RYBELSUS 14MG 30CP NOVO NORDISK</t>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XXG 74</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>1150</v>
+        <v>2010.13</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>1975.25</v>
+        <v>2857.64</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-825.25</v>
+        <v>-847.51</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>-0.418</v>
+        <v>-0.297</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>2755</v>
+        <v>4879</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>2.19</v>
+        <v>3.88</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K41" s="7" t="n">
-        <v>1301.17</v>
-      </c>
-      <c r="L41" s="12" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="n">
-        <v>1301.17</v>
-      </c>
-      <c r="N41" s="31" t="n">
-        <v>0</v>
-      </c>
+      <c r="K41" s="26" t="inlineStr"/>
+      <c r="L41" s="12" t="inlineStr"/>
+      <c r="M41" s="26" t="inlineStr"/>
+      <c r="N41" s="27" t="inlineStr"/>
       <c r="O41" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P41" s="12" t="inlineStr">
@@ -3106,9 +3086,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q41" s="29" t="inlineStr">
-        <is>
-          <t>Push CRM / Recompra 30d no App</t>
+      <c r="Q41" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3118,40 +3098,46 @@
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>10001098</t>
+          <t>10025098</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>TOALHAS UMED HUGGIES 192UN HIDRATACAO</t>
+          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
         </is>
       </c>
       <c r="D42" s="17" t="n">
-        <v>958.1900000000001</v>
+        <v>0</v>
       </c>
       <c r="E42" s="17" t="n">
-        <v>1772.86</v>
+        <v>830.47</v>
       </c>
       <c r="F42" s="18" t="n">
-        <v>-814.67</v>
+        <v>-830.47</v>
       </c>
       <c r="G42" s="19" t="n">
-        <v>-0.46</v>
+        <v>-1</v>
       </c>
       <c r="H42" s="20" t="n">
-        <v>8108</v>
+        <v>182</v>
       </c>
       <c r="I42" s="21" t="n">
-        <v>6.44</v>
+        <v>0.14</v>
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K42" s="22" t="inlineStr"/>
-      <c r="L42" s="23" t="inlineStr"/>
-      <c r="M42" s="22" t="inlineStr"/>
+      <c r="L42" s="23" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M42" s="17" t="n">
+        <v>1212.9</v>
+      </c>
       <c r="N42" s="24" t="inlineStr"/>
       <c r="O42" s="23" t="inlineStr">
         <is>
@@ -3165,7 +3151,7 @@
       </c>
       <c r="Q42" s="25" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -3175,44 +3161,54 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>10023713</t>
+          <t>5309</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>KIT PANTENE SH 350+COND 175ML LISO</t>
+          <t>EXPEC 120ML XPE LEGRAND</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>118.93</v>
+        <v>1271.63</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>929.6</v>
+        <v>2092.95</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-810.67</v>
+        <v>-821.3200000000001</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>-0.872</v>
+        <v>-0.392</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>17139</v>
+        <v>61236</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>13.61</v>
+        <v>48.64</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K43" s="27" t="inlineStr"/>
-      <c r="L43" s="12" t="inlineStr"/>
-      <c r="M43" s="27" t="inlineStr"/>
-      <c r="N43" s="28" t="inlineStr"/>
+      <c r="K43" s="7" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="L43" s="12" t="inlineStr">
+        <is>
+          <t>DROGARAIA</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="n">
+        <v>27.72</v>
+      </c>
+      <c r="N43" s="13" t="n">
+        <v>0.006</v>
+      </c>
       <c r="O43" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P43" s="12" t="inlineStr">
@@ -3220,7 +3216,7 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q43" s="29" t="inlineStr">
+      <c r="Q43" s="28" t="inlineStr">
         <is>
           <t>Ação Promocional / Destaque Home</t>
         </is>
@@ -3232,44 +3228,54 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>10052538</t>
+          <t>10105798</t>
         </is>
       </c>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XXG 74</t>
+          <t>PRISTIQ 100MG 28CP PFIZER (C1)</t>
         </is>
       </c>
       <c r="D44" s="17" t="n">
-        <v>1770.33</v>
+        <v>0</v>
       </c>
       <c r="E44" s="17" t="n">
-        <v>2563.77</v>
+        <v>811.75</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>-793.4400000000001</v>
+        <v>-811.75</v>
       </c>
       <c r="G44" s="19" t="n">
-        <v>-0.309</v>
+        <v>-1</v>
       </c>
       <c r="H44" s="20" t="n">
-        <v>4879</v>
+        <v>1693</v>
       </c>
       <c r="I44" s="21" t="n">
-        <v>3.88</v>
+        <v>1.34</v>
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K44" s="22" t="inlineStr"/>
-      <c r="L44" s="23" t="inlineStr"/>
-      <c r="M44" s="22" t="inlineStr"/>
-      <c r="N44" s="24" t="inlineStr"/>
+          <t>⚠️ Duplo Detrator</t>
+        </is>
+      </c>
+      <c r="K44" s="17" t="n">
+        <v>291.89</v>
+      </c>
+      <c r="L44" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M44" s="17" t="n">
+        <v>229.9</v>
+      </c>
+      <c r="N44" s="31" t="n">
+        <v>0.27</v>
+      </c>
       <c r="O44" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P44" s="23" t="inlineStr">
@@ -3277,9 +3283,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q44" s="25" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q44" s="16" t="inlineStr">
+        <is>
+          <t>Reprecificar e Remanejar (Precopopular R$ 229.90)</t>
         </is>
       </c>
     </row>
@@ -3289,54 +3295,54 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>10040802</t>
+          <t>100015009</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>WEGOVY 2,4MG 3ML NOVO NORDISK</t>
+          <t>SAB DOVE 90G LV+ PG- 6UN ORIGINAL</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>5247</v>
+        <v>1198.85</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>6008.19</v>
+        <v>2003.42</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-761.1900000000001</v>
+        <v>-804.5700000000001</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>-0.127</v>
+        <v>-0.402</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>3682</v>
+        <v>59032</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>2.92</v>
+        <v>46.89</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K45" s="7" t="n">
-        <v>2501.8</v>
+        <v>27.9</v>
       </c>
       <c r="L45" s="12" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M45" s="7" t="n">
-        <v>2501.8</v>
-      </c>
-      <c r="N45" s="31" t="n">
-        <v>0</v>
+        <v>24.9</v>
+      </c>
+      <c r="N45" s="13" t="n">
+        <v>0.12</v>
       </c>
       <c r="O45" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P45" s="12" t="inlineStr">
@@ -3344,9 +3350,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q45" s="29" t="inlineStr">
-        <is>
-          <t>Push CRM / Recompra 30d no App</t>
+      <c r="Q45" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Panvel R$ 24.90)</t>
         </is>
       </c>
     </row>
@@ -3356,50 +3362,54 @@
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>10025098</t>
+          <t>100013366</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
+          <t>DYMISTA 137+50MCG 23G SPRAY NASAL MYLAN</t>
         </is>
       </c>
       <c r="D46" s="17" t="n">
-        <v>0</v>
+        <v>248.89</v>
       </c>
       <c r="E46" s="17" t="n">
-        <v>745.0700000000001</v>
+        <v>1041.31</v>
       </c>
       <c r="F46" s="18" t="n">
-        <v>-745.0700000000001</v>
+        <v>-792.42</v>
       </c>
       <c r="G46" s="19" t="n">
-        <v>-1</v>
+        <v>-0.7609999999999999</v>
       </c>
       <c r="H46" s="20" t="n">
-        <v>182</v>
-      </c>
-      <c r="I46" s="33" t="n">
-        <v>0.14</v>
+        <v>6142</v>
+      </c>
+      <c r="I46" s="29" t="n">
+        <v>4.88</v>
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K46" s="22" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K46" s="17" t="n">
+        <v>156.21</v>
+      </c>
       <c r="L46" s="23" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M46" s="17" t="n">
-        <v>1212.9</v>
-      </c>
-      <c r="N46" s="24" t="inlineStr"/>
+        <v>119.89</v>
+      </c>
+      <c r="N46" s="31" t="n">
+        <v>0.303</v>
+      </c>
       <c r="O46" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P46" s="23" t="inlineStr">
@@ -3407,9 +3417,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q46" s="25" t="inlineStr">
-        <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+      <c r="Q46" s="16" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Farmaciasnissei R$ 119.89)</t>
         </is>
       </c>
     </row>
@@ -3419,31 +3429,31 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>100015009</t>
+          <t>10032148</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>SAB DOVE 90G LV+ PG- 6UN ORIGINAL</t>
+          <t>APTAMIL PROFUTURA GOLD 1 800G DANONE</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>1060.76</v>
+        <v>114.6</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>1797.4</v>
+        <v>905.33</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-736.64</v>
+        <v>-790.73</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>-0.41</v>
+        <v>-0.873</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>59032</v>
+        <v>6458</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>46.89</v>
+        <v>5.13</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
@@ -3451,18 +3461,18 @@
         </is>
       </c>
       <c r="K47" s="7" t="n">
-        <v>27.9</v>
+        <v>130.99</v>
       </c>
       <c r="L47" s="12" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>AMAZON</t>
         </is>
       </c>
       <c r="M47" s="7" t="n">
-        <v>24.9</v>
+        <v>119.59</v>
       </c>
       <c r="N47" s="13" t="n">
-        <v>0.12</v>
+        <v>0.095</v>
       </c>
       <c r="O47" s="12" t="inlineStr">
         <is>
@@ -3476,7 +3486,7 @@
       </c>
       <c r="Q47" s="6" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Panvel R$ 24.90)</t>
+          <t>Reprecificar no Digital (Amazon R$ 119.59)</t>
         </is>
       </c>
     </row>
@@ -3486,54 +3496,50 @@
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>10033463</t>
+          <t>10028116</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>FR BABYSEC ULTRA HIPER XG 56UN</t>
+          <t>SLINDA 4MG 24CP+4PLACEBOS EXELTIS</t>
         </is>
       </c>
       <c r="D48" s="17" t="n">
-        <v>2254.67</v>
+        <v>109.59</v>
       </c>
       <c r="E48" s="17" t="n">
-        <v>2987.6</v>
+        <v>883.78</v>
       </c>
       <c r="F48" s="18" t="n">
-        <v>-732.9299999999999</v>
+        <v>-774.1900000000001</v>
       </c>
       <c r="G48" s="19" t="n">
-        <v>-0.245</v>
+        <v>-0.8759999999999999</v>
       </c>
       <c r="H48" s="20" t="n">
-        <v>11371</v>
-      </c>
-      <c r="I48" s="21" t="n">
-        <v>9.029999999999999</v>
+        <v>5338</v>
+      </c>
+      <c r="I48" s="29" t="n">
+        <v>4.24</v>
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
-        </is>
-      </c>
-      <c r="K48" s="17" t="n">
-        <v>69.90000000000001</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K48" s="22" t="inlineStr"/>
       <c r="L48" s="23" t="inlineStr">
         <is>
           <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M48" s="17" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="N48" s="32" t="n">
-        <v>0.167</v>
-      </c>
+        <v>99.31999999999999</v>
+      </c>
+      <c r="N48" s="24" t="inlineStr"/>
       <c r="O48" s="23" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P48" s="23" t="inlineStr">
@@ -3541,9 +3547,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q48" s="16" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 59.90)</t>
+      <c r="Q48" s="25" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3553,39 +3559,39 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>10105798</t>
+          <t>10033760</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>PRISTIQ 100MG 28CP PFIZER (C1)</t>
+          <t>FR HUGGIES MAXIMA PROT HIPER G 58UN</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>0</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>728.27</v>
+        <v>851.96</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-728.27</v>
+        <v>-767.0599999999999</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>-1</v>
+        <v>-0.9</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>1693</v>
-      </c>
-      <c r="I49" s="26" t="n">
-        <v>1.34</v>
+        <v>20831</v>
+      </c>
+      <c r="I49" s="11" t="n">
+        <v>16.55</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Duplo Detrator</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K49" s="7" t="n">
-        <v>291.89</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="L49" s="12" t="inlineStr">
         <is>
@@ -3593,10 +3599,10 @@
         </is>
       </c>
       <c r="M49" s="7" t="n">
-        <v>229.9</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="N49" s="13" t="n">
-        <v>0.27</v>
+        <v>0.165</v>
       </c>
       <c r="O49" s="12" t="inlineStr">
         <is>
@@ -3610,7 +3616,7 @@
       </c>
       <c r="Q49" s="6" t="inlineStr">
         <is>
-          <t>Reprecificar e Remanejar (Precopopular R$ 229.90)</t>
+          <t>Reprecificar no Digital (Precopopular R$ 72.90)</t>
         </is>
       </c>
     </row>
@@ -3620,31 +3626,31 @@
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>5309</t>
+          <t>100010880</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
-          <t>EXPEC 120ML XPE LEGRAND</t>
+          <t>JARDIANCE 25MG 30CP REV BOEHRINGER</t>
         </is>
       </c>
       <c r="D50" s="17" t="n">
-        <v>1160.03</v>
+        <v>0</v>
       </c>
       <c r="E50" s="17" t="n">
-        <v>1877.72</v>
+        <v>765.51</v>
       </c>
       <c r="F50" s="18" t="n">
-        <v>-717.6900000000001</v>
+        <v>-765.51</v>
       </c>
       <c r="G50" s="19" t="n">
-        <v>-0.382</v>
+        <v>-1</v>
       </c>
       <c r="H50" s="20" t="n">
-        <v>61236</v>
-      </c>
-      <c r="I50" s="21" t="n">
-        <v>48.64</v>
+        <v>5841</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>4.64</v>
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
@@ -3652,18 +3658,18 @@
         </is>
       </c>
       <c r="K50" s="17" t="n">
-        <v>27.9</v>
+        <v>320.99</v>
       </c>
       <c r="L50" s="23" t="inlineStr">
         <is>
-          <t>DROGARAIA</t>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M50" s="17" t="n">
-        <v>27.72</v>
-      </c>
-      <c r="N50" s="32" t="n">
-        <v>0.006</v>
+        <v>320.99</v>
+      </c>
+      <c r="N50" s="33" t="n">
+        <v>0</v>
       </c>
       <c r="O50" s="23" t="inlineStr">
         <is>
@@ -3687,54 +3693,44 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>100001702</t>
+          <t>10046473</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>FR MATURI CARE CONFORT G 30UN</t>
+          <t>ROUPA INT SAO JOAO ADULTO PANTS G/XG 32UN</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>0</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>708.2</v>
+        <v>838.26</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-708.2</v>
+        <v>-743.27</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>-1</v>
+        <v>-0.887</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>10776</v>
+        <v>19215</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>8.56</v>
+        <v>15.26</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K51" s="7" t="n">
-        <v>75.98999999999999</v>
-      </c>
-      <c r="L51" s="12" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M51" s="7" t="n">
-        <v>87.90000000000001</v>
-      </c>
-      <c r="N51" s="31" t="n">
-        <v>-0.135</v>
-      </c>
+      <c r="K51" s="26" t="inlineStr"/>
+      <c r="L51" s="12" t="inlineStr"/>
+      <c r="M51" s="26" t="inlineStr"/>
+      <c r="N51" s="27" t="inlineStr"/>
       <c r="O51" s="12" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P51" s="12" t="inlineStr">
@@ -3742,7 +3738,7 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q51" s="29" t="inlineStr">
+      <c r="Q51" s="28" t="inlineStr">
         <is>
           <t>Ação Promocional / Destaque Home</t>
         </is>
@@ -3754,44 +3750,54 @@
       </c>
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>10052540</t>
+          <t>10031305</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX G 90UN</t>
+          <t>AMMY 4MG 28CP REV MANTECORP</t>
         </is>
       </c>
       <c r="D52" s="17" t="n">
-        <v>589.5</v>
+        <v>0</v>
       </c>
       <c r="E52" s="17" t="n">
-        <v>1290.79</v>
+        <v>729.28</v>
       </c>
       <c r="F52" s="18" t="n">
-        <v>-701.29</v>
+        <v>-729.28</v>
       </c>
       <c r="G52" s="19" t="n">
-        <v>-0.5429999999999999</v>
+        <v>-1</v>
       </c>
       <c r="H52" s="20" t="n">
-        <v>2498</v>
-      </c>
-      <c r="I52" s="21" t="n">
-        <v>1.98</v>
+        <v>9175</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>7.29</v>
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K52" s="22" t="inlineStr"/>
-      <c r="L52" s="23" t="inlineStr"/>
-      <c r="M52" s="22" t="inlineStr"/>
-      <c r="N52" s="24" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K52" s="17" t="n">
+        <v>132.43</v>
+      </c>
+      <c r="L52" s="23" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M52" s="17" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="N52" s="31" t="n">
+        <v>0.333</v>
+      </c>
       <c r="O52" s="23" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P52" s="23" t="inlineStr">
@@ -3799,9 +3805,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q52" s="25" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q52" s="16" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 99.32)</t>
         </is>
       </c>
     </row>
@@ -3811,54 +3817,54 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>10032148</t>
+          <t>100001702</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>APTAMIL PROFUTURA GOLD 1 800G DANONE</t>
+          <t>FR MATURI CARE CONFORT G 30UN</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>114.6</v>
+        <v>68.86</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>812.23</v>
+        <v>789.38</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-697.63</v>
+        <v>-720.52</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>-0.8590000000000001</v>
+        <v>-0.9129999999999999</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>6458</v>
+        <v>10776</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>5.13</v>
+        <v>8.56</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K53" s="7" t="n">
-        <v>130.99</v>
+        <v>75.98999999999999</v>
       </c>
       <c r="L53" s="12" t="inlineStr">
         <is>
-          <t>AMAZON</t>
+          <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M53" s="7" t="n">
-        <v>119.59</v>
-      </c>
-      <c r="N53" s="13" t="n">
-        <v>0.095</v>
+        <v>87.90000000000001</v>
+      </c>
+      <c r="N53" s="30" t="n">
+        <v>-0.135</v>
       </c>
       <c r="O53" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P53" s="12" t="inlineStr">
@@ -3866,9 +3872,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q53" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 119.59)</t>
+      <c r="Q53" s="28" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3878,54 +3884,54 @@
       </c>
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>100010880</t>
+          <t>10023372</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>JARDIANCE 25MG 30CP REV BOEHRINGER</t>
+          <t>REXULTI 1MG 30CP LUNDBECK (C1)</t>
         </is>
       </c>
       <c r="D54" s="17" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="17" t="n">
-        <v>686.78</v>
+        <v>705.35</v>
       </c>
       <c r="F54" s="18" t="n">
-        <v>-686.78</v>
+        <v>-705.35</v>
       </c>
       <c r="G54" s="19" t="n">
         <v>-1</v>
       </c>
       <c r="H54" s="20" t="n">
-        <v>5841</v>
+        <v>1615</v>
       </c>
       <c r="I54" s="21" t="n">
-        <v>4.64</v>
+        <v>1.28</v>
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>⚠️ Duplo Detrator</t>
         </is>
       </c>
       <c r="K54" s="17" t="n">
-        <v>320.99</v>
+        <v>422.26</v>
       </c>
       <c r="L54" s="23" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M54" s="17" t="n">
-        <v>320.99</v>
-      </c>
-      <c r="N54" s="30" t="n">
-        <v>0</v>
+        <v>355.64</v>
+      </c>
+      <c r="N54" s="31" t="n">
+        <v>0.187</v>
       </c>
       <c r="O54" s="23" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P54" s="23" t="inlineStr">
@@ -3933,9 +3939,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q54" s="25" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q54" s="16" t="inlineStr">
+        <is>
+          <t>Reprecificar e Remanejar (Farmaciasnissei R$ 355.64)</t>
         </is>
       </c>
     </row>

</xml_diff>